<commit_message>
Fix Excel email draft link on Mac
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R3227513ec2e440a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R3cf339cad2834473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R000feaed12d34dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Red235a641382445c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1137,12 +1137,32 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -1201,7 +1221,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1286,6 +1306,24 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
@@ -1606,19 +1644,19 @@
       <x:c r="L1" s="1" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="32" t="str">
+      <x:c r="M1" s="39" t="str">
         <x:v>Notify?</x:v>
       </x:c>
-      <x:c r="N1" s="32" t="str">
+      <x:c r="N1" s="39" t="str">
         <x:v>Email subject</x:v>
       </x:c>
-      <x:c r="O1" s="32" t="str">
+      <x:c r="O1" s="39" t="str">
         <x:v>Email body</x:v>
       </x:c>
-      <x:c r="P1" s="32" t="str">
+      <x:c r="P1" s="39" t="str">
         <x:v>Open email draft</x:v>
       </x:c>
-      <x:c r="Q1" s="32" t="str">
+      <x:c r="Q1" s="39" t="str">
         <x:v>Notification date</x:v>
       </x:c>
     </x:row>
@@ -1659,17 +1697,17 @@
       <x:c r="L2" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M2" s="29"/>
-      <x:c r="N2" s="30" t="str">
+      <x:c r="M2" s="36"/>
+      <x:c r="N2" s="37" t="str">
         <x:f>IF(M2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
       </x:c>
-      <x:c r="O2" s="30" t="str">
+      <x:c r="O2" s="37" t="str">
         <x:f>IF(M2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K2&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P2" s="30" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N2)&amp;"&amp;body="&amp;ENCODEURL(O2),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q2" s="31"/>
+      <x:c r="P2" s="37" t="str">
+        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N2,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O2,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q2" s="38"/>
     </x:row>
     <x:row r="3" ht="31">
       <x:c r="A3" s="2" t="s">
@@ -1708,17 +1746,17 @@
       <x:c r="L3" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M3" s="29"/>
-      <x:c r="N3" s="30" t="str">
+      <x:c r="M3" s="36"/>
+      <x:c r="N3" s="37" t="str">
         <x:f>IF(M3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
       </x:c>
-      <x:c r="O3" s="30" t="str">
+      <x:c r="O3" s="37" t="str">
         <x:f>IF(M3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K3&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P3" s="30" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N3)&amp;"&amp;body="&amp;ENCODEURL(O3),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q3" s="31"/>
+      <x:c r="P3" s="37" t="str">
+        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N3,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O3,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q3" s="38"/>
     </x:row>
     <x:row r="4" ht="31">
       <x:c r="A4" s="2" t="s">
@@ -1757,17 +1795,17 @@
       <x:c r="L4" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M4" s="29"/>
-      <x:c r="N4" s="30" t="str">
+      <x:c r="M4" s="36"/>
+      <x:c r="N4" s="37" t="str">
         <x:f>IF(M4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
       </x:c>
-      <x:c r="O4" s="30" t="str">
+      <x:c r="O4" s="37" t="str">
         <x:f>IF(M4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K4&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P4" s="30" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N4)&amp;"&amp;body="&amp;ENCODEURL(O4),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q4" s="31"/>
+      <x:c r="P4" s="37" t="str">
+        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N4,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O4,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q4" s="38"/>
     </x:row>
     <x:row r="5" ht="46">
       <x:c r="A5" s="2" t="s">
@@ -1806,17 +1844,17 @@
       <x:c r="L5" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M5" s="29"/>
-      <x:c r="N5" s="30" t="str">
+      <x:c r="M5" s="36"/>
+      <x:c r="N5" s="37" t="str">
         <x:f>IF(M5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
       </x:c>
-      <x:c r="O5" s="30" t="str">
+      <x:c r="O5" s="37" t="str">
         <x:f>IF(M5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K5&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P5" s="30" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N5)&amp;"&amp;body="&amp;ENCODEURL(O5),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q5" s="31"/>
+      <x:c r="P5" s="37" t="str">
+        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N5,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O5,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q5" s="38"/>
     </x:row>
     <x:row r="6" ht="31">
       <x:c r="A6" s="2" t="s">
@@ -1855,17 +1893,17 @@
       <x:c r="L6" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M6" s="29"/>
-      <x:c r="N6" s="30" t="str">
+      <x:c r="M6" s="36"/>
+      <x:c r="N6" s="37" t="str">
         <x:f>IF(M6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
       </x:c>
-      <x:c r="O6" s="30" t="str">
+      <x:c r="O6" s="37" t="str">
         <x:f>IF(M6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K6&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P6" s="30" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N6)&amp;"&amp;body="&amp;ENCODEURL(O6),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q6" s="31"/>
+      <x:c r="P6" s="37" t="str">
+        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N6,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O6,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q6" s="38"/>
     </x:row>
     <x:row r="7" ht="31">
       <x:c r="A7" s="2" t="s">
@@ -1904,17 +1942,17 @@
       <x:c r="L7" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M7" s="29"/>
-      <x:c r="N7" s="30" t="str">
+      <x:c r="M7" s="36"/>
+      <x:c r="N7" s="37" t="str">
         <x:f>IF(M7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
       </x:c>
-      <x:c r="O7" s="30" t="str">
+      <x:c r="O7" s="37" t="str">
         <x:f>IF(M7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K7&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P7" s="30" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N7)&amp;"&amp;body="&amp;ENCODEURL(O7),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q7" s="31"/>
+      <x:c r="P7" s="37" t="str">
+        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N7,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O7,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q7" s="38"/>
     </x:row>
     <x:row r="8" ht="46">
       <x:c r="A8" s="2" t="s">
@@ -1953,17 +1991,17 @@
       <x:c r="L8" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M8" s="29"/>
-      <x:c r="N8" s="30" t="str">
+      <x:c r="M8" s="36"/>
+      <x:c r="N8" s="37" t="str">
         <x:f>IF(M8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
       </x:c>
-      <x:c r="O8" s="30" t="str">
+      <x:c r="O8" s="37" t="str">
         <x:f>IF(M8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K8&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P8" s="30" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N8)&amp;"&amp;body="&amp;ENCODEURL(O8),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q8" s="31"/>
+      <x:c r="P8" s="37" t="str">
+        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N8,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O8,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q8" s="38"/>
     </x:row>
     <x:row r="9" ht="31">
       <x:c r="A9" s="2" t="s">
@@ -2002,17 +2040,17 @@
       <x:c r="L9" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M9" s="29"/>
-      <x:c r="N9" s="30" t="str">
+      <x:c r="M9" s="36"/>
+      <x:c r="N9" s="37" t="str">
         <x:f>IF(M9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
       </x:c>
-      <x:c r="O9" s="30" t="str">
+      <x:c r="O9" s="37" t="str">
         <x:f>IF(M9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K9&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P9" s="30" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N9)&amp;"&amp;body="&amp;ENCODEURL(O9),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q9" s="31"/>
+      <x:c r="P9" s="37" t="str">
+        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N9,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O9,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q9" s="38"/>
     </x:row>
     <x:row r="10" ht="31">
       <x:c r="A10" s="2" t="s">
@@ -2051,17 +2089,17 @@
       <x:c r="L10" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M10" s="29"/>
-      <x:c r="N10" s="30" t="str">
+      <x:c r="M10" s="36"/>
+      <x:c r="N10" s="37" t="str">
         <x:f>IF(M10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
       </x:c>
-      <x:c r="O10" s="30" t="str">
+      <x:c r="O10" s="37" t="str">
         <x:f>IF(M10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K10&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P10" s="30" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N10)&amp;"&amp;body="&amp;ENCODEURL(O10),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q10" s="31"/>
+      <x:c r="P10" s="37" t="str">
+        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N10,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O10,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q10" s="38"/>
     </x:row>
     <x:row r="11" ht="31">
       <x:c r="A11" s="2" t="s">
@@ -2100,17 +2138,17 @@
       <x:c r="L11" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M11" s="29"/>
-      <x:c r="N11" s="30" t="str">
+      <x:c r="M11" s="36"/>
+      <x:c r="N11" s="37" t="str">
         <x:f>IF(M11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
       </x:c>
-      <x:c r="O11" s="30" t="str">
+      <x:c r="O11" s="37" t="str">
         <x:f>IF(M11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K11&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P11" s="30" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N11)&amp;"&amp;body="&amp;ENCODEURL(O11),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q11" s="31"/>
+      <x:c r="P11" s="37" t="str">
+        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N11,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O11,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q11" s="38"/>
     </x:row>
     <x:row r="12" ht="31">
       <x:c r="A12" s="2" t="s">
@@ -2149,17 +2187,17 @@
       <x:c r="L12" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M12" s="29"/>
-      <x:c r="N12" s="30" t="str">
+      <x:c r="M12" s="36"/>
+      <x:c r="N12" s="37" t="str">
         <x:f>IF(M12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
       </x:c>
-      <x:c r="O12" s="30" t="str">
+      <x:c r="O12" s="37" t="str">
         <x:f>IF(M12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K12&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P12" s="30" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N12)&amp;"&amp;body="&amp;ENCODEURL(O12),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q12" s="31"/>
+      <x:c r="P12" s="37" t="str">
+        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N12,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O12,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q12" s="38"/>
     </x:row>
     <x:row r="13" ht="31">
       <x:c r="A13" s="2" t="s">
@@ -2198,17 +2236,17 @@
       <x:c r="L13" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M13" s="29"/>
-      <x:c r="N13" s="30" t="str">
+      <x:c r="M13" s="36"/>
+      <x:c r="N13" s="37" t="str">
         <x:f>IF(M13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
       </x:c>
-      <x:c r="O13" s="30" t="str">
+      <x:c r="O13" s="37" t="str">
         <x:f>IF(M13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K13&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P13" s="30" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N13)&amp;"&amp;body="&amp;ENCODEURL(O13),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q13" s="31"/>
+      <x:c r="P13" s="37" t="str">
+        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N13,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O13,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q13" s="38"/>
     </x:row>
     <x:row r="14" ht="46">
       <x:c r="A14" s="2" t="s">
@@ -2247,17 +2285,17 @@
       <x:c r="L14" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M14" s="29"/>
-      <x:c r="N14" s="30" t="str">
+      <x:c r="M14" s="36"/>
+      <x:c r="N14" s="37" t="str">
         <x:f>IF(M14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
       </x:c>
-      <x:c r="O14" s="30" t="str">
+      <x:c r="O14" s="37" t="str">
         <x:f>IF(M14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K14&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P14" s="30" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N14)&amp;"&amp;body="&amp;ENCODEURL(O14),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q14" s="31"/>
+      <x:c r="P14" s="37" t="str">
+        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N14,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O14,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q14" s="38"/>
     </x:row>
     <x:row r="15" ht="46">
       <x:c r="A15" s="2" t="s">
@@ -2296,17 +2334,17 @@
       <x:c r="L15" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M15" s="29"/>
-      <x:c r="N15" s="30" t="str">
+      <x:c r="M15" s="36"/>
+      <x:c r="N15" s="37" t="str">
         <x:f>IF(M15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
       </x:c>
-      <x:c r="O15" s="30" t="str">
+      <x:c r="O15" s="37" t="str">
         <x:f>IF(M15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K15&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P15" s="30" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N15)&amp;"&amp;body="&amp;ENCODEURL(O15),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q15" s="31"/>
+      <x:c r="P15" s="37" t="str">
+        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N15,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O15,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q15" s="38"/>
     </x:row>
     <x:row r="16" ht="31">
       <x:c r="A16" s="2" t="s">
@@ -2345,17 +2383,17 @@
       <x:c r="L16" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M16" s="29"/>
-      <x:c r="N16" s="30" t="str">
+      <x:c r="M16" s="36"/>
+      <x:c r="N16" s="37" t="str">
         <x:f>IF(M16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
       </x:c>
-      <x:c r="O16" s="30" t="str">
+      <x:c r="O16" s="37" t="str">
         <x:f>IF(M16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K16&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P16" s="30" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N16)&amp;"&amp;body="&amp;ENCODEURL(O16),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q16" s="31"/>
+      <x:c r="P16" s="37" t="str">
+        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N16,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O16,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q16" s="38"/>
     </x:row>
     <x:row r="17" ht="31">
       <x:c r="A17" s="2" t="s">
@@ -2394,17 +2432,17 @@
       <x:c r="L17" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M17" s="29"/>
-      <x:c r="N17" s="30" t="str">
+      <x:c r="M17" s="36"/>
+      <x:c r="N17" s="37" t="str">
         <x:f>IF(M17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
       </x:c>
-      <x:c r="O17" s="30" t="str">
+      <x:c r="O17" s="37" t="str">
         <x:f>IF(M17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K17&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P17" s="30" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N17)&amp;"&amp;body="&amp;ENCODEURL(O17),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q17" s="31"/>
+      <x:c r="P17" s="37" t="str">
+        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N17,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O17,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q17" s="38"/>
     </x:row>
     <x:row r="18" ht="46">
       <x:c r="A18" s="2" t="s">
@@ -2443,17 +2481,17 @@
       <x:c r="L18" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M18" s="29"/>
-      <x:c r="N18" s="30" t="str">
+      <x:c r="M18" s="36"/>
+      <x:c r="N18" s="37" t="str">
         <x:f>IF(M18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
       </x:c>
-      <x:c r="O18" s="30" t="str">
+      <x:c r="O18" s="37" t="str">
         <x:f>IF(M18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K18&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P18" s="30" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N18)&amp;"&amp;body="&amp;ENCODEURL(O18),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q18" s="31"/>
+      <x:c r="P18" s="37" t="str">
+        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N18,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O18,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q18" s="38"/>
     </x:row>
     <x:row r="19" ht="31">
       <x:c r="A19" s="2" t="s">
@@ -2492,17 +2530,17 @@
       <x:c r="L19" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M19" s="29"/>
-      <x:c r="N19" s="30" t="str">
+      <x:c r="M19" s="36"/>
+      <x:c r="N19" s="37" t="str">
         <x:f>IF(M19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
       </x:c>
-      <x:c r="O19" s="30" t="str">
+      <x:c r="O19" s="37" t="str">
         <x:f>IF(M19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K19&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P19" s="30" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N19)&amp;"&amp;body="&amp;ENCODEURL(O19),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q19" s="31"/>
+      <x:c r="P19" s="37" t="str">
+        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N19,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O19,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q19" s="38"/>
     </x:row>
     <x:row r="20" ht="46">
       <x:c r="A20" s="2" t="s">
@@ -2541,17 +2579,17 @@
       <x:c r="L20" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M20" s="29"/>
-      <x:c r="N20" s="30" t="str">
+      <x:c r="M20" s="36"/>
+      <x:c r="N20" s="37" t="str">
         <x:f>IF(M20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
       </x:c>
-      <x:c r="O20" s="30" t="str">
+      <x:c r="O20" s="37" t="str">
         <x:f>IF(M20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K20&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P20" s="30" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N20)&amp;"&amp;body="&amp;ENCODEURL(O20),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q20" s="31"/>
+      <x:c r="P20" s="37" t="str">
+        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N20,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O20,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q20" s="38"/>
     </x:row>
     <x:row r="21" ht="31">
       <x:c r="A21" s="2" t="s">
@@ -2590,17 +2628,17 @@
       <x:c r="L21" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M21" s="29"/>
-      <x:c r="N21" s="30" t="str">
+      <x:c r="M21" s="36"/>
+      <x:c r="N21" s="37" t="str">
         <x:f>IF(M21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
       </x:c>
-      <x:c r="O21" s="30" t="str">
+      <x:c r="O21" s="37" t="str">
         <x:f>IF(M21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K21&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P21" s="30" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N21)&amp;"&amp;body="&amp;ENCODEURL(O21),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q21" s="31"/>
+      <x:c r="P21" s="37" t="str">
+        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N21,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O21,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q21" s="38"/>
     </x:row>
     <x:row r="22" ht="31">
       <x:c r="A22" s="2" t="s">
@@ -2639,17 +2677,17 @@
       <x:c r="L22" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M22" s="29"/>
-      <x:c r="N22" s="30" t="str">
+      <x:c r="M22" s="36"/>
+      <x:c r="N22" s="37" t="str">
         <x:f>IF(M22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
       </x:c>
-      <x:c r="O22" s="30" t="str">
+      <x:c r="O22" s="37" t="str">
         <x:f>IF(M22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K22&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P22" s="30" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N22)&amp;"&amp;body="&amp;ENCODEURL(O22),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q22" s="31"/>
+      <x:c r="P22" s="37" t="str">
+        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N22,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O22,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q22" s="38"/>
     </x:row>
     <x:row r="23" ht="31">
       <x:c r="A23" s="2" t="s">
@@ -2688,17 +2726,17 @@
       <x:c r="L23" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M23" s="29"/>
-      <x:c r="N23" s="30" t="str">
+      <x:c r="M23" s="36"/>
+      <x:c r="N23" s="37" t="str">
         <x:f>IF(M23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
       </x:c>
-      <x:c r="O23" s="30" t="str">
+      <x:c r="O23" s="37" t="str">
         <x:f>IF(M23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K23&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P23" s="30" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N23)&amp;"&amp;body="&amp;ENCODEURL(O23),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q23" s="31"/>
+      <x:c r="P23" s="37" t="str">
+        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N23,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O23,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q23" s="38"/>
     </x:row>
     <x:row r="24" ht="31">
       <x:c r="A24" s="2" t="s">
@@ -2737,17 +2775,17 @@
       <x:c r="L24" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M24" s="29"/>
-      <x:c r="N24" s="30" t="str">
+      <x:c r="M24" s="36"/>
+      <x:c r="N24" s="37" t="str">
         <x:f>IF(M24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
       </x:c>
-      <x:c r="O24" s="30" t="str">
+      <x:c r="O24" s="37" t="str">
         <x:f>IF(M24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K24&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P24" s="30" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N24)&amp;"&amp;body="&amp;ENCODEURL(O24),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q24" s="31"/>
+      <x:c r="P24" s="37" t="str">
+        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N24,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O24,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q24" s="38"/>
     </x:row>
     <x:row r="25" ht="31">
       <x:c r="A25" s="2" t="s">
@@ -2786,17 +2824,17 @@
       <x:c r="L25" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M25" s="29"/>
-      <x:c r="N25" s="30" t="str">
+      <x:c r="M25" s="36"/>
+      <x:c r="N25" s="37" t="str">
         <x:f>IF(M25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
       </x:c>
-      <x:c r="O25" s="30" t="str">
+      <x:c r="O25" s="37" t="str">
         <x:f>IF(M25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K25&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P25" s="30" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N25)&amp;"&amp;body="&amp;ENCODEURL(O25),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q25" s="31"/>
+      <x:c r="P25" s="37" t="str">
+        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N25,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O25,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q25" s="38"/>
     </x:row>
     <x:row r="26" ht="31">
       <x:c r="A26" s="2" t="s">
@@ -2835,17 +2873,17 @@
       <x:c r="L26" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M26" s="29"/>
-      <x:c r="N26" s="30" t="str">
+      <x:c r="M26" s="36"/>
+      <x:c r="N26" s="37" t="str">
         <x:f>IF(M26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
       </x:c>
-      <x:c r="O26" s="30" t="str">
+      <x:c r="O26" s="37" t="str">
         <x:f>IF(M26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K26&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P26" s="30" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N26)&amp;"&amp;body="&amp;ENCODEURL(O26),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q26" s="31"/>
+      <x:c r="P26" s="37" t="str">
+        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N26,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O26,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q26" s="38"/>
     </x:row>
     <x:row r="27" ht="31">
       <x:c r="A27" s="2" t="s">
@@ -2884,17 +2922,17 @@
       <x:c r="L27" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M27" s="29"/>
-      <x:c r="N27" s="30" t="str">
+      <x:c r="M27" s="36"/>
+      <x:c r="N27" s="37" t="str">
         <x:f>IF(M27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
       </x:c>
-      <x:c r="O27" s="30" t="str">
+      <x:c r="O27" s="37" t="str">
         <x:f>IF(M27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K27&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P27" s="30" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N27)&amp;"&amp;body="&amp;ENCODEURL(O27),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q27" s="31"/>
+      <x:c r="P27" s="37" t="str">
+        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N27,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O27,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q27" s="38"/>
     </x:row>
     <x:row r="28" ht="46">
       <x:c r="A28" s="2" t="s">
@@ -2933,17 +2971,17 @@
       <x:c r="L28" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M28" s="29"/>
-      <x:c r="N28" s="30" t="str">
+      <x:c r="M28" s="36"/>
+      <x:c r="N28" s="37" t="str">
         <x:f>IF(M28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
       </x:c>
-      <x:c r="O28" s="30" t="str">
+      <x:c r="O28" s="37" t="str">
         <x:f>IF(M28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K28&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P28" s="30" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N28)&amp;"&amp;body="&amp;ENCODEURL(O28),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q28" s="31"/>
+      <x:c r="P28" s="37" t="str">
+        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N28,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O28,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q28" s="38"/>
     </x:row>
     <x:row r="29" ht="46">
       <x:c r="A29" s="2" t="s">
@@ -2982,17 +3020,17 @@
       <x:c r="L29" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M29" s="29"/>
-      <x:c r="N29" s="30" t="str">
+      <x:c r="M29" s="36"/>
+      <x:c r="N29" s="37" t="str">
         <x:f>IF(M29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
       </x:c>
-      <x:c r="O29" s="30" t="str">
+      <x:c r="O29" s="37" t="str">
         <x:f>IF(M29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K29&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P29" s="30" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N29)&amp;"&amp;body="&amp;ENCODEURL(O29),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q29" s="31"/>
+      <x:c r="P29" s="37" t="str">
+        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N29,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O29,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q29" s="38"/>
     </x:row>
     <x:row r="30" ht="31">
       <x:c r="A30" s="2" t="s">
@@ -3031,17 +3069,17 @@
       <x:c r="L30" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M30" s="29"/>
-      <x:c r="N30" s="30" t="str">
+      <x:c r="M30" s="36"/>
+      <x:c r="N30" s="37" t="str">
         <x:f>IF(M30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
       </x:c>
-      <x:c r="O30" s="30" t="str">
+      <x:c r="O30" s="37" t="str">
         <x:f>IF(M30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K30&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P30" s="30" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N30)&amp;"&amp;body="&amp;ENCODEURL(O30),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q30" s="31"/>
+      <x:c r="P30" s="37" t="str">
+        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N30,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O30,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q30" s="38"/>
     </x:row>
     <x:row r="31" ht="31">
       <x:c r="A31" s="2" t="s">
@@ -3080,17 +3118,17 @@
       <x:c r="L31" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M31" s="29"/>
-      <x:c r="N31" s="30" t="str">
+      <x:c r="M31" s="36"/>
+      <x:c r="N31" s="37" t="str">
         <x:f>IF(M31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
       </x:c>
-      <x:c r="O31" s="30" t="str">
+      <x:c r="O31" s="37" t="str">
         <x:f>IF(M31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K31&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P31" s="30" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N31)&amp;"&amp;body="&amp;ENCODEURL(O31),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q31" s="31"/>
+      <x:c r="P31" s="37" t="str">
+        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N31,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O31,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q31" s="38"/>
     </x:row>
     <x:row r="32" ht="46">
       <x:c r="A32" s="2" t="s">
@@ -3129,17 +3167,17 @@
       <x:c r="L32" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M32" s="29"/>
-      <x:c r="N32" s="30" t="str">
+      <x:c r="M32" s="36"/>
+      <x:c r="N32" s="37" t="str">
         <x:f>IF(M32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
       </x:c>
-      <x:c r="O32" s="30" t="str">
+      <x:c r="O32" s="37" t="str">
         <x:f>IF(M32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K32&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P32" s="30" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N32)&amp;"&amp;body="&amp;ENCODEURL(O32),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q32" s="31"/>
+      <x:c r="P32" s="37" t="str">
+        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N32,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O32,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q32" s="38"/>
     </x:row>
     <x:row r="33" ht="61">
       <x:c r="A33" s="2" t="s">
@@ -3178,17 +3216,17 @@
       <x:c r="L33" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M33" s="29"/>
-      <x:c r="N33" s="30" t="str">
+      <x:c r="M33" s="36"/>
+      <x:c r="N33" s="37" t="str">
         <x:f>IF(M33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
       </x:c>
-      <x:c r="O33" s="30" t="str">
+      <x:c r="O33" s="37" t="str">
         <x:f>IF(M33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K33&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P33" s="30" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N33)&amp;"&amp;body="&amp;ENCODEURL(O33),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q33" s="31"/>
+      <x:c r="P33" s="37" t="str">
+        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N33,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O33,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q33" s="38"/>
     </x:row>
     <x:row r="34" ht="46">
       <x:c r="A34" s="2" t="s">
@@ -3227,17 +3265,17 @@
       <x:c r="L34" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M34" s="29"/>
-      <x:c r="N34" s="30" t="str">
+      <x:c r="M34" s="36"/>
+      <x:c r="N34" s="37" t="str">
         <x:f>IF(M34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
       </x:c>
-      <x:c r="O34" s="30" t="str">
+      <x:c r="O34" s="37" t="str">
         <x:f>IF(M34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K34&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P34" s="30" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N34)&amp;"&amp;body="&amp;ENCODEURL(O34),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q34" s="31"/>
+      <x:c r="P34" s="37" t="str">
+        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N34,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O34,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q34" s="38"/>
     </x:row>
     <x:row r="35" ht="31">
       <x:c r="A35" s="2" t="s">
@@ -3276,17 +3314,17 @@
       <x:c r="L35" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M35" s="29"/>
-      <x:c r="N35" s="30" t="str">
+      <x:c r="M35" s="36"/>
+      <x:c r="N35" s="37" t="str">
         <x:f>IF(M35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
       </x:c>
-      <x:c r="O35" s="30" t="str">
+      <x:c r="O35" s="37" t="str">
         <x:f>IF(M35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K35&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P35" s="30" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N35)&amp;"&amp;body="&amp;ENCODEURL(O35),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q35" s="31"/>
+      <x:c r="P35" s="37" t="str">
+        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N35,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O35,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q35" s="38"/>
     </x:row>
     <x:row r="36" ht="31">
       <x:c r="A36" s="2" t="s">
@@ -3325,17 +3363,17 @@
       <x:c r="L36" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M36" s="29"/>
-      <x:c r="N36" s="30" t="str">
+      <x:c r="M36" s="36"/>
+      <x:c r="N36" s="37" t="str">
         <x:f>IF(M36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
       </x:c>
-      <x:c r="O36" s="30" t="str">
+      <x:c r="O36" s="37" t="str">
         <x:f>IF(M36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K36&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P36" s="30" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N36)&amp;"&amp;body="&amp;ENCODEURL(O36),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q36" s="31"/>
+      <x:c r="P36" s="37" t="str">
+        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N36,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O36,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q36" s="38"/>
     </x:row>
     <x:row r="37" ht="31">
       <x:c r="A37" s="2" t="s">
@@ -3374,17 +3412,17 @@
       <x:c r="L37" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M37" s="29"/>
-      <x:c r="N37" s="30" t="str">
+      <x:c r="M37" s="36"/>
+      <x:c r="N37" s="37" t="str">
         <x:f>IF(M37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
       </x:c>
-      <x:c r="O37" s="30" t="str">
+      <x:c r="O37" s="37" t="str">
         <x:f>IF(M37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K37&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P37" s="30" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N37)&amp;"&amp;body="&amp;ENCODEURL(O37),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q37" s="31"/>
+      <x:c r="P37" s="37" t="str">
+        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N37,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O37,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q37" s="38"/>
     </x:row>
     <x:row r="38" ht="31">
       <x:c r="A38" s="2" t="s">
@@ -3423,17 +3461,17 @@
       <x:c r="L38" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M38" s="29"/>
-      <x:c r="N38" s="30" t="str">
+      <x:c r="M38" s="36"/>
+      <x:c r="N38" s="37" t="str">
         <x:f>IF(M38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
       </x:c>
-      <x:c r="O38" s="30" t="str">
+      <x:c r="O38" s="37" t="str">
         <x:f>IF(M38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K38&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P38" s="30" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N38)&amp;"&amp;body="&amp;ENCODEURL(O38),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q38" s="31"/>
+      <x:c r="P38" s="37" t="str">
+        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N38,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O38,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q38" s="38"/>
     </x:row>
     <x:row r="39" ht="31">
       <x:c r="A39" s="2" t="s">
@@ -3472,17 +3510,17 @@
       <x:c r="L39" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M39" s="29"/>
-      <x:c r="N39" s="30" t="str">
+      <x:c r="M39" s="36"/>
+      <x:c r="N39" s="37" t="str">
         <x:f>IF(M39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
       </x:c>
-      <x:c r="O39" s="30" t="str">
+      <x:c r="O39" s="37" t="str">
         <x:f>IF(M39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K39&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P39" s="30" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N39)&amp;"&amp;body="&amp;ENCODEURL(O39),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q39" s="31"/>
+      <x:c r="P39" s="37" t="str">
+        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N39,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O39,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q39" s="38"/>
     </x:row>
     <x:row r="40" ht="31">
       <x:c r="A40" s="2" t="s">
@@ -3521,17 +3559,17 @@
       <x:c r="L40" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M40" s="29"/>
-      <x:c r="N40" s="30" t="str">
+      <x:c r="M40" s="36"/>
+      <x:c r="N40" s="37" t="str">
         <x:f>IF(M40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
       </x:c>
-      <x:c r="O40" s="30" t="str">
+      <x:c r="O40" s="37" t="str">
         <x:f>IF(M40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K40&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P40" s="30" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N40)&amp;"&amp;body="&amp;ENCODEURL(O40),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q40" s="31"/>
+      <x:c r="P40" s="37" t="str">
+        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N40,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O40,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q40" s="38"/>
     </x:row>
     <x:row r="41" ht="45">
       <x:c r="A41" s="2" t="s">
@@ -3570,17 +3608,17 @@
       <x:c r="L41" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M41" s="29"/>
-      <x:c r="N41" s="30" t="str">
+      <x:c r="M41" s="36"/>
+      <x:c r="N41" s="37" t="str">
         <x:f>IF(M41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
       </x:c>
-      <x:c r="O41" s="30" t="str">
+      <x:c r="O41" s="37" t="str">
         <x:f>IF(M41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K41&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P41" s="30" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N41)&amp;"&amp;body="&amp;ENCODEURL(O41),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q41" s="31"/>
+      <x:c r="P41" s="37" t="str">
+        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N41,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O41,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q41" s="38"/>
     </x:row>
     <x:row r="42" ht="45">
       <x:c r="A42" s="2" t="s">
@@ -3619,17 +3657,17 @@
       <x:c r="L42" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M42" s="29"/>
-      <x:c r="N42" s="30" t="str">
+      <x:c r="M42" s="36"/>
+      <x:c r="N42" s="37" t="str">
         <x:f>IF(M42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
       </x:c>
-      <x:c r="O42" s="30" t="str">
+      <x:c r="O42" s="37" t="str">
         <x:f>IF(M42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K42&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
       </x:c>
-      <x:c r="P42" s="30" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;ENCODEURL(N42)&amp;"&amp;body="&amp;ENCODEURL(O42),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q42" s="31"/>
+      <x:c r="P42" s="37" t="str">
+        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N42,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O42,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
+      </x:c>
+      <x:c r="Q42" s="38"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
@@ -3650,7 +3688,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35649410c1e849d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27120be6cc1d44c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3814,15 +3852,15 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
-      <x:c r="A21" s="34" t="str">
+      <x:c r="A21" s="40" t="str">
         <x:v>Email draft workflow</x:v>
       </x:c>
-      <x:c r="B21" s="34" t="str">
+      <x:c r="B21" s="40" t="str">
         <x:v>Use the final five columns of the Funding opportunities table to prepare an Outlook email without sending it automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="35" t="str">
+      <x:c r="A22" s="41" t="str">
         <x:v>Step 1</x:v>
       </x:c>
       <x:c r="B22" s="28" t="str">
@@ -3830,7 +3868,7 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="35" t="str">
+      <x:c r="A23" s="41" t="str">
         <x:v>Step 2</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
@@ -3838,7 +3876,7 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="35" t="str">
+      <x:c r="A24" s="41" t="str">
         <x:v>Step 3</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
@@ -3846,7 +3884,7 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="35" t="str">
+      <x:c r="A25" s="41" t="str">
         <x:v>Step 4</x:v>
       </x:c>
       <x:c r="B25" s="28" t="str">

</xml_diff>

<commit_message>
Replace email draft action with hyperlink fields
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R000feaed12d34dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Red235a641382445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R524526c8ae454713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Radc8776f72584b17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1137,12 +1137,32 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -1221,7 +1241,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1324,6 +1344,50 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
@@ -1368,9 +1432,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:Q42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:Q42"/>
-  <x:tableColumns count="17">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:R42"/>
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Deadline"/>
     <x:tableColumn id="3" name="Funder"/>
@@ -1386,8 +1450,9 @@
     <x:tableColumn id="13" name="Notify?"/>
     <x:tableColumn id="14" name="Email subject"/>
     <x:tableColumn id="15" name="Email body"/>
-    <x:tableColumn id="16" name="Open email draft"/>
-    <x:tableColumn id="17" name="Notification date"/>
+    <x:tableColumn id="16" name="Official opportunity link"/>
+    <x:tableColumn id="17" name="Funding Finder link"/>
+    <x:tableColumn id="18" name="Notification date"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1603,8 +1668,9 @@
     <x:col min="13" max="13" width="11" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="32" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="45.25" customHeight="1">
@@ -1644,19 +1710,22 @@
       <x:c r="L1" s="1" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="39" t="str">
+      <x:c r="M1" s="53" t="str">
         <x:v>Notify?</x:v>
       </x:c>
-      <x:c r="N1" s="39" t="str">
+      <x:c r="N1" s="53" t="str">
         <x:v>Email subject</x:v>
       </x:c>
-      <x:c r="O1" s="39" t="str">
+      <x:c r="O1" s="53" t="str">
         <x:v>Email body</x:v>
       </x:c>
-      <x:c r="P1" s="39" t="str">
-        <x:v>Open email draft</x:v>
-      </x:c>
-      <x:c r="Q1" s="39" t="str">
+      <x:c r="P1" s="53" t="str">
+        <x:v>Official opportunity link</x:v>
+      </x:c>
+      <x:c r="Q1" s="53" t="str">
+        <x:v>Funding Finder link</x:v>
+      </x:c>
+      <x:c r="R1" s="53" t="str">
         <x:v>Notification date</x:v>
       </x:c>
     </x:row>
@@ -1697,17 +1766,20 @@
       <x:c r="L2" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M2" s="36"/>
-      <x:c r="N2" s="37" t="str">
+      <x:c r="M2" s="42"/>
+      <x:c r="N2" s="43" t="str">
         <x:f>IF(M2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
       </x:c>
-      <x:c r="O2" s="37" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K2&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P2" s="37" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N2,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O2,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q2" s="38"/>
+      <x:c r="O2" s="43" t="str">
+        <x:f>IF(M2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P2" s="43" t="str">
+        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK(K2,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q2" s="47" t="str">
+        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R2" s="52"/>
     </x:row>
     <x:row r="3" ht="31">
       <x:c r="A3" s="2" t="s">
@@ -1746,17 +1818,20 @@
       <x:c r="L3" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M3" s="36"/>
-      <x:c r="N3" s="37" t="str">
+      <x:c r="M3" s="42"/>
+      <x:c r="N3" s="43" t="str">
         <x:f>IF(M3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
       </x:c>
-      <x:c r="O3" s="37" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K3&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P3" s="37" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N3,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O3,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q3" s="38"/>
+      <x:c r="O3" s="43" t="str">
+        <x:f>IF(M3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P3" s="43" t="str">
+        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK(K3,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q3" s="47" t="str">
+        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R3" s="52"/>
     </x:row>
     <x:row r="4" ht="31">
       <x:c r="A4" s="2" t="s">
@@ -1795,17 +1870,20 @@
       <x:c r="L4" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M4" s="36"/>
-      <x:c r="N4" s="37" t="str">
+      <x:c r="M4" s="42"/>
+      <x:c r="N4" s="43" t="str">
         <x:f>IF(M4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
       </x:c>
-      <x:c r="O4" s="37" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K4&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P4" s="37" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N4,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O4,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q4" s="38"/>
+      <x:c r="O4" s="43" t="str">
+        <x:f>IF(M4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P4" s="43" t="str">
+        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK(K4,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q4" s="47" t="str">
+        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R4" s="52"/>
     </x:row>
     <x:row r="5" ht="46">
       <x:c r="A5" s="2" t="s">
@@ -1844,17 +1922,20 @@
       <x:c r="L5" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M5" s="36"/>
-      <x:c r="N5" s="37" t="str">
+      <x:c r="M5" s="42"/>
+      <x:c r="N5" s="43" t="str">
         <x:f>IF(M5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
       </x:c>
-      <x:c r="O5" s="37" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K5&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P5" s="37" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N5,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O5,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q5" s="38"/>
+      <x:c r="O5" s="43" t="str">
+        <x:f>IF(M5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P5" s="43" t="str">
+        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK(K5,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q5" s="47" t="str">
+        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R5" s="52"/>
     </x:row>
     <x:row r="6" ht="31">
       <x:c r="A6" s="2" t="s">
@@ -1893,17 +1974,20 @@
       <x:c r="L6" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M6" s="36"/>
-      <x:c r="N6" s="37" t="str">
+      <x:c r="M6" s="42"/>
+      <x:c r="N6" s="43" t="str">
         <x:f>IF(M6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
       </x:c>
-      <x:c r="O6" s="37" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K6&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P6" s="37" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N6,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O6,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q6" s="38"/>
+      <x:c r="O6" s="43" t="str">
+        <x:f>IF(M6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P6" s="43" t="str">
+        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK(K6,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q6" s="47" t="str">
+        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R6" s="52"/>
     </x:row>
     <x:row r="7" ht="31">
       <x:c r="A7" s="2" t="s">
@@ -1942,17 +2026,20 @@
       <x:c r="L7" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M7" s="36"/>
-      <x:c r="N7" s="37" t="str">
+      <x:c r="M7" s="42"/>
+      <x:c r="N7" s="43" t="str">
         <x:f>IF(M7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
       </x:c>
-      <x:c r="O7" s="37" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K7&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P7" s="37" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N7,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O7,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q7" s="38"/>
+      <x:c r="O7" s="43" t="str">
+        <x:f>IF(M7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P7" s="43" t="str">
+        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK(K7,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q7" s="47" t="str">
+        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R7" s="52"/>
     </x:row>
     <x:row r="8" ht="46">
       <x:c r="A8" s="2" t="s">
@@ -1991,17 +2078,20 @@
       <x:c r="L8" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M8" s="36"/>
-      <x:c r="N8" s="37" t="str">
+      <x:c r="M8" s="42"/>
+      <x:c r="N8" s="43" t="str">
         <x:f>IF(M8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
       </x:c>
-      <x:c r="O8" s="37" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K8&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P8" s="37" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N8,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O8,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q8" s="38"/>
+      <x:c r="O8" s="43" t="str">
+        <x:f>IF(M8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P8" s="43" t="str">
+        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK(K8,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q8" s="47" t="str">
+        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R8" s="52"/>
     </x:row>
     <x:row r="9" ht="31">
       <x:c r="A9" s="2" t="s">
@@ -2040,17 +2130,20 @@
       <x:c r="L9" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M9" s="36"/>
-      <x:c r="N9" s="37" t="str">
+      <x:c r="M9" s="42"/>
+      <x:c r="N9" s="43" t="str">
         <x:f>IF(M9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
       </x:c>
-      <x:c r="O9" s="37" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K9&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P9" s="37" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N9,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O9,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q9" s="38"/>
+      <x:c r="O9" s="43" t="str">
+        <x:f>IF(M9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P9" s="43" t="str">
+        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK(K9,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q9" s="47" t="str">
+        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R9" s="52"/>
     </x:row>
     <x:row r="10" ht="31">
       <x:c r="A10" s="2" t="s">
@@ -2089,17 +2182,20 @@
       <x:c r="L10" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M10" s="36"/>
-      <x:c r="N10" s="37" t="str">
+      <x:c r="M10" s="42"/>
+      <x:c r="N10" s="43" t="str">
         <x:f>IF(M10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
       </x:c>
-      <x:c r="O10" s="37" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K10&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P10" s="37" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N10,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O10,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q10" s="38"/>
+      <x:c r="O10" s="43" t="str">
+        <x:f>IF(M10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P10" s="43" t="str">
+        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK(K10,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q10" s="47" t="str">
+        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R10" s="52"/>
     </x:row>
     <x:row r="11" ht="31">
       <x:c r="A11" s="2" t="s">
@@ -2138,17 +2234,20 @@
       <x:c r="L11" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M11" s="36"/>
-      <x:c r="N11" s="37" t="str">
+      <x:c r="M11" s="42"/>
+      <x:c r="N11" s="43" t="str">
         <x:f>IF(M11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
       </x:c>
-      <x:c r="O11" s="37" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K11&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P11" s="37" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N11,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O11,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q11" s="38"/>
+      <x:c r="O11" s="43" t="str">
+        <x:f>IF(M11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P11" s="43" t="str">
+        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK(K11,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q11" s="47" t="str">
+        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R11" s="52"/>
     </x:row>
     <x:row r="12" ht="31">
       <x:c r="A12" s="2" t="s">
@@ -2187,17 +2286,20 @@
       <x:c r="L12" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M12" s="36"/>
-      <x:c r="N12" s="37" t="str">
+      <x:c r="M12" s="42"/>
+      <x:c r="N12" s="43" t="str">
         <x:f>IF(M12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
       </x:c>
-      <x:c r="O12" s="37" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K12&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P12" s="37" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N12,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O12,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q12" s="38"/>
+      <x:c r="O12" s="43" t="str">
+        <x:f>IF(M12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P12" s="43" t="str">
+        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK(K12,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q12" s="47" t="str">
+        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R12" s="52"/>
     </x:row>
     <x:row r="13" ht="31">
       <x:c r="A13" s="2" t="s">
@@ -2236,17 +2338,20 @@
       <x:c r="L13" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M13" s="36"/>
-      <x:c r="N13" s="37" t="str">
+      <x:c r="M13" s="42"/>
+      <x:c r="N13" s="43" t="str">
         <x:f>IF(M13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
       </x:c>
-      <x:c r="O13" s="37" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K13&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P13" s="37" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N13,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O13,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q13" s="38"/>
+      <x:c r="O13" s="43" t="str">
+        <x:f>IF(M13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P13" s="43" t="str">
+        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK(K13,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q13" s="47" t="str">
+        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R13" s="52"/>
     </x:row>
     <x:row r="14" ht="46">
       <x:c r="A14" s="2" t="s">
@@ -2285,17 +2390,20 @@
       <x:c r="L14" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M14" s="36"/>
-      <x:c r="N14" s="37" t="str">
+      <x:c r="M14" s="42"/>
+      <x:c r="N14" s="43" t="str">
         <x:f>IF(M14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
       </x:c>
-      <x:c r="O14" s="37" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K14&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P14" s="37" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N14,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O14,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q14" s="38"/>
+      <x:c r="O14" s="43" t="str">
+        <x:f>IF(M14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P14" s="43" t="str">
+        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK(K14,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q14" s="47" t="str">
+        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R14" s="52"/>
     </x:row>
     <x:row r="15" ht="46">
       <x:c r="A15" s="2" t="s">
@@ -2334,17 +2442,20 @@
       <x:c r="L15" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M15" s="36"/>
-      <x:c r="N15" s="37" t="str">
+      <x:c r="M15" s="42"/>
+      <x:c r="N15" s="43" t="str">
         <x:f>IF(M15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
       </x:c>
-      <x:c r="O15" s="37" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K15&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P15" s="37" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N15,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O15,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q15" s="38"/>
+      <x:c r="O15" s="43" t="str">
+        <x:f>IF(M15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P15" s="43" t="str">
+        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK(K15,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q15" s="47" t="str">
+        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R15" s="52"/>
     </x:row>
     <x:row r="16" ht="31">
       <x:c r="A16" s="2" t="s">
@@ -2383,17 +2494,20 @@
       <x:c r="L16" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M16" s="36"/>
-      <x:c r="N16" s="37" t="str">
+      <x:c r="M16" s="42"/>
+      <x:c r="N16" s="43" t="str">
         <x:f>IF(M16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
       </x:c>
-      <x:c r="O16" s="37" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K16&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P16" s="37" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N16,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O16,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q16" s="38"/>
+      <x:c r="O16" s="43" t="str">
+        <x:f>IF(M16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P16" s="43" t="str">
+        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK(K16,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q16" s="47" t="str">
+        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R16" s="52"/>
     </x:row>
     <x:row r="17" ht="31">
       <x:c r="A17" s="2" t="s">
@@ -2432,17 +2546,20 @@
       <x:c r="L17" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M17" s="36"/>
-      <x:c r="N17" s="37" t="str">
+      <x:c r="M17" s="42"/>
+      <x:c r="N17" s="43" t="str">
         <x:f>IF(M17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
       </x:c>
-      <x:c r="O17" s="37" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K17&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P17" s="37" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N17,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O17,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q17" s="38"/>
+      <x:c r="O17" s="43" t="str">
+        <x:f>IF(M17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P17" s="43" t="str">
+        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK(K17,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q17" s="47" t="str">
+        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R17" s="52"/>
     </x:row>
     <x:row r="18" ht="46">
       <x:c r="A18" s="2" t="s">
@@ -2481,17 +2598,20 @@
       <x:c r="L18" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M18" s="36"/>
-      <x:c r="N18" s="37" t="str">
+      <x:c r="M18" s="42"/>
+      <x:c r="N18" s="43" t="str">
         <x:f>IF(M18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
       </x:c>
-      <x:c r="O18" s="37" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K18&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P18" s="37" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N18,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O18,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q18" s="38"/>
+      <x:c r="O18" s="43" t="str">
+        <x:f>IF(M18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P18" s="43" t="str">
+        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK(K18,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q18" s="47" t="str">
+        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R18" s="52"/>
     </x:row>
     <x:row r="19" ht="31">
       <x:c r="A19" s="2" t="s">
@@ -2530,17 +2650,20 @@
       <x:c r="L19" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M19" s="36"/>
-      <x:c r="N19" s="37" t="str">
+      <x:c r="M19" s="42"/>
+      <x:c r="N19" s="43" t="str">
         <x:f>IF(M19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
       </x:c>
-      <x:c r="O19" s="37" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K19&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P19" s="37" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N19,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O19,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q19" s="38"/>
+      <x:c r="O19" s="43" t="str">
+        <x:f>IF(M19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P19" s="43" t="str">
+        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK(K19,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q19" s="47" t="str">
+        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R19" s="52"/>
     </x:row>
     <x:row r="20" ht="46">
       <x:c r="A20" s="2" t="s">
@@ -2579,17 +2702,20 @@
       <x:c r="L20" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M20" s="36"/>
-      <x:c r="N20" s="37" t="str">
+      <x:c r="M20" s="42"/>
+      <x:c r="N20" s="43" t="str">
         <x:f>IF(M20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
       </x:c>
-      <x:c r="O20" s="37" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K20&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P20" s="37" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N20,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O20,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q20" s="38"/>
+      <x:c r="O20" s="43" t="str">
+        <x:f>IF(M20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P20" s="43" t="str">
+        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK(K20,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q20" s="47" t="str">
+        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R20" s="52"/>
     </x:row>
     <x:row r="21" ht="31">
       <x:c r="A21" s="2" t="s">
@@ -2628,17 +2754,20 @@
       <x:c r="L21" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="M21" s="36"/>
-      <x:c r="N21" s="37" t="str">
+      <x:c r="M21" s="42"/>
+      <x:c r="N21" s="43" t="str">
         <x:f>IF(M21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
       </x:c>
-      <x:c r="O21" s="37" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K21&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P21" s="37" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N21,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O21,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q21" s="38"/>
+      <x:c r="O21" s="43" t="str">
+        <x:f>IF(M21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P21" s="43" t="str">
+        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK(K21,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q21" s="47" t="str">
+        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R21" s="52"/>
     </x:row>
     <x:row r="22" ht="31">
       <x:c r="A22" s="2" t="s">
@@ -2677,17 +2806,20 @@
       <x:c r="L22" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M22" s="36"/>
-      <x:c r="N22" s="37" t="str">
+      <x:c r="M22" s="42"/>
+      <x:c r="N22" s="43" t="str">
         <x:f>IF(M22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
       </x:c>
-      <x:c r="O22" s="37" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K22&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P22" s="37" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N22,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O22,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q22" s="38"/>
+      <x:c r="O22" s="43" t="str">
+        <x:f>IF(M22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P22" s="43" t="str">
+        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK(K22,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q22" s="47" t="str">
+        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R22" s="52"/>
     </x:row>
     <x:row r="23" ht="31">
       <x:c r="A23" s="2" t="s">
@@ -2726,17 +2858,20 @@
       <x:c r="L23" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M23" s="36"/>
-      <x:c r="N23" s="37" t="str">
+      <x:c r="M23" s="42"/>
+      <x:c r="N23" s="43" t="str">
         <x:f>IF(M23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
       </x:c>
-      <x:c r="O23" s="37" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K23&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P23" s="37" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N23,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O23,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q23" s="38"/>
+      <x:c r="O23" s="43" t="str">
+        <x:f>IF(M23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P23" s="43" t="str">
+        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK(K23,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q23" s="47" t="str">
+        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R23" s="52"/>
     </x:row>
     <x:row r="24" ht="31">
       <x:c r="A24" s="2" t="s">
@@ -2775,17 +2910,20 @@
       <x:c r="L24" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M24" s="36"/>
-      <x:c r="N24" s="37" t="str">
+      <x:c r="M24" s="42"/>
+      <x:c r="N24" s="43" t="str">
         <x:f>IF(M24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
       </x:c>
-      <x:c r="O24" s="37" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K24&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P24" s="37" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N24,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O24,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q24" s="38"/>
+      <x:c r="O24" s="43" t="str">
+        <x:f>IF(M24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P24" s="43" t="str">
+        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK(K24,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q24" s="47" t="str">
+        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R24" s="52"/>
     </x:row>
     <x:row r="25" ht="31">
       <x:c r="A25" s="2" t="s">
@@ -2824,17 +2962,20 @@
       <x:c r="L25" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M25" s="36"/>
-      <x:c r="N25" s="37" t="str">
+      <x:c r="M25" s="42"/>
+      <x:c r="N25" s="43" t="str">
         <x:f>IF(M25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
       </x:c>
-      <x:c r="O25" s="37" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K25&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P25" s="37" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N25,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O25,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q25" s="38"/>
+      <x:c r="O25" s="43" t="str">
+        <x:f>IF(M25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P25" s="43" t="str">
+        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK(K25,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q25" s="47" t="str">
+        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R25" s="52"/>
     </x:row>
     <x:row r="26" ht="31">
       <x:c r="A26" s="2" t="s">
@@ -2873,17 +3014,20 @@
       <x:c r="L26" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M26" s="36"/>
-      <x:c r="N26" s="37" t="str">
+      <x:c r="M26" s="42"/>
+      <x:c r="N26" s="43" t="str">
         <x:f>IF(M26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
       </x:c>
-      <x:c r="O26" s="37" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K26&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P26" s="37" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N26,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O26,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q26" s="38"/>
+      <x:c r="O26" s="43" t="str">
+        <x:f>IF(M26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P26" s="43" t="str">
+        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK(K26,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q26" s="47" t="str">
+        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R26" s="52"/>
     </x:row>
     <x:row r="27" ht="31">
       <x:c r="A27" s="2" t="s">
@@ -2922,17 +3066,20 @@
       <x:c r="L27" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="M27" s="36"/>
-      <x:c r="N27" s="37" t="str">
+      <x:c r="M27" s="42"/>
+      <x:c r="N27" s="43" t="str">
         <x:f>IF(M27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
       </x:c>
-      <x:c r="O27" s="37" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K27&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P27" s="37" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N27,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O27,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q27" s="38"/>
+      <x:c r="O27" s="43" t="str">
+        <x:f>IF(M27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P27" s="43" t="str">
+        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK(K27,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q27" s="47" t="str">
+        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R27" s="52"/>
     </x:row>
     <x:row r="28" ht="46">
       <x:c r="A28" s="2" t="s">
@@ -2971,17 +3118,20 @@
       <x:c r="L28" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M28" s="36"/>
-      <x:c r="N28" s="37" t="str">
+      <x:c r="M28" s="42"/>
+      <x:c r="N28" s="43" t="str">
         <x:f>IF(M28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
       </x:c>
-      <x:c r="O28" s="37" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K28&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P28" s="37" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N28,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O28,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q28" s="38"/>
+      <x:c r="O28" s="43" t="str">
+        <x:f>IF(M28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P28" s="43" t="str">
+        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK(K28,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q28" s="47" t="str">
+        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R28" s="52"/>
     </x:row>
     <x:row r="29" ht="46">
       <x:c r="A29" s="2" t="s">
@@ -3020,17 +3170,20 @@
       <x:c r="L29" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M29" s="36"/>
-      <x:c r="N29" s="37" t="str">
+      <x:c r="M29" s="42"/>
+      <x:c r="N29" s="43" t="str">
         <x:f>IF(M29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
       </x:c>
-      <x:c r="O29" s="37" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K29&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P29" s="37" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N29,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O29,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q29" s="38"/>
+      <x:c r="O29" s="43" t="str">
+        <x:f>IF(M29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P29" s="43" t="str">
+        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK(K29,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q29" s="47" t="str">
+        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R29" s="52"/>
     </x:row>
     <x:row r="30" ht="31">
       <x:c r="A30" s="2" t="s">
@@ -3069,17 +3222,20 @@
       <x:c r="L30" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M30" s="36"/>
-      <x:c r="N30" s="37" t="str">
+      <x:c r="M30" s="42"/>
+      <x:c r="N30" s="43" t="str">
         <x:f>IF(M30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
       </x:c>
-      <x:c r="O30" s="37" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K30&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P30" s="37" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N30,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O30,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q30" s="38"/>
+      <x:c r="O30" s="43" t="str">
+        <x:f>IF(M30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P30" s="43" t="str">
+        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK(K30,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q30" s="47" t="str">
+        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R30" s="52"/>
     </x:row>
     <x:row r="31" ht="31">
       <x:c r="A31" s="2" t="s">
@@ -3118,17 +3274,20 @@
       <x:c r="L31" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M31" s="36"/>
-      <x:c r="N31" s="37" t="str">
+      <x:c r="M31" s="42"/>
+      <x:c r="N31" s="43" t="str">
         <x:f>IF(M31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
       </x:c>
-      <x:c r="O31" s="37" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K31&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P31" s="37" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N31,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O31,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q31" s="38"/>
+      <x:c r="O31" s="43" t="str">
+        <x:f>IF(M31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P31" s="43" t="str">
+        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK(K31,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q31" s="47" t="str">
+        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R31" s="52"/>
     </x:row>
     <x:row r="32" ht="46">
       <x:c r="A32" s="2" t="s">
@@ -3167,17 +3326,20 @@
       <x:c r="L32" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M32" s="36"/>
-      <x:c r="N32" s="37" t="str">
+      <x:c r="M32" s="42"/>
+      <x:c r="N32" s="43" t="str">
         <x:f>IF(M32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
       </x:c>
-      <x:c r="O32" s="37" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K32&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P32" s="37" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N32,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O32,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q32" s="38"/>
+      <x:c r="O32" s="43" t="str">
+        <x:f>IF(M32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P32" s="43" t="str">
+        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK(K32,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q32" s="47" t="str">
+        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R32" s="52"/>
     </x:row>
     <x:row r="33" ht="61">
       <x:c r="A33" s="2" t="s">
@@ -3216,17 +3378,20 @@
       <x:c r="L33" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M33" s="36"/>
-      <x:c r="N33" s="37" t="str">
+      <x:c r="M33" s="42"/>
+      <x:c r="N33" s="43" t="str">
         <x:f>IF(M33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
       </x:c>
-      <x:c r="O33" s="37" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K33&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P33" s="37" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N33,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O33,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q33" s="38"/>
+      <x:c r="O33" s="43" t="str">
+        <x:f>IF(M33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P33" s="43" t="str">
+        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK(K33,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q33" s="47" t="str">
+        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R33" s="52"/>
     </x:row>
     <x:row r="34" ht="46">
       <x:c r="A34" s="2" t="s">
@@ -3265,17 +3430,20 @@
       <x:c r="L34" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M34" s="36"/>
-      <x:c r="N34" s="37" t="str">
+      <x:c r="M34" s="42"/>
+      <x:c r="N34" s="43" t="str">
         <x:f>IF(M34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
       </x:c>
-      <x:c r="O34" s="37" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K34&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P34" s="37" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N34,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O34,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q34" s="38"/>
+      <x:c r="O34" s="43" t="str">
+        <x:f>IF(M34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P34" s="43" t="str">
+        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK(K34,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q34" s="47" t="str">
+        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R34" s="52"/>
     </x:row>
     <x:row r="35" ht="31">
       <x:c r="A35" s="2" t="s">
@@ -3314,17 +3482,20 @@
       <x:c r="L35" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M35" s="36"/>
-      <x:c r="N35" s="37" t="str">
+      <x:c r="M35" s="42"/>
+      <x:c r="N35" s="43" t="str">
         <x:f>IF(M35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
       </x:c>
-      <x:c r="O35" s="37" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K35&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P35" s="37" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N35,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O35,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q35" s="38"/>
+      <x:c r="O35" s="43" t="str">
+        <x:f>IF(M35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P35" s="43" t="str">
+        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK(K35,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q35" s="47" t="str">
+        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R35" s="52"/>
     </x:row>
     <x:row r="36" ht="31">
       <x:c r="A36" s="2" t="s">
@@ -3363,17 +3534,20 @@
       <x:c r="L36" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M36" s="36"/>
-      <x:c r="N36" s="37" t="str">
+      <x:c r="M36" s="42"/>
+      <x:c r="N36" s="43" t="str">
         <x:f>IF(M36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
       </x:c>
-      <x:c r="O36" s="37" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K36&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P36" s="37" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N36,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O36,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q36" s="38"/>
+      <x:c r="O36" s="43" t="str">
+        <x:f>IF(M36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P36" s="43" t="str">
+        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK(K36,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q36" s="47" t="str">
+        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R36" s="52"/>
     </x:row>
     <x:row r="37" ht="31">
       <x:c r="A37" s="2" t="s">
@@ -3412,17 +3586,20 @@
       <x:c r="L37" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M37" s="36"/>
-      <x:c r="N37" s="37" t="str">
+      <x:c r="M37" s="42"/>
+      <x:c r="N37" s="43" t="str">
         <x:f>IF(M37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
       </x:c>
-      <x:c r="O37" s="37" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K37&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P37" s="37" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N37,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O37,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q37" s="38"/>
+      <x:c r="O37" s="43" t="str">
+        <x:f>IF(M37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P37" s="43" t="str">
+        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK(K37,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q37" s="47" t="str">
+        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R37" s="52"/>
     </x:row>
     <x:row r="38" ht="31">
       <x:c r="A38" s="2" t="s">
@@ -3461,17 +3638,20 @@
       <x:c r="L38" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M38" s="36"/>
-      <x:c r="N38" s="37" t="str">
+      <x:c r="M38" s="42"/>
+      <x:c r="N38" s="43" t="str">
         <x:f>IF(M38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
       </x:c>
-      <x:c r="O38" s="37" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K38&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P38" s="37" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N38,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O38,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q38" s="38"/>
+      <x:c r="O38" s="43" t="str">
+        <x:f>IF(M38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P38" s="43" t="str">
+        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK(K38,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q38" s="47" t="str">
+        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R38" s="52"/>
     </x:row>
     <x:row r="39" ht="31">
       <x:c r="A39" s="2" t="s">
@@ -3510,17 +3690,20 @@
       <x:c r="L39" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M39" s="36"/>
-      <x:c r="N39" s="37" t="str">
+      <x:c r="M39" s="42"/>
+      <x:c r="N39" s="43" t="str">
         <x:f>IF(M39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
       </x:c>
-      <x:c r="O39" s="37" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K39&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P39" s="37" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N39,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O39,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q39" s="38"/>
+      <x:c r="O39" s="43" t="str">
+        <x:f>IF(M39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P39" s="43" t="str">
+        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK(K39,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q39" s="47" t="str">
+        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R39" s="52"/>
     </x:row>
     <x:row r="40" ht="31">
       <x:c r="A40" s="2" t="s">
@@ -3559,17 +3742,20 @@
       <x:c r="L40" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M40" s="36"/>
-      <x:c r="N40" s="37" t="str">
+      <x:c r="M40" s="42"/>
+      <x:c r="N40" s="43" t="str">
         <x:f>IF(M40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
       </x:c>
-      <x:c r="O40" s="37" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K40&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P40" s="37" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N40,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O40,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q40" s="38"/>
+      <x:c r="O40" s="43" t="str">
+        <x:f>IF(M40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P40" s="43" t="str">
+        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK(K40,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q40" s="47" t="str">
+        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R40" s="52"/>
     </x:row>
     <x:row r="41" ht="45">
       <x:c r="A41" s="2" t="s">
@@ -3608,17 +3794,20 @@
       <x:c r="L41" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M41" s="36"/>
-      <x:c r="N41" s="37" t="str">
+      <x:c r="M41" s="42"/>
+      <x:c r="N41" s="43" t="str">
         <x:f>IF(M41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
       </x:c>
-      <x:c r="O41" s="37" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K41&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P41" s="37" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N41,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O41,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q41" s="38"/>
+      <x:c r="O41" s="43" t="str">
+        <x:f>IF(M41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P41" s="43" t="str">
+        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK(K41,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q41" s="47" t="str">
+        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R41" s="52"/>
     </x:row>
     <x:row r="42" ht="45">
       <x:c r="A42" s="2" t="s">
@@ -3657,17 +3846,20 @@
       <x:c r="L42" s="2" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="M42" s="36"/>
-      <x:c r="N42" s="37" t="str">
+      <x:c r="M42" s="42"/>
+      <x:c r="N42" s="43" t="str">
         <x:f>IF(M42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
       </x:c>
-      <x:c r="O42" s="37" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;K42&amp;CHAR(10)&amp;CHAR(10)&amp;"Browse all current opportunities:"&amp;CHAR(10)&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P42" s="37" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK("mailto:daniela.castrocamilo@glasgow.ac.uk?subject="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(N42,"%","%25"),"&amp;","%26"),"#","%23")," ","%20")&amp;"&amp;body="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(O42,"%","%25"),"&amp;","%26"),"#","%23"),CHAR(10),"%0A")," ","%20"),"Open email draft"))</x:f>
-      </x:c>
-      <x:c r="Q42" s="38"/>
+      <x:c r="O42" s="43" t="str">
+        <x:f>IF(M42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="P42" s="43" t="str">
+        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK(K42,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="Q42" s="47" t="str">
+        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="R42" s="52"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
@@ -3688,7 +3880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27120be6cc1d44c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc72960c867a644e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3852,15 +4044,15 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
-      <x:c r="A21" s="40" t="str">
+      <x:c r="A21" s="58" t="str">
         <x:v>Email draft workflow</x:v>
       </x:c>
-      <x:c r="B21" s="40" t="str">
-        <x:v>Use the final five columns of the Funding opportunities table to prepare an Outlook email without sending it automatically.</x:v>
+      <x:c r="B21" s="58" t="str">
+        <x:v>Use the final six columns of the Funding opportunities table to prepare an Outlook email without sending it automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="41" t="str">
+      <x:c r="A22" s="59" t="str">
         <x:v>Step 1</x:v>
       </x:c>
       <x:c r="B22" s="28" t="str">
@@ -3868,7 +4060,7 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="41" t="str">
+      <x:c r="A23" s="59" t="str">
         <x:v>Step 2</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
@@ -3876,19 +4068,19 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="41" t="str">
+      <x:c r="A24" s="59" t="str">
         <x:v>Step 3</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
-        <x:v>Click Open email draft. Outlook will open a pre-addressed message for daniela.castrocamilo@glasgow.ac.uk.</x:v>
+        <x:v>Copy the subject and body into Outlook, then copy the two hyperlink cells using Keep Source Formatting.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="41" t="str">
+      <x:c r="A25" s="59" t="str">
         <x:v>Step 4</x:v>
       </x:c>
       <x:c r="B25" s="28" t="str">
-        <x:v>Review the message, send it manually, then enter the date in Notification date.</x:v>
+        <x:v>Review and send the message manually, then enter the date in Notification date.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Automatically mark passed funding deadlines
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R524526c8ae454713"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Radc8776f72584b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="Rcb104da50cfe4301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Ref6975e7535a448a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,9 +47,6 @@
     <x:t xml:space="preserve">Source list</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">OPEN</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">LMS</x:t>
   </x:si>
   <x:si>
@@ -764,9 +761,6 @@
     <x:t xml:space="preserve">https://www.ukri.org/opportunity/?keywords=postdoctoral+fellowships</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">FORTHCOMING</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Sep/Oct 2026</x:t>
   </x:si>
   <x:si>
@@ -953,9 +947,6 @@
     <x:t xml:space="preserve">Important plan-ahead opportunity; likely internal selection at UofG—confirm when launched.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">CLOSED – monitor recurrence</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">University of Glasgow</x:t>
   </x:si>
   <x:si>
@@ -983,9 +974,6 @@
     <x:t xml:space="preserve">https://www.gla.ac.uk/myglasgow/ris/ieed/innovation/innovationfunds/medtechinnovationfund/</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">CLOSED – invited stage continues</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">SWIFT / EPSRC</x:t>
   </x:si>
   <x:si>
@@ -1035,9 +1023,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Status definitions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OPEN = live and accepting applications; FORTHCOMING = announced by funder but final call may not yet be live; CLOSED – monitor recurrence = useful recurring/strategic call retained for planning.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Suggested SharePoint filters</x:t>
@@ -1137,7 +1122,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1234,6 +1219,21 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -1241,7 +1241,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="80">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1390,11 +1390,61 @@
     <x:xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="4">
     <x:dxf>
       <x:font>
         <x:color rgb="FF666666"/>
@@ -1427,14 +1477,25 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF990000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:R42"/>
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:S42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:S42"/>
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Deadline"/>
     <x:tableColumn id="3" name="Funder"/>
@@ -1447,12 +1508,13 @@
     <x:tableColumn id="10" name="Internal action / note"/>
     <x:tableColumn id="11" name="Source"/>
     <x:tableColumn id="12" name="Source list"/>
-    <x:tableColumn id="13" name="Notify?"/>
-    <x:tableColumn id="14" name="Email subject"/>
-    <x:tableColumn id="15" name="Email body"/>
-    <x:tableColumn id="16" name="Official opportunity link"/>
-    <x:tableColumn id="17" name="Funding Finder link"/>
-    <x:tableColumn id="18" name="Notification date"/>
+    <x:tableColumn id="13" name="Status setting"/>
+    <x:tableColumn id="14" name="Notify?"/>
+    <x:tableColumn id="15" name="Email subject"/>
+    <x:tableColumn id="16" name="Email body"/>
+    <x:tableColumn id="17" name="Official opportunity link"/>
+    <x:tableColumn id="18" name="Funding Finder link"/>
+    <x:tableColumn id="19" name="Notification date"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1665,12 +1727,13 @@
     <x:col min="10" max="10" width="42" customWidth="1"/>
     <x:col min="11" max="11" width="50" customWidth="1"/>
     <x:col min="12" max="12" width="18" customWidth="1"/>
-    <x:col min="13" max="13" width="11" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="32" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="27" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="11" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="32" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="48" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="45.25" customHeight="1">
@@ -1710,2156 +1773,2323 @@
       <x:c r="L1" s="1" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="53" t="str">
+      <x:c r="M1" s="75" t="str">
+        <x:v>Status setting</x:v>
+      </x:c>
+      <x:c r="N1" s="75" t="str">
         <x:v>Notify?</x:v>
       </x:c>
-      <x:c r="N1" s="53" t="str">
+      <x:c r="O1" s="75" t="str">
         <x:v>Email subject</x:v>
       </x:c>
-      <x:c r="O1" s="53" t="str">
+      <x:c r="P1" s="75" t="str">
         <x:v>Email body</x:v>
       </x:c>
-      <x:c r="P1" s="53" t="str">
+      <x:c r="Q1" s="75" t="str">
         <x:v>Official opportunity link</x:v>
       </x:c>
-      <x:c r="Q1" s="53" t="str">
+      <x:c r="R1" s="75" t="str">
         <x:v>Funding Finder link</x:v>
       </x:c>
-      <x:c r="R1" s="53" t="str">
+      <x:c r="S1" s="75" t="str">
         <x:v>Notification date</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="31">
-      <x:c r="A2" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A2" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",M2)</x:f>
+        <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B2" s="3">
         <x:v>46295</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="s">
+      <x:c r="E2" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="s">
+      <x:c r="F2" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="s">
+      <x:c r="G2" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G2" s="2" t="s">
+      <x:c r="H2" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H2" s="2" t="s">
+      <x:c r="I2" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I2" s="2" t="s">
+      <x:c r="J2" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J2" s="2" t="s">
+      <x:c r="K2" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K2" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="L2" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M2" s="42"/>
-      <x:c r="N2" s="43" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
-      </x:c>
-      <x:c r="O2" s="43" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P2" s="43" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK(K2,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q2" s="47" t="str">
-        <x:f>IF(M2&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R2" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M2" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N2" s="64"/>
+      <x:c r="O2" s="65" t="str">
+        <x:f>IF(N2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
+      </x:c>
+      <x:c r="P2" s="65" t="str">
+        <x:f>IF(N2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q2" s="66" t="str">
+        <x:f>IF(N2&lt;&gt;"Yes","",HYPERLINK(K2,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R2" s="66" t="str">
+        <x:f>IF(N2&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S2" s="74"/>
     </x:row>
     <x:row r="3" ht="31">
-      <x:c r="A3" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A3" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B3),B3&lt;TODAY()),"DEADLINE PASSED",M3)</x:f>
+        <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>46295</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
+      <x:c r="E3" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="E3" s="2" t="s">
+      <x:c r="F3" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="F3" s="2" t="s">
+      <x:c r="G3" s="2" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="G3" s="2" t="s">
+      <x:c r="H3" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="H3" s="2" t="s">
+      <x:c r="I3" s="2" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="I3" s="2" t="s">
+      <x:c r="J3" s="2" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="J3" s="2" t="s">
+      <x:c r="K3" s="2" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="K3" s="2" t="s">
-        <x:v>30</x:v>
-      </x:c>
       <x:c r="L3" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="M3" s="42"/>
-      <x:c r="N3" s="43" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
-      </x:c>
-      <x:c r="O3" s="43" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P3" s="43" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK(K3,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q3" s="47" t="str">
-        <x:f>IF(M3&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R3" s="52"/>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M3" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N3" s="64"/>
+      <x:c r="O3" s="65" t="str">
+        <x:f>IF(N3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
+      </x:c>
+      <x:c r="P3" s="65" t="str">
+        <x:f>IF(N3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q3" s="66" t="str">
+        <x:f>IF(N3&lt;&gt;"Yes","",HYPERLINK(K3,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R3" s="66" t="str">
+        <x:f>IF(N3&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S3" s="74"/>
     </x:row>
     <x:row r="4" ht="31">
-      <x:c r="A4" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A4" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B4),B4&lt;TODAY()),"DEADLINE PASSED",M4)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B4" s="3">
         <x:v>46296</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="E4" s="2" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="F4" s="2" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="F4" s="2" t="s">
+      <x:c r="G4" s="2" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G4" s="2" t="s">
+      <x:c r="H4" s="2" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="H4" s="2" t="s">
+      <x:c r="I4" s="2" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="I4" s="2" t="s">
+      <x:c r="J4" s="2" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="J4" s="2" t="s">
+      <x:c r="K4" s="2" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="K4" s="2" t="s">
-        <x:v>39</x:v>
-      </x:c>
       <x:c r="L4" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M4" s="42"/>
-      <x:c r="N4" s="43" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
-      </x:c>
-      <x:c r="O4" s="43" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P4" s="43" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK(K4,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q4" s="47" t="str">
-        <x:f>IF(M4&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R4" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M4" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N4" s="64"/>
+      <x:c r="O4" s="65" t="str">
+        <x:f>IF(N4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
+      </x:c>
+      <x:c r="P4" s="65" t="str">
+        <x:f>IF(N4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q4" s="66" t="str">
+        <x:f>IF(N4&lt;&gt;"Yes","",HYPERLINK(K4,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R4" s="66" t="str">
+        <x:f>IF(N4&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S4" s="74"/>
     </x:row>
     <x:row r="5" ht="46">
-      <x:c r="A5" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A5" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B5),B5&lt;TODAY()),"DEADLINE PASSED",M5)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B5" s="3">
         <x:v>46304</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="2" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E5" s="2" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F5" s="2" t="s">
+      <x:c r="G5" s="2" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="G5" s="2" t="s">
+      <x:c r="H5" s="2" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="H5" s="2" t="s">
+      <x:c r="I5" s="2" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="I5" s="2" t="s">
+      <x:c r="J5" s="2" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="J5" s="2" t="s">
+      <x:c r="K5" s="2" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="K5" s="2" t="s">
-        <x:v>46</x:v>
-      </x:c>
       <x:c r="L5" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="M5" s="42"/>
-      <x:c r="N5" s="43" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
-      </x:c>
-      <x:c r="O5" s="43" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P5" s="43" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK(K5,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q5" s="47" t="str">
-        <x:f>IF(M5&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R5" s="52"/>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M5" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N5" s="64"/>
+      <x:c r="O5" s="65" t="str">
+        <x:f>IF(N5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
+      </x:c>
+      <x:c r="P5" s="65" t="str">
+        <x:f>IF(N5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q5" s="66" t="str">
+        <x:f>IF(N5&lt;&gt;"Yes","",HYPERLINK(K5,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R5" s="66" t="str">
+        <x:f>IF(N5&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S5" s="74"/>
     </x:row>
     <x:row r="6" ht="31">
-      <x:c r="A6" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A6" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B6),B6&lt;TODAY()),"DEADLINE PASSED",M6)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B6" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C6" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D6" s="2" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="E6" s="2" t="s">
+      <x:c r="F6" s="2" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="F6" s="2" t="s">
+      <x:c r="G6" s="2" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="G6" s="2" t="s">
+      <x:c r="H6" s="2" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="H6" s="2" t="s">
+      <x:c r="I6" s="2" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="I6" s="2" t="s">
+      <x:c r="J6" s="2" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="J6" s="2" t="s">
-        <x:v>53</x:v>
-      </x:c>
       <x:c r="K6" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L6" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M6" s="42"/>
-      <x:c r="N6" s="43" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
-      </x:c>
-      <x:c r="O6" s="43" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P6" s="43" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK(K6,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q6" s="47" t="str">
-        <x:f>IF(M6&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R6" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M6" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N6" s="64"/>
+      <x:c r="O6" s="65" t="str">
+        <x:f>IF(N6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
+      </x:c>
+      <x:c r="P6" s="65" t="str">
+        <x:f>IF(N6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q6" s="66" t="str">
+        <x:f>IF(N6&lt;&gt;"Yes","",HYPERLINK(K6,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R6" s="66" t="str">
+        <x:f>IF(N6&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S6" s="74"/>
     </x:row>
     <x:row r="7" ht="31">
-      <x:c r="A7" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A7" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B7),B7&lt;TODAY()),"DEADLINE PASSED",M7)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B7" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D7" s="2" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="E7" s="2" t="s">
+      <x:c r="F7" s="2" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="F7" s="2" t="s">
+      <x:c r="G7" s="2" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="G7" s="2" t="s">
+      <x:c r="H7" s="2" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="H7" s="2" t="s">
+      <x:c r="I7" s="2" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="I7" s="2" t="s">
-        <x:v>59</x:v>
-      </x:c>
       <x:c r="J7" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="K7" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L7" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M7" s="42"/>
-      <x:c r="N7" s="43" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
-      </x:c>
-      <x:c r="O7" s="43" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P7" s="43" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK(K7,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q7" s="47" t="str">
-        <x:f>IF(M7&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R7" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M7" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N7" s="64"/>
+      <x:c r="O7" s="65" t="str">
+        <x:f>IF(N7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
+      </x:c>
+      <x:c r="P7" s="65" t="str">
+        <x:f>IF(N7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q7" s="66" t="str">
+        <x:f>IF(N7&lt;&gt;"Yes","",HYPERLINK(K7,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R7" s="66" t="str">
+        <x:f>IF(N7&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S7" s="74"/>
     </x:row>
     <x:row r="8" ht="46">
-      <x:c r="A8" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A8" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B8),B8&lt;TODAY()),"DEADLINE PASSED",M8)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B8" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D8" s="2" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E8" s="2" t="s">
+      <x:c r="F8" s="2" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="F8" s="2" t="s">
+      <x:c r="G8" s="2" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="G8" s="2" t="s">
+      <x:c r="H8" s="2" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="H8" s="2" t="s">
+      <x:c r="I8" s="2" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="I8" s="2" t="s">
+      <x:c r="J8" s="2" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="J8" s="2" t="s">
+      <x:c r="K8" s="2" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="K8" s="2" t="s">
-        <x:v>67</x:v>
-      </x:c>
       <x:c r="L8" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M8" s="42"/>
-      <x:c r="N8" s="43" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
-      </x:c>
-      <x:c r="O8" s="43" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P8" s="43" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK(K8,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q8" s="47" t="str">
-        <x:f>IF(M8&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R8" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M8" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N8" s="64"/>
+      <x:c r="O8" s="65" t="str">
+        <x:f>IF(N8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
+      </x:c>
+      <x:c r="P8" s="65" t="str">
+        <x:f>IF(N8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q8" s="66" t="str">
+        <x:f>IF(N8&lt;&gt;"Yes","",HYPERLINK(K8,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R8" s="66" t="str">
+        <x:f>IF(N8&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S8" s="74"/>
     </x:row>
     <x:row r="9" ht="31">
-      <x:c r="A9" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A9" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B9),B9&lt;TODAY()),"DEADLINE PASSED",M9)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B9" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="D9" s="2" t="s">
+      <x:c r="E9" s="2" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="E9" s="2" t="s">
+      <x:c r="F9" s="2" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F9" s="2" t="s">
+      <x:c r="G9" s="2" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="G9" s="2" t="s">
+      <x:c r="H9" s="2" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="H9" s="2" t="s">
+      <x:c r="I9" s="2" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="I9" s="2" t="s">
+      <x:c r="J9" s="2" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="J9" s="2" t="s">
+      <x:c r="K9" s="2" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="K9" s="2" t="s">
-        <x:v>76</x:v>
-      </x:c>
       <x:c r="L9" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M9" s="42"/>
-      <x:c r="N9" s="43" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
-      </x:c>
-      <x:c r="O9" s="43" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P9" s="43" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK(K9,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q9" s="47" t="str">
-        <x:f>IF(M9&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R9" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M9" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N9" s="64"/>
+      <x:c r="O9" s="65" t="str">
+        <x:f>IF(N9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
+      </x:c>
+      <x:c r="P9" s="65" t="str">
+        <x:f>IF(N9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q9" s="66" t="str">
+        <x:f>IF(N9&lt;&gt;"Yes","",HYPERLINK(K9,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R9" s="66" t="str">
+        <x:f>IF(N9&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S9" s="74"/>
     </x:row>
     <x:row r="10" ht="31">
-      <x:c r="A10" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A10" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B10),B10&lt;TODAY()),"DEADLINE PASSED",M10)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B10" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D10" s="2" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="E10" s="2" t="s">
+      <x:c r="F10" s="2" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F10" s="2" t="s">
+      <x:c r="G10" s="2" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="G10" s="2" t="s">
+      <x:c r="H10" s="2" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="H10" s="2" t="s">
+      <x:c r="I10" s="2" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="I10" s="2" t="s">
+      <x:c r="J10" s="2" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="J10" s="2" t="s">
+      <x:c r="K10" s="2" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="K10" s="2" t="s">
-        <x:v>84</x:v>
-      </x:c>
       <x:c r="L10" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M10" s="42"/>
-      <x:c r="N10" s="43" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
-      </x:c>
-      <x:c r="O10" s="43" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P10" s="43" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK(K10,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q10" s="47" t="str">
-        <x:f>IF(M10&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R10" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M10" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N10" s="64"/>
+      <x:c r="O10" s="65" t="str">
+        <x:f>IF(N10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
+      </x:c>
+      <x:c r="P10" s="65" t="str">
+        <x:f>IF(N10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q10" s="66" t="str">
+        <x:f>IF(N10&lt;&gt;"Yes","",HYPERLINK(K10,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R10" s="66" t="str">
+        <x:f>IF(N10&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S10" s="74"/>
     </x:row>
     <x:row r="11" ht="31">
-      <x:c r="A11" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A11" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B11),B11&lt;TODAY()),"DEADLINE PASSED",M11)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B11" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D11" s="2" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="E11" s="2" t="s">
+      <x:c r="F11" s="2" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="F11" s="2" t="s">
+      <x:c r="G11" s="2" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="G11" s="2" t="s">
+      <x:c r="H11" s="2" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="H11" s="2" t="s">
+      <x:c r="I11" s="2" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="I11" s="2" t="s">
+      <x:c r="J11" s="2" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="J11" s="2" t="s">
+      <x:c r="K11" s="2" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="K11" s="2" t="s">
-        <x:v>92</x:v>
-      </x:c>
       <x:c r="L11" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M11" s="42"/>
-      <x:c r="N11" s="43" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
-      </x:c>
-      <x:c r="O11" s="43" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P11" s="43" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK(K11,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q11" s="47" t="str">
-        <x:f>IF(M11&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R11" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M11" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N11" s="64"/>
+      <x:c r="O11" s="65" t="str">
+        <x:f>IF(N11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
+      </x:c>
+      <x:c r="P11" s="65" t="str">
+        <x:f>IF(N11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q11" s="66" t="str">
+        <x:f>IF(N11&lt;&gt;"Yes","",HYPERLINK(K11,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R11" s="66" t="str">
+        <x:f>IF(N11&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S11" s="74"/>
     </x:row>
     <x:row r="12" ht="31">
-      <x:c r="A12" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A12" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B12),B12&lt;TODAY()),"DEADLINE PASSED",M12)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B12" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C12" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D12" s="2" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="E12" s="2" t="s">
+      <x:c r="F12" s="2" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="s">
+      <x:c r="G12" s="2" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="G12" s="2" t="s">
+      <x:c r="H12" s="2" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="H12" s="2" t="s">
+      <x:c r="I12" s="2" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="I12" s="2" t="s">
+      <x:c r="J12" s="2" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="J12" s="2" t="s">
+      <x:c r="K12" s="2" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="K12" s="2" t="s">
-        <x:v>100</x:v>
-      </x:c>
       <x:c r="L12" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M12" s="42"/>
-      <x:c r="N12" s="43" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
-      </x:c>
-      <x:c r="O12" s="43" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P12" s="43" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK(K12,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q12" s="47" t="str">
-        <x:f>IF(M12&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R12" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M12" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N12" s="64"/>
+      <x:c r="O12" s="65" t="str">
+        <x:f>IF(N12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
+      </x:c>
+      <x:c r="P12" s="65" t="str">
+        <x:f>IF(N12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q12" s="66" t="str">
+        <x:f>IF(N12&lt;&gt;"Yes","",HYPERLINK(K12,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R12" s="66" t="str">
+        <x:f>IF(N12&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S12" s="74"/>
     </x:row>
     <x:row r="13" ht="31">
-      <x:c r="A13" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A13" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B13),B13&lt;TODAY()),"DEADLINE PASSED",M13)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B13" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C13" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D13" s="2" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="E13" s="2" t="s">
+      <x:c r="F13" s="2" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="F13" s="2" t="s">
+      <x:c r="G13" s="2" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="G13" s="2" t="s">
+      <x:c r="H13" s="2" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="H13" s="2" t="s">
+      <x:c r="I13" s="2" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="I13" s="2" t="s">
+      <x:c r="J13" s="2" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="J13" s="2" t="s">
+      <x:c r="K13" s="2" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="K13" s="2" t="s">
-        <x:v>108</x:v>
-      </x:c>
       <x:c r="L13" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M13" s="42"/>
-      <x:c r="N13" s="43" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
-      </x:c>
-      <x:c r="O13" s="43" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P13" s="43" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK(K13,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q13" s="47" t="str">
-        <x:f>IF(M13&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R13" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M13" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N13" s="64"/>
+      <x:c r="O13" s="65" t="str">
+        <x:f>IF(N13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
+      </x:c>
+      <x:c r="P13" s="65" t="str">
+        <x:f>IF(N13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q13" s="66" t="str">
+        <x:f>IF(N13&lt;&gt;"Yes","",HYPERLINK(K13,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R13" s="66" t="str">
+        <x:f>IF(N13&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S13" s="74"/>
     </x:row>
     <x:row r="14" ht="46">
-      <x:c r="A14" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A14" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B14),B14&lt;TODAY()),"DEADLINE PASSED",M14)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B14" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C14" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D14" s="2" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="E14" s="2" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="F14" s="2" t="s">
+      <x:c r="G14" s="2" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="G14" s="2" t="s">
+      <x:c r="H14" s="2" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="H14" s="2" t="s">
+      <x:c r="I14" s="2" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="I14" s="2" t="s">
+      <x:c r="J14" s="2" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="J14" s="2" t="s">
+      <x:c r="K14" s="2" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="K14" s="2" t="s">
-        <x:v>115</x:v>
-      </x:c>
       <x:c r="L14" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M14" s="42"/>
-      <x:c r="N14" s="43" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
-      </x:c>
-      <x:c r="O14" s="43" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P14" s="43" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK(K14,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q14" s="47" t="str">
-        <x:f>IF(M14&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R14" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M14" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N14" s="64"/>
+      <x:c r="O14" s="65" t="str">
+        <x:f>IF(N14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
+      </x:c>
+      <x:c r="P14" s="65" t="str">
+        <x:f>IF(N14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q14" s="66" t="str">
+        <x:f>IF(N14&lt;&gt;"Yes","",HYPERLINK(K14,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R14" s="66" t="str">
+        <x:f>IF(N14&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S14" s="74"/>
     </x:row>
     <x:row r="15" ht="46">
-      <x:c r="A15" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A15" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B15),B15&lt;TODAY()),"DEADLINE PASSED",M15)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B15" s="3">
         <x:v>46323</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="D15" s="2" t="s">
+      <x:c r="E15" s="2" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="E15" s="2" t="s">
+      <x:c r="F15" s="2" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="F15" s="2" t="s">
+      <x:c r="G15" s="2" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="G15" s="2" t="s">
+      <x:c r="H15" s="2" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="H15" s="2" t="s">
+      <x:c r="I15" s="2" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="I15" s="2" t="s">
+      <x:c r="J15" s="2" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="J15" s="2" t="s">
+      <x:c r="K15" s="2" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="K15" s="2" t="s">
+      <x:c r="L15" s="2" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="L15" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M15" s="42"/>
-      <x:c r="N15" s="43" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
-      </x:c>
-      <x:c r="O15" s="43" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P15" s="43" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK(K15,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q15" s="47" t="str">
-        <x:f>IF(M15&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R15" s="52"/>
+      <x:c r="M15" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N15" s="64"/>
+      <x:c r="O15" s="65" t="str">
+        <x:f>IF(N15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
+      </x:c>
+      <x:c r="P15" s="65" t="str">
+        <x:f>IF(N15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q15" s="66" t="str">
+        <x:f>IF(N15&lt;&gt;"Yes","",HYPERLINK(K15,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R15" s="66" t="str">
+        <x:f>IF(N15&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S15" s="74"/>
     </x:row>
     <x:row r="16" ht="31">
-      <x:c r="A16" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A16" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B16),B16&lt;TODAY()),"DEADLINE PASSED",M16)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B16" s="3">
         <x:v>46328</x:v>
       </x:c>
       <x:c r="C16" s="2" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="D16" s="2" t="s">
+      <x:c r="E16" s="2" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="E16" s="2" t="s">
+      <x:c r="F16" s="2" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F16" s="2" t="s">
+      <x:c r="G16" s="2" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="G16" s="2" t="s">
+      <x:c r="H16" s="2" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="H16" s="2" t="s">
+      <x:c r="I16" s="2" t="s">
         <x:v>131</x:v>
       </x:c>
-      <x:c r="I16" s="2" t="s">
+      <x:c r="J16" s="2" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="J16" s="2" t="s">
+      <x:c r="K16" s="2" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="K16" s="2" t="s">
-        <x:v>134</x:v>
-      </x:c>
       <x:c r="L16" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M16" s="42"/>
-      <x:c r="N16" s="43" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
-      </x:c>
-      <x:c r="O16" s="43" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P16" s="43" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK(K16,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q16" s="47" t="str">
-        <x:f>IF(M16&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R16" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M16" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N16" s="64"/>
+      <x:c r="O16" s="65" t="str">
+        <x:f>IF(N16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
+      </x:c>
+      <x:c r="P16" s="65" t="str">
+        <x:f>IF(N16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q16" s="66" t="str">
+        <x:f>IF(N16&lt;&gt;"Yes","",HYPERLINK(K16,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R16" s="66" t="str">
+        <x:f>IF(N16&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S16" s="74"/>
     </x:row>
     <x:row r="17" ht="31">
-      <x:c r="A17" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A17" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B17),B17&lt;TODAY()),"DEADLINE PASSED",M17)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B17" s="3">
         <x:v>46336</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="D17" s="2" t="s">
+      <x:c r="E17" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="F17" s="2" t="s">
+      <x:c r="G17" s="2" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="G17" s="2" t="s">
+      <x:c r="H17" s="2" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="H17" s="2" t="s">
+      <x:c r="I17" s="2" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="I17" s="2" t="s">
+      <x:c r="J17" s="2" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="J17" s="2" t="s">
+      <x:c r="K17" s="2" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="K17" s="2" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="L17" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M17" s="42"/>
-      <x:c r="N17" s="43" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
-      </x:c>
-      <x:c r="O17" s="43" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P17" s="43" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK(K17,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q17" s="47" t="str">
-        <x:f>IF(M17&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R17" s="52"/>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M17" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N17" s="64"/>
+      <x:c r="O17" s="65" t="str">
+        <x:f>IF(N17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
+      </x:c>
+      <x:c r="P17" s="65" t="str">
+        <x:f>IF(N17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q17" s="66" t="str">
+        <x:f>IF(N17&lt;&gt;"Yes","",HYPERLINK(K17,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R17" s="66" t="str">
+        <x:f>IF(N17&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S17" s="74"/>
     </x:row>
     <x:row r="18" ht="46">
-      <x:c r="A18" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A18" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B18),B18&lt;TODAY()),"DEADLINE PASSED",M18)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B18" s="3">
         <x:v>46338</x:v>
       </x:c>
       <x:c r="C18" s="2" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="D18" s="2" t="s">
+      <x:c r="E18" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="E18" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="F18" s="2" t="s">
+      <x:c r="G18" s="2" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="G18" s="2" t="s">
+      <x:c r="H18" s="2" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="H18" s="2" t="s">
+      <x:c r="I18" s="2" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="I18" s="2" t="s">
+      <x:c r="J18" s="2" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="J18" s="2" t="s">
+      <x:c r="K18" s="2" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="K18" s="2" t="s">
-        <x:v>150</x:v>
-      </x:c>
       <x:c r="L18" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M18" s="42"/>
-      <x:c r="N18" s="43" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
-      </x:c>
-      <x:c r="O18" s="43" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P18" s="43" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK(K18,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q18" s="47" t="str">
-        <x:f>IF(M18&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R18" s="52"/>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M18" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N18" s="64"/>
+      <x:c r="O18" s="65" t="str">
+        <x:f>IF(N18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
+      </x:c>
+      <x:c r="P18" s="65" t="str">
+        <x:f>IF(N18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q18" s="66" t="str">
+        <x:f>IF(N18&lt;&gt;"Yes","",HYPERLINK(K18,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R18" s="66" t="str">
+        <x:f>IF(N18&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S18" s="74"/>
     </x:row>
     <x:row r="19" ht="31">
-      <x:c r="A19" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A19" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B19),B19&lt;TODAY()),"DEADLINE PASSED",M19)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B19" s="3">
         <x:v>46356</x:v>
       </x:c>
       <x:c r="C19" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D19" s="2" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="E19" s="2" t="s">
+      <x:c r="F19" s="2" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="F19" s="2" t="s">
+      <x:c r="G19" s="2" t="s">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="G19" s="2" t="s">
+      <x:c r="H19" s="2" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="H19" s="2" t="s">
+      <x:c r="I19" s="2" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="I19" s="2" t="s">
+      <x:c r="J19" s="2" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="J19" s="2" t="s">
+      <x:c r="K19" s="2" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="K19" s="2" t="s">
-        <x:v>158</x:v>
-      </x:c>
       <x:c r="L19" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M19" s="42"/>
-      <x:c r="N19" s="43" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
-      </x:c>
-      <x:c r="O19" s="43" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P19" s="43" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK(K19,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q19" s="47" t="str">
-        <x:f>IF(M19&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R19" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M19" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N19" s="64"/>
+      <x:c r="O19" s="65" t="str">
+        <x:f>IF(N19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
+      </x:c>
+      <x:c r="P19" s="65" t="str">
+        <x:f>IF(N19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q19" s="66" t="str">
+        <x:f>IF(N19&lt;&gt;"Yes","",HYPERLINK(K19,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R19" s="66" t="str">
+        <x:f>IF(N19&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S19" s="74"/>
     </x:row>
     <x:row r="20" ht="46">
-      <x:c r="A20" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A20" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B20),B20&lt;TODAY()),"DEADLINE PASSED",M20)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B20" s="3">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C20" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D20" s="2" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="E20" s="2" t="s">
+      <x:c r="F20" s="2" t="s">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="F20" s="2" t="s">
+      <x:c r="G20" s="2" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="G20" s="2" t="s">
+      <x:c r="H20" s="2" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="H20" s="2" t="s">
+      <x:c r="I20" s="2" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="I20" s="2" t="s">
+      <x:c r="J20" s="2" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="J20" s="2" t="s">
+      <x:c r="K20" s="2" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="K20" s="2" t="s">
-        <x:v>166</x:v>
-      </x:c>
       <x:c r="L20" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M20" s="42"/>
-      <x:c r="N20" s="43" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
-      </x:c>
-      <x:c r="O20" s="43" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P20" s="43" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK(K20,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q20" s="47" t="str">
-        <x:f>IF(M20&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R20" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M20" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N20" s="64"/>
+      <x:c r="O20" s="65" t="str">
+        <x:f>IF(N20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
+      </x:c>
+      <x:c r="P20" s="65" t="str">
+        <x:f>IF(N20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q20" s="66" t="str">
+        <x:f>IF(N20&lt;&gt;"Yes","",HYPERLINK(K20,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R20" s="66" t="str">
+        <x:f>IF(N20&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S20" s="74"/>
     </x:row>
     <x:row r="21" ht="31">
-      <x:c r="A21" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A21" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B21),B21&lt;TODAY()),"DEADLINE PASSED",M21)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B21" s="3">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C21" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D21" s="2" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="E21" s="2" t="s">
+      <x:c r="F21" s="2" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F21" s="2" t="s">
+      <x:c r="G21" s="2" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="G21" s="2" t="s">
+      <x:c r="H21" s="2" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="H21" s="2" t="s">
+      <x:c r="I21" s="2" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="I21" s="2" t="s">
+      <x:c r="J21" s="2" t="s">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="J21" s="2" t="s">
-        <x:v>173</x:v>
-      </x:c>
       <x:c r="K21" s="2" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="L21" s="2" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="M21" s="42"/>
-      <x:c r="N21" s="43" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
-      </x:c>
-      <x:c r="O21" s="43" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P21" s="43" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK(K21,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q21" s="47" t="str">
-        <x:f>IF(M21&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R21" s="52"/>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M21" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N21" s="64"/>
+      <x:c r="O21" s="65" t="str">
+        <x:f>IF(N21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
+      </x:c>
+      <x:c r="P21" s="65" t="str">
+        <x:f>IF(N21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q21" s="66" t="str">
+        <x:f>IF(N21&lt;&gt;"Yes","",HYPERLINK(K21,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R21" s="66" t="str">
+        <x:f>IF(N21&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S21" s="74"/>
     </x:row>
     <x:row r="22" ht="31">
-      <x:c r="A22" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A22" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B22),B22&lt;TODAY()),"DEADLINE PASSED",M22)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B22" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C22" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D22" s="2" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="E22" s="2" t="s">
+      <x:c r="F22" s="2" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="F22" s="2" t="s">
+      <x:c r="G22" s="2" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="G22" s="2" t="s">
+      <x:c r="H22" s="2" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="H22" s="2" t="s">
+      <x:c r="I22" s="2" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="I22" s="2" t="s">
+      <x:c r="J22" s="2" t="s">
         <x:v>179</x:v>
       </x:c>
-      <x:c r="J22" s="2" t="s">
+      <x:c r="K22" s="2" t="s">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="K22" s="2" t="s">
-        <x:v>181</x:v>
-      </x:c>
       <x:c r="L22" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M22" s="42"/>
-      <x:c r="N22" s="43" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
-      </x:c>
-      <x:c r="O22" s="43" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P22" s="43" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK(K22,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q22" s="47" t="str">
-        <x:f>IF(M22&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R22" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M22" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N22" s="64"/>
+      <x:c r="O22" s="65" t="str">
+        <x:f>IF(N22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
+      </x:c>
+      <x:c r="P22" s="65" t="str">
+        <x:f>IF(N22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q22" s="66" t="str">
+        <x:f>IF(N22&lt;&gt;"Yes","",HYPERLINK(K22,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R22" s="66" t="str">
+        <x:f>IF(N22&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S22" s="74"/>
     </x:row>
     <x:row r="23" ht="31">
-      <x:c r="A23" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A23" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B23),B23&lt;TODAY()),"DEADLINE PASSED",M23)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B23" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C23" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D23" s="2" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="E23" s="2" t="s">
+      <x:c r="F23" s="2" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="F23" s="2" t="s">
+      <x:c r="G23" s="2" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="G23" s="2" t="s">
+      <x:c r="H23" s="2" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="H23" s="2" t="s">
+      <x:c r="I23" s="2" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="I23" s="2" t="s">
+      <x:c r="J23" s="2" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="K23" s="2" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="J23" s="2" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="K23" s="2" t="s">
-        <x:v>188</x:v>
-      </x:c>
       <x:c r="L23" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M23" s="42"/>
-      <x:c r="N23" s="43" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
-      </x:c>
-      <x:c r="O23" s="43" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P23" s="43" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK(K23,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q23" s="47" t="str">
-        <x:f>IF(M23&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R23" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M23" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N23" s="64"/>
+      <x:c r="O23" s="65" t="str">
+        <x:f>IF(N23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
+      </x:c>
+      <x:c r="P23" s="65" t="str">
+        <x:f>IF(N23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q23" s="66" t="str">
+        <x:f>IF(N23&lt;&gt;"Yes","",HYPERLINK(K23,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R23" s="66" t="str">
+        <x:f>IF(N23&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S23" s="74"/>
     </x:row>
     <x:row r="24" ht="31">
-      <x:c r="A24" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A24" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B24),B24&lt;TODAY()),"DEADLINE PASSED",M24)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B24" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C24" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D24" s="2" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="E24" s="2" t="s">
+      <x:c r="F24" s="2" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="F24" s="2" t="s">
+      <x:c r="G24" s="2" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="G24" s="2" t="s">
+      <x:c r="H24" s="2" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="H24" s="2" t="s">
+      <x:c r="I24" s="2" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J24" s="2" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="K24" s="2" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="I24" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="J24" s="2" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="K24" s="2" t="s">
-        <x:v>194</x:v>
-      </x:c>
       <x:c r="L24" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M24" s="42"/>
-      <x:c r="N24" s="43" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
-      </x:c>
-      <x:c r="O24" s="43" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P24" s="43" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK(K24,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q24" s="47" t="str">
-        <x:f>IF(M24&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R24" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M24" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N24" s="64"/>
+      <x:c r="O24" s="65" t="str">
+        <x:f>IF(N24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
+      </x:c>
+      <x:c r="P24" s="65" t="str">
+        <x:f>IF(N24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q24" s="66" t="str">
+        <x:f>IF(N24&lt;&gt;"Yes","",HYPERLINK(K24,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R24" s="66" t="str">
+        <x:f>IF(N24&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S24" s="74"/>
     </x:row>
     <x:row r="25" ht="31">
-      <x:c r="A25" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A25" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B25),B25&lt;TODAY()),"DEADLINE PASSED",M25)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B25" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C25" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D25" s="2" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="E25" s="2" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="F25" s="2" t="s">
+      <x:c r="G25" s="2" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="G25" s="2" t="s">
+      <x:c r="H25" s="2" t="s">
         <x:v>197</x:v>
       </x:c>
-      <x:c r="H25" s="2" t="s">
+      <x:c r="I25" s="2" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="I25" s="2" t="s">
-        <x:v>199</x:v>
-      </x:c>
       <x:c r="J25" s="2" t="s">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="K25" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L25" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M25" s="42"/>
-      <x:c r="N25" s="43" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
-      </x:c>
-      <x:c r="O25" s="43" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P25" s="43" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK(K25,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q25" s="47" t="str">
-        <x:f>IF(M25&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R25" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M25" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N25" s="64"/>
+      <x:c r="O25" s="65" t="str">
+        <x:f>IF(N25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
+      </x:c>
+      <x:c r="P25" s="65" t="str">
+        <x:f>IF(N25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q25" s="66" t="str">
+        <x:f>IF(N25&lt;&gt;"Yes","",HYPERLINK(K25,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R25" s="66" t="str">
+        <x:f>IF(N25&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S25" s="74"/>
     </x:row>
     <x:row r="26" ht="31">
-      <x:c r="A26" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A26" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B26),B26&lt;TODAY()),"DEADLINE PASSED",M26)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B26" s="3">
         <x:v>46418</x:v>
       </x:c>
       <x:c r="C26" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D26" s="2" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="E26" s="2" t="s">
+      <x:c r="F26" s="2" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="F26" s="2" t="s">
+      <x:c r="G26" s="2" t="s">
         <x:v>202</x:v>
       </x:c>
-      <x:c r="G26" s="2" t="s">
+      <x:c r="H26" s="2" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="H26" s="2" t="s">
+      <x:c r="I26" s="2" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="J26" s="2" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="I26" s="2" t="s">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="J26" s="2" t="s">
-        <x:v>205</x:v>
-      </x:c>
       <x:c r="K26" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L26" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M26" s="42"/>
-      <x:c r="N26" s="43" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
-      </x:c>
-      <x:c r="O26" s="43" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P26" s="43" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK(K26,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q26" s="47" t="str">
-        <x:f>IF(M26&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R26" s="52"/>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M26" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N26" s="64"/>
+      <x:c r="O26" s="65" t="str">
+        <x:f>IF(N26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
+      </x:c>
+      <x:c r="P26" s="65" t="str">
+        <x:f>IF(N26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q26" s="66" t="str">
+        <x:f>IF(N26&lt;&gt;"Yes","",HYPERLINK(K26,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R26" s="66" t="str">
+        <x:f>IF(N26&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S26" s="74"/>
     </x:row>
     <x:row r="27" ht="31">
-      <x:c r="A27" s="2" t="s">
-        <x:v>12</x:v>
+      <x:c r="A27" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B27),B27&lt;TODAY()),"DEADLINE PASSED",M27)</x:f>
+        <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B27" s="3">
         <x:v>46419</x:v>
       </x:c>
       <x:c r="C27" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D27" s="2" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="E27" s="2" t="s">
+      <x:c r="F27" s="2" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="F27" s="2" t="s">
+      <x:c r="G27" s="2" t="s">
         <x:v>208</x:v>
       </x:c>
-      <x:c r="G27" s="2" t="s">
+      <x:c r="H27" s="2" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="H27" s="2" t="s">
+      <x:c r="I27" s="2" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="I27" s="2" t="s">
+      <x:c r="J27" s="2" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="J27" s="2" t="s">
+      <x:c r="K27" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L27" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M27" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N27" s="64"/>
+      <x:c r="O27" s="65" t="str">
+        <x:f>IF(N27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
+      </x:c>
+      <x:c r="P27" s="65" t="str">
+        <x:f>IF(N27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q27" s="66" t="str">
+        <x:f>IF(N27&lt;&gt;"Yes","",HYPERLINK(K27,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R27" s="66" t="str">
+        <x:f>IF(N27&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S27" s="74"/>
+    </x:row>
+    <x:row r="28" ht="46">
+      <x:c r="A28" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B28),B28&lt;TODAY()),"DEADLINE PASSED",M28)</x:f>
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="B28" s="3" t="s">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="K27" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="L27" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="M27" s="42"/>
-      <x:c r="N27" s="43" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
-      </x:c>
-      <x:c r="O27" s="43" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P27" s="43" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK(K27,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q27" s="47" t="str">
-        <x:f>IF(M27&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R27" s="52"/>
-    </x:row>
-    <x:row r="28" ht="46">
-      <x:c r="A28" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B28" s="3" t="s">
+      <x:c r="C28" s="2" t="s">
         <x:v>213</x:v>
       </x:c>
-      <x:c r="C28" s="2" t="s">
+      <x:c r="D28" s="2" t="s">
         <x:v>214</x:v>
       </x:c>
-      <x:c r="D28" s="2" t="s">
+      <x:c r="E28" s="2" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="E28" s="2" t="s">
+      <x:c r="F28" s="2" t="s">
         <x:v>216</x:v>
       </x:c>
-      <x:c r="F28" s="2" t="s">
+      <x:c r="G28" s="2" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="G28" s="2" t="s">
+      <x:c r="H28" s="2" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="H28" s="2" t="s">
+      <x:c r="I28" s="2" t="s">
         <x:v>219</x:v>
       </x:c>
-      <x:c r="I28" s="2" t="s">
+      <x:c r="J28" s="2" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="J28" s="2" t="s">
+      <x:c r="K28" s="2" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="K28" s="2" t="s">
+      <x:c r="L28" s="2" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M28" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N28" s="64"/>
+      <x:c r="O28" s="65" t="str">
+        <x:f>IF(N28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
+      </x:c>
+      <x:c r="P28" s="65" t="str">
+        <x:f>IF(N28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q28" s="66" t="str">
+        <x:f>IF(N28&lt;&gt;"Yes","",HYPERLINK(K28,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R28" s="66" t="str">
+        <x:f>IF(N28&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S28" s="74"/>
+    </x:row>
+    <x:row r="29" ht="46">
+      <x:c r="A29" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B29),B29&lt;TODAY()),"DEADLINE PASSED",M29)</x:f>
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="B29" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="s">
         <x:v>222</x:v>
       </x:c>
-      <x:c r="L28" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M28" s="42"/>
-      <x:c r="N28" s="43" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
-      </x:c>
-      <x:c r="O28" s="43" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P28" s="43" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK(K28,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q28" s="47" t="str">
-        <x:f>IF(M28&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R28" s="52"/>
-    </x:row>
-    <x:row r="29" ht="46">
-      <x:c r="A29" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B29" s="3" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="C29" s="2" t="s">
+      <x:c r="D29" s="2" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="D29" s="2" t="s">
+      <x:c r="E29" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="E29" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="F29" s="2" t="s">
+      <x:c r="G29" s="2" t="s">
         <x:v>225</x:v>
       </x:c>
-      <x:c r="G29" s="2" t="s">
+      <x:c r="H29" s="2" t="s">
         <x:v>226</x:v>
       </x:c>
-      <x:c r="H29" s="2" t="s">
+      <x:c r="I29" s="2" t="s">
         <x:v>227</x:v>
       </x:c>
-      <x:c r="I29" s="2" t="s">
+      <x:c r="J29" s="2" t="s">
         <x:v>228</x:v>
       </x:c>
-      <x:c r="J29" s="2" t="s">
+      <x:c r="K29" s="2" t="s">
         <x:v>229</x:v>
       </x:c>
-      <x:c r="K29" s="2" t="s">
+      <x:c r="L29" s="2" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="L29" s="2" t="s">
+      <x:c r="M29" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N29" s="64"/>
+      <x:c r="O29" s="65" t="str">
+        <x:f>IF(N29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
+      </x:c>
+      <x:c r="P29" s="65" t="str">
+        <x:f>IF(N29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q29" s="66" t="str">
+        <x:f>IF(N29&lt;&gt;"Yes","",HYPERLINK(K29,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R29" s="66" t="str">
+        <x:f>IF(N29&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S29" s="74"/>
+    </x:row>
+    <x:row r="30" ht="31">
+      <x:c r="A30" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B30),B30&lt;TODAY()),"DEADLINE PASSED",M30)</x:f>
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="B30" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="M29" s="42"/>
-      <x:c r="N29" s="43" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
-      </x:c>
-      <x:c r="O29" s="43" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P29" s="43" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK(K29,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q29" s="47" t="str">
-        <x:f>IF(M29&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R29" s="52"/>
-    </x:row>
-    <x:row r="30" ht="31">
-      <x:c r="A30" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B30" s="3" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="D30" s="2" t="s">
+      <x:c r="E30" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="s">
         <x:v>232</x:v>
       </x:c>
-      <x:c r="E30" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="F30" s="2" t="s">
+      <x:c r="G30" s="2" t="s">
         <x:v>233</x:v>
       </x:c>
-      <x:c r="G30" s="2" t="s">
+      <x:c r="H30" s="2" t="s">
         <x:v>234</x:v>
       </x:c>
-      <x:c r="H30" s="2" t="s">
+      <x:c r="I30" s="2" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="I30" s="2" t="s">
+      <x:c r="J30" s="2" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="J30" s="2" t="s">
+      <x:c r="K30" s="2" t="s">
         <x:v>237</x:v>
       </x:c>
-      <x:c r="K30" s="2" t="s">
+      <x:c r="L30" s="2" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="M30" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N30" s="64"/>
+      <x:c r="O30" s="65" t="str">
+        <x:f>IF(N30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
+      </x:c>
+      <x:c r="P30" s="65" t="str">
+        <x:f>IF(N30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q30" s="66" t="str">
+        <x:f>IF(N30&lt;&gt;"Yes","",HYPERLINK(K30,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R30" s="66" t="str">
+        <x:f>IF(N30&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S30" s="74"/>
+    </x:row>
+    <x:row r="31" ht="31">
+      <x:c r="A31" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B31),B31&lt;TODAY()),"DEADLINE PASSED",M31)</x:f>
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="B31" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="s">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="L30" s="2" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="M30" s="42"/>
-      <x:c r="N30" s="43" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
-      </x:c>
-      <x:c r="O30" s="43" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P30" s="43" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK(K30,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q30" s="47" t="str">
-        <x:f>IF(M30&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R30" s="52"/>
-    </x:row>
-    <x:row r="31" ht="31">
-      <x:c r="A31" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B31" s="3" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="C31" s="2" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="D31" s="2" t="s">
+      <x:c r="E31" s="2" t="s">
         <x:v>239</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="s">
+      <x:c r="F31" s="2" t="s">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="F31" s="2" t="s">
+      <x:c r="G31" s="2" t="s">
         <x:v>241</x:v>
       </x:c>
-      <x:c r="G31" s="2" t="s">
+      <x:c r="H31" s="2" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="H31" s="2" t="s">
+      <x:c r="I31" s="2" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="J31" s="2" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="K31" s="2" t="s">
         <x:v>243</x:v>
       </x:c>
-      <x:c r="I31" s="2" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="J31" s="2" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="K31" s="2" t="s">
+      <x:c r="L31" s="2" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="M31" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N31" s="64"/>
+      <x:c r="O31" s="65" t="str">
+        <x:f>IF(N31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
+      </x:c>
+      <x:c r="P31" s="65" t="str">
+        <x:f>IF(N31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q31" s="66" t="str">
+        <x:f>IF(N31&lt;&gt;"Yes","",HYPERLINK(K31,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R31" s="66" t="str">
+        <x:f>IF(N31&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S31" s="74"/>
+    </x:row>
+    <x:row r="32" ht="46">
+      <x:c r="A32" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B32),B32&lt;TODAY()),"DEADLINE PASSED",M32)</x:f>
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="L31" s="2" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="M31" s="42"/>
-      <x:c r="N31" s="43" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
-      </x:c>
-      <x:c r="O31" s="43" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P31" s="43" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK(K31,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q31" s="47" t="str">
-        <x:f>IF(M31&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R31" s="52"/>
-    </x:row>
-    <x:row r="32" ht="46">
-      <x:c r="A32" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B32" s="3" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="C32" s="2" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="D32" s="2" t="s">
+      <x:c r="E32" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="E32" s="2" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F32" s="2" t="s">
+      <x:c r="G32" s="2" t="s">
         <x:v>246</x:v>
       </x:c>
-      <x:c r="G32" s="2" t="s">
+      <x:c r="H32" s="2" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="H32" s="2" t="s">
+      <x:c r="I32" s="2" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="J32" s="2" t="s">
         <x:v>248</x:v>
       </x:c>
-      <x:c r="I32" s="2" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="J32" s="2" t="s">
+      <x:c r="K32" s="2" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="K32" s="2" t="s">
+      <x:c r="L32" s="2" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="M32" s="60" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="N32" s="64"/>
+      <x:c r="O32" s="65" t="str">
+        <x:f>IF(N32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
+      </x:c>
+      <x:c r="P32" s="65" t="str">
+        <x:f>IF(N32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q32" s="66" t="str">
+        <x:f>IF(N32&lt;&gt;"Yes","",HYPERLINK(K32,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R32" s="66" t="str">
+        <x:f>IF(N32&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S32" s="74"/>
+    </x:row>
+    <x:row r="33" ht="61">
+      <x:c r="A33" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B33),B33&lt;TODAY()),"DEADLINE PASSED",M33)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="s">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="L32" s="2" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="M32" s="42"/>
-      <x:c r="N32" s="43" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
-      </x:c>
-      <x:c r="O32" s="43" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P32" s="43" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK(K32,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q32" s="47" t="str">
-        <x:f>IF(M32&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R32" s="52"/>
-    </x:row>
-    <x:row r="33" ht="61">
-      <x:c r="A33" s="2" t="s">
+      <x:c r="C33" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="B33" s="3" t="s">
+      <x:c r="E33" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="s">
         <x:v>252</x:v>
       </x:c>
-      <x:c r="C33" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D33" s="2" t="s">
+      <x:c r="G33" s="2" t="s">
         <x:v>253</x:v>
       </x:c>
-      <x:c r="E33" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="F33" s="2" t="s">
+      <x:c r="H33" s="2" t="s">
         <x:v>254</x:v>
       </x:c>
-      <x:c r="G33" s="2" t="s">
+      <x:c r="I33" s="2" t="s">
         <x:v>255</x:v>
       </x:c>
-      <x:c r="H33" s="2" t="s">
+      <x:c r="J33" s="2" t="s">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="I33" s="2" t="s">
+      <x:c r="K33" s="2" t="s">
         <x:v>257</x:v>
       </x:c>
-      <x:c r="J33" s="2" t="s">
+      <x:c r="L33" s="2" t="s">
         <x:v>258</x:v>
       </x:c>
-      <x:c r="K33" s="2" t="s">
+      <x:c r="M33" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N33" s="64"/>
+      <x:c r="O33" s="65" t="str">
+        <x:f>IF(N33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
+      </x:c>
+      <x:c r="P33" s="65" t="str">
+        <x:f>IF(N33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q33" s="66" t="str">
+        <x:f>IF(N33&lt;&gt;"Yes","",HYPERLINK(K33,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R33" s="66" t="str">
+        <x:f>IF(N33&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S33" s="74"/>
+    </x:row>
+    <x:row r="34" ht="46">
+      <x:c r="A34" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B34),B34&lt;TODAY()),"DEADLINE PASSED",M34)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="s">
         <x:v>259</x:v>
       </x:c>
-      <x:c r="L33" s="2" t="s">
+      <x:c r="C34" s="2" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="M33" s="42"/>
-      <x:c r="N33" s="43" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
-      </x:c>
-      <x:c r="O33" s="43" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P33" s="43" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK(K33,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q33" s="47" t="str">
-        <x:f>IF(M33&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R33" s="52"/>
-    </x:row>
-    <x:row r="34" ht="46">
-      <x:c r="A34" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B34" s="3" t="s">
+      <x:c r="D34" s="2" t="s">
         <x:v>261</x:v>
       </x:c>
-      <x:c r="C34" s="2" t="s">
+      <x:c r="E34" s="2" t="s">
         <x:v>262</x:v>
       </x:c>
-      <x:c r="D34" s="2" t="s">
+      <x:c r="F34" s="2" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="E34" s="2" t="s">
+      <x:c r="G34" s="2" t="s">
         <x:v>264</x:v>
       </x:c>
-      <x:c r="F34" s="2" t="s">
+      <x:c r="H34" s="2" t="s">
         <x:v>265</x:v>
       </x:c>
-      <x:c r="G34" s="2" t="s">
+      <x:c r="I34" s="2" t="s">
         <x:v>266</x:v>
       </x:c>
-      <x:c r="H34" s="2" t="s">
+      <x:c r="J34" s="2" t="s">
         <x:v>267</x:v>
       </x:c>
-      <x:c r="I34" s="2" t="s">
+      <x:c r="K34" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L34" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M34" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N34" s="64"/>
+      <x:c r="O34" s="65" t="str">
+        <x:f>IF(N34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
+      </x:c>
+      <x:c r="P34" s="65" t="str">
+        <x:f>IF(N34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q34" s="66" t="str">
+        <x:f>IF(N34&lt;&gt;"Yes","",HYPERLINK(K34,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R34" s="66" t="str">
+        <x:f>IF(N34&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S34" s="74"/>
+    </x:row>
+    <x:row r="35" ht="31">
+      <x:c r="A35" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B35),B35&lt;TODAY()),"DEADLINE PASSED",M35)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="J34" s="2" t="s">
+      <x:c r="E35" s="2" t="s">
         <x:v>269</x:v>
       </x:c>
-      <x:c r="K34" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L34" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M34" s="42"/>
-      <x:c r="N34" s="43" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
-      </x:c>
-      <x:c r="O34" s="43" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P34" s="43" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK(K34,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q34" s="47" t="str">
-        <x:f>IF(M34&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R34" s="52"/>
-    </x:row>
-    <x:row r="35" ht="31">
-      <x:c r="A35" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B35" s="3" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="C35" s="2" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="D35" s="2" t="s">
+      <x:c r="F35" s="2" t="s">
         <x:v>270</x:v>
       </x:c>
-      <x:c r="E35" s="2" t="s">
+      <x:c r="G35" s="2" t="s">
         <x:v>271</x:v>
       </x:c>
-      <x:c r="F35" s="2" t="s">
+      <x:c r="H35" s="2" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="G35" s="2" t="s">
+      <x:c r="I35" s="2" t="s">
         <x:v>273</x:v>
       </x:c>
-      <x:c r="H35" s="2" t="s">
+      <x:c r="J35" s="2" t="s">
         <x:v>274</x:v>
       </x:c>
-      <x:c r="I35" s="2" t="s">
+      <x:c r="K35" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L35" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M35" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N35" s="64"/>
+      <x:c r="O35" s="65" t="str">
+        <x:f>IF(N35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
+      </x:c>
+      <x:c r="P35" s="65" t="str">
+        <x:f>IF(N35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q35" s="66" t="str">
+        <x:f>IF(N35&lt;&gt;"Yes","",HYPERLINK(K35,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R35" s="66" t="str">
+        <x:f>IF(N35&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S35" s="74"/>
+    </x:row>
+    <x:row r="36" ht="31">
+      <x:c r="A36" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B36),B36&lt;TODAY()),"DEADLINE PASSED",M36)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="s">
         <x:v>275</x:v>
       </x:c>
-      <x:c r="J35" s="2" t="s">
+      <x:c r="C36" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="s">
         <x:v>276</x:v>
       </x:c>
-      <x:c r="K35" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L35" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M35" s="42"/>
-      <x:c r="N35" s="43" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
-      </x:c>
-      <x:c r="O35" s="43" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P35" s="43" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK(K35,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q35" s="47" t="str">
-        <x:f>IF(M35&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R35" s="52"/>
-    </x:row>
-    <x:row r="36" ht="31">
-      <x:c r="A36" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B36" s="3" t="s">
+      <x:c r="E36" s="2" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="C36" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D36" s="2" t="s">
+      <x:c r="F36" s="2" t="s">
         <x:v>278</x:v>
       </x:c>
-      <x:c r="E36" s="2" t="s">
+      <x:c r="G36" s="2" t="s">
         <x:v>279</x:v>
       </x:c>
-      <x:c r="F36" s="2" t="s">
+      <x:c r="H36" s="2" t="s">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="G36" s="2" t="s">
+      <x:c r="I36" s="2" t="s">
         <x:v>281</x:v>
       </x:c>
-      <x:c r="H36" s="2" t="s">
+      <x:c r="J36" s="2" t="s">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="I36" s="2" t="s">
+      <x:c r="K36" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L36" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M36" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N36" s="64"/>
+      <x:c r="O36" s="65" t="str">
+        <x:f>IF(N36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
+      </x:c>
+      <x:c r="P36" s="65" t="str">
+        <x:f>IF(N36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q36" s="66" t="str">
+        <x:f>IF(N36&lt;&gt;"Yes","",HYPERLINK(K36,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R36" s="66" t="str">
+        <x:f>IF(N36&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S36" s="74"/>
+    </x:row>
+    <x:row r="37" ht="31">
+      <x:c r="A37" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B37),B37&lt;TODAY()),"DEADLINE PASSED",M37)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="J36" s="2" t="s">
+      <x:c r="D37" s="2" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="K36" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L36" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M36" s="42"/>
-      <x:c r="N36" s="43" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
-      </x:c>
-      <x:c r="O36" s="43" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P36" s="43" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK(K36,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q36" s="47" t="str">
-        <x:f>IF(M36&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R36" s="52"/>
-    </x:row>
-    <x:row r="37" ht="31">
-      <x:c r="A37" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B37" s="3" t="s">
-        <x:v>277</x:v>
-      </x:c>
-      <x:c r="C37" s="2" t="s">
+      <x:c r="E37" s="2" t="s">
         <x:v>285</x:v>
       </x:c>
-      <x:c r="D37" s="2" t="s">
+      <x:c r="F37" s="2" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="E37" s="2" t="s">
+      <x:c r="G37" s="2" t="s">
         <x:v>287</x:v>
       </x:c>
-      <x:c r="F37" s="2" t="s">
+      <x:c r="H37" s="2" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="G37" s="2" t="s">
+      <x:c r="I37" s="2" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="H37" s="2" t="s">
+      <x:c r="J37" s="2" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="I37" s="2" t="s">
+      <x:c r="K37" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L37" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M37" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N37" s="64"/>
+      <x:c r="O37" s="65" t="str">
+        <x:f>IF(N37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
+      </x:c>
+      <x:c r="P37" s="65" t="str">
+        <x:f>IF(N37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q37" s="66" t="str">
+        <x:f>IF(N37&lt;&gt;"Yes","",HYPERLINK(K37,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R37" s="66" t="str">
+        <x:f>IF(N37&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S37" s="74"/>
+    </x:row>
+    <x:row r="38" ht="31">
+      <x:c r="A38" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B38),B38&lt;TODAY()),"DEADLINE PASSED",M38)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="s">
         <x:v>291</x:v>
       </x:c>
-      <x:c r="J37" s="2" t="s">
+      <x:c r="C38" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D38" s="2" t="s">
         <x:v>292</x:v>
       </x:c>
-      <x:c r="K37" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L37" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M37" s="42"/>
-      <x:c r="N37" s="43" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
-      </x:c>
-      <x:c r="O37" s="43" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P37" s="43" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK(K37,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q37" s="47" t="str">
-        <x:f>IF(M37&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R37" s="52"/>
-    </x:row>
-    <x:row r="38" ht="31">
-      <x:c r="A38" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B38" s="3" t="s">
+      <x:c r="E38" s="2" t="s">
         <x:v>293</x:v>
       </x:c>
-      <x:c r="C38" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D38" s="2" t="s">
+      <x:c r="F38" s="2" t="s">
         <x:v>294</x:v>
       </x:c>
-      <x:c r="E38" s="2" t="s">
+      <x:c r="G38" s="2" t="s">
         <x:v>295</x:v>
       </x:c>
-      <x:c r="F38" s="2" t="s">
+      <x:c r="H38" s="2" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="G38" s="2" t="s">
+      <x:c r="I38" s="2" t="s">
         <x:v>297</x:v>
       </x:c>
-      <x:c r="H38" s="2" t="s">
+      <x:c r="J38" s="2" t="s">
         <x:v>298</x:v>
       </x:c>
-      <x:c r="I38" s="2" t="s">
+      <x:c r="K38" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L38" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M38" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N38" s="64"/>
+      <x:c r="O38" s="65" t="str">
+        <x:f>IF(N38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
+      </x:c>
+      <x:c r="P38" s="65" t="str">
+        <x:f>IF(N38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q38" s="66" t="str">
+        <x:f>IF(N38&lt;&gt;"Yes","",HYPERLINK(K38,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R38" s="66" t="str">
+        <x:f>IF(N38&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S38" s="74"/>
+    </x:row>
+    <x:row r="39" ht="31">
+      <x:c r="A39" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B39),B39&lt;TODAY()),"DEADLINE PASSED",M39)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D39" s="2" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="J38" s="2" t="s">
+      <x:c r="E39" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F39" s="2" t="s">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="K38" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L38" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M38" s="42"/>
-      <x:c r="N38" s="43" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
-      </x:c>
-      <x:c r="O38" s="43" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P38" s="43" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK(K38,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q38" s="47" t="str">
-        <x:f>IF(M38&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R38" s="52"/>
-    </x:row>
-    <x:row r="39" ht="31">
-      <x:c r="A39" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B39" s="3" t="s">
-        <x:v>293</x:v>
-      </x:c>
-      <x:c r="C39" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D39" s="2" t="s">
+      <x:c r="G39" s="2" t="s">
         <x:v>301</x:v>
       </x:c>
-      <x:c r="E39" s="2" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F39" s="2" t="s">
+      <x:c r="H39" s="2" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="G39" s="2" t="s">
+      <x:c r="I39" s="2" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="H39" s="2" t="s">
+      <x:c r="J39" s="2" t="s">
         <x:v>304</x:v>
       </x:c>
-      <x:c r="I39" s="2" t="s">
+      <x:c r="K39" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L39" s="2" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M39" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N39" s="64"/>
+      <x:c r="O39" s="65" t="str">
+        <x:f>IF(N39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
+      </x:c>
+      <x:c r="P39" s="65" t="str">
+        <x:f>IF(N39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q39" s="66" t="str">
+        <x:f>IF(N39&lt;&gt;"Yes","",HYPERLINK(K39,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R39" s="66" t="str">
+        <x:f>IF(N39&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S39" s="74"/>
+    </x:row>
+    <x:row r="40" ht="31">
+      <x:c r="A40" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B40),B40&lt;TODAY()),"DEADLINE PASSED",M40)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="s">
         <x:v>305</x:v>
       </x:c>
-      <x:c r="J39" s="2" t="s">
+      <x:c r="C40" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D40" s="2" t="s">
         <x:v>306</x:v>
       </x:c>
-      <x:c r="K39" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="L39" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M39" s="42"/>
-      <x:c r="N39" s="43" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
-      </x:c>
-      <x:c r="O39" s="43" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P39" s="43" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK(K39,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q39" s="47" t="str">
-        <x:f>IF(M39&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R39" s="52"/>
-    </x:row>
-    <x:row r="40" ht="31">
-      <x:c r="A40" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="B40" s="3" t="s">
+      <x:c r="E40" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F40" s="2" t="s">
         <x:v>307</x:v>
       </x:c>
-      <x:c r="C40" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D40" s="2" t="s">
+      <x:c r="G40" s="2" t="s">
         <x:v>308</x:v>
       </x:c>
-      <x:c r="E40" s="2" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F40" s="2" t="s">
+      <x:c r="H40" s="2" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="G40" s="2" t="s">
+      <x:c r="I40" s="2" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="H40" s="2" t="s">
+      <x:c r="J40" s="2" t="s">
         <x:v>311</x:v>
       </x:c>
-      <x:c r="I40" s="2" t="s">
-        <x:v>312</x:v>
-      </x:c>
-      <x:c r="J40" s="2" t="s">
-        <x:v>313</x:v>
-      </x:c>
       <x:c r="K40" s="2" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L40" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="M40" s="42"/>
-      <x:c r="N40" s="43" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
-      </x:c>
-      <x:c r="O40" s="43" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P40" s="43" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK(K40,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q40" s="47" t="str">
-        <x:f>IF(M40&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R40" s="52"/>
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M40" s="60" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="N40" s="64"/>
+      <x:c r="O40" s="65" t="str">
+        <x:f>IF(N40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
+      </x:c>
+      <x:c r="P40" s="65" t="str">
+        <x:f>IF(N40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q40" s="66" t="str">
+        <x:f>IF(N40&lt;&gt;"Yes","",HYPERLINK(K40,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R40" s="66" t="str">
+        <x:f>IF(N40&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S40" s="74"/>
     </x:row>
     <x:row r="41" ht="45">
-      <x:c r="A41" s="2" t="s">
-        <x:v>314</x:v>
+      <x:c r="A41" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B41),B41&lt;TODAY()),"DEADLINE PASSED",M41)</x:f>
+        <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B41" s="3">
         <x:v>46283</x:v>
       </x:c>
       <x:c r="C41" s="2" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="D41" s="2" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="E41" s="2" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="F41" s="2" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="D41" s="2" t="s">
+      <x:c r="G41" s="2" t="s">
         <x:v>316</x:v>
       </x:c>
-      <x:c r="E41" s="2" t="s">
+      <x:c r="H41" s="2" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="F41" s="2" t="s">
+      <x:c r="I41" s="2" t="s">
         <x:v>318</x:v>
       </x:c>
-      <x:c r="G41" s="2" t="s">
+      <x:c r="J41" s="2" t="s">
         <x:v>319</x:v>
       </x:c>
-      <x:c r="H41" s="2" t="s">
+      <x:c r="K41" s="2" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="I41" s="2" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="J41" s="2" t="s">
-        <x:v>322</x:v>
-      </x:c>
-      <x:c r="K41" s="2" t="s">
-        <x:v>323</x:v>
-      </x:c>
       <x:c r="L41" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M41" s="42"/>
-      <x:c r="N41" s="43" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
-      </x:c>
-      <x:c r="O41" s="43" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P41" s="43" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK(K41,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q41" s="47" t="str">
-        <x:f>IF(M41&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R41" s="52"/>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M41" s="60" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="N41" s="64"/>
+      <x:c r="O41" s="65" t="str">
+        <x:f>IF(N41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
+      </x:c>
+      <x:c r="P41" s="65" t="str">
+        <x:f>IF(N41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q41" s="66" t="str">
+        <x:f>IF(N41&lt;&gt;"Yes","",HYPERLINK(K41,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R41" s="66" t="str">
+        <x:f>IF(N41&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S41" s="74"/>
     </x:row>
     <x:row r="42" ht="45">
-      <x:c r="A42" s="2" t="s">
-        <x:v>324</x:v>
+      <x:c r="A42" s="2" t="str">
+        <x:f>IF(AND(ISNUMBER(B42),B42&lt;TODAY()),"DEADLINE PASSED",M42)</x:f>
+        <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B42" s="3">
         <x:v>46286</x:v>
       </x:c>
       <x:c r="C42" s="2" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="D42" s="2" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="E42" s="2" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="F42" s="2" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="G42" s="2" t="s">
         <x:v>325</x:v>
       </x:c>
-      <x:c r="D42" s="2" t="s">
+      <x:c r="H42" s="2" t="s">
         <x:v>326</x:v>
       </x:c>
-      <x:c r="E42" s="2" t="s">
+      <x:c r="I42" s="2" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="F42" s="2" t="s">
+      <x:c r="J42" s="2" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="G42" s="2" t="s">
+      <x:c r="K42" s="2" t="s">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="H42" s="2" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="I42" s="2" t="s">
-        <x:v>331</x:v>
-      </x:c>
-      <x:c r="J42" s="2" t="s">
-        <x:v>332</x:v>
-      </x:c>
-      <x:c r="K42" s="2" t="s">
-        <x:v>333</x:v>
-      </x:c>
       <x:c r="L42" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="M42" s="42"/>
-      <x:c r="N42" s="43" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
-      </x:c>
-      <x:c r="O42" s="43" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="P42" s="43" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK(K42,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="Q42" s="47" t="str">
-        <x:f>IF(M42&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="R42" s="52"/>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M42" s="60" t="str">
+        <x:v>CLOSED – invited stage continues</x:v>
+      </x:c>
+      <x:c r="N42" s="64"/>
+      <x:c r="O42" s="65" t="str">
+        <x:f>IF(N42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
+      </x:c>
+      <x:c r="P42" s="65" t="str">
+        <x:f>IF(N42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="Q42" s="66" t="str">
+        <x:f>IF(N42&lt;&gt;"Yes","",HYPERLINK(K42,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="R42" s="66" t="str">
+        <x:f>IF(N42&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="S42" s="74"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
@@ -3872,15 +4102,19 @@
     <x:cfRule type="expression" dxfId="0" priority="3">
       <x:formula>LEFT(A2,6)="CLOSED"</x:formula>
     </x:cfRule>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="DEADLINE PASSED"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="M2:M500">
+      <x:formula1>"OPEN,FORTHCOMING,CLOSED – monitor recurrence,CLOSED – invited stage continues"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N2:N500">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc72960c867a644e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa1ba6ec97d4c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3895,152 +4129,152 @@
   <x:sheetData>
     <x:row r="1" ht="21">
       <x:c r="A1" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
     </x:row>
     <x:row r="2" ht="30">
       <x:c r="A2" s="4" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>336</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="16">
       <x:c r="A3" s="4" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>338</x:v>
+        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45">
       <x:c r="A4" s="4" t="s">
-        <x:v>339</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>340</x:v>
+        <x:v>336</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30">
       <x:c r="A5" s="4" t="s">
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>342</x:v>
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>OPEN = live and accepting applications; FORTHCOMING = announced by funder but final call may not yet be live; CLOSED – monitor recurrence = useful recurring/strategic call retained for planning; DEADLINE PASSED = assigned automatically when an exact deadline is before today.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
       <x:c r="A6" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>344</x:v>
+        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30">
       <x:c r="A7" s="4" t="s">
-        <x:v>345</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>346</x:v>
+        <x:v>341</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>348</x:v>
+        <x:v>343</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>350</x:v>
+        <x:v>345</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>351</x:v>
+        <x:v>346</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="4" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="B13" s="2" t="s">
-        <x:v>352</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B14" s="2" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B15" s="2" t="s">
-        <x:v>353</x:v>
+        <x:v>348</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="16">
       <x:c r="A16" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B16" s="2" t="s">
-        <x:v>326</x:v>
+        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="16">
       <x:c r="A17" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B17" s="2" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16">
       <x:c r="A18" s="4" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B18" s="2" t="s">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="45">
       <x:c r="A19" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="B19" s="2" t="s">
-        <x:v>355</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">

</xml_diff>

<commit_message>
Fix passed deadline status formatting
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="Rcb104da50cfe4301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Ref6975e7535a448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="Rce7cf20ff58f49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R3b30b56cb3b94a0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1072,7 +1072,7 @@
     <x:numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
     <x:numFmt numFmtId="200" formatCode="dd mmm yyyy"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1121,8 +1121,14 @@
       <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF990000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1234,6 +1240,11 @@
         <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -1241,7 +1252,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="80">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1440,11 +1451,20 @@
     <x:xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="5">
     <x:dxf>
       <x:font>
         <x:color rgb="FF666666"/>
@@ -1474,6 +1494,17 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF990000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1796,7 +1827,7 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="31">
-      <x:c r="A2" s="2" t="str">
+      <x:c r="A2" s="82" t="str">
         <x:f>IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",M2)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
@@ -1852,7 +1883,7 @@
       <x:c r="S2" s="74"/>
     </x:row>
     <x:row r="3" ht="31">
-      <x:c r="A3" s="2" t="str">
+      <x:c r="A3" s="82" t="str">
         <x:f>IF(AND(ISNUMBER(B3),B3&lt;TODAY()),"DEADLINE PASSED",M3)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
@@ -3980,7 +4011,7 @@
       <x:c r="S40" s="74"/>
     </x:row>
     <x:row r="41" ht="45">
-      <x:c r="A41" s="2" t="str">
+      <x:c r="A41" s="82" t="str">
         <x:f>IF(AND(ISNUMBER(B41),B41&lt;TODAY()),"DEADLINE PASSED",M41)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
@@ -4036,7 +4067,7 @@
       <x:c r="S41" s="74"/>
     </x:row>
     <x:row r="42" ht="45">
-      <x:c r="A42" s="2" t="str">
+      <x:c r="A42" s="82" t="str">
         <x:f>IF(AND(ISNUMBER(B42),B42&lt;TODAY()),"DEADLINE PASSED",M42)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
@@ -4093,16 +4124,9 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
-    <x:cfRule type="expression" dxfId="2" priority="1">
-      <x:formula>A2="OPEN"</x:formula>
+    <x:cfRule type="expression" dxfId="4" priority="1">
+      <x:formula>$A2="DEADLINE PASSED"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="1" priority="2">
-      <x:formula>A2="FORTHCOMING"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="0" priority="3">
-      <x:formula>LEFT(A2,6)="CLOSED"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="DEADLINE PASSED"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="M2:M500">
@@ -4114,7 +4138,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa1ba6ec97d4c36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra524a45f248d4a59"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Classify funding by research or scholarship
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="Rc981d89a9e014432"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="Rb04f1adb9c9f4d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R19e92bb378c240d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R792b31c736944b7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,27 +47,6 @@
     <x:t xml:space="preserve">Source list</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Manual Status</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notify?</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Email subject</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Email body</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Official opportunity link</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Funding Finder link</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notification date</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">LMS</x:t>
   </x:si>
   <x:si>
@@ -95,9 +74,6 @@
     <x:t xml:space="preserve">https://www.lms.ac.uk/grants/calendar</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">OPEN</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">ARIA</x:t>
   </x:si>
   <x:si>
@@ -812,9 +788,6 @@
     <x:t xml:space="preserve">UKRI future</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">FORTHCOMING</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Oct 2026</x:t>
   </x:si>
   <x:si>
@@ -1001,9 +974,6 @@
     <x:t xml:space="preserve">https://www.gla.ac.uk/myglasgow/ris/ieed/innovation/innovationfunds/medtechinnovationfund/</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">CLOSED – monitor recurrence</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">SWIFT / EPSRC</x:t>
   </x:si>
   <x:si>
@@ -1029,9 +999,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://swiftoffshore.co.uk/funding/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CLOSED – invited stage continues</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Funding Finder for Statistics (FFS) – working master list</x:t>
@@ -1134,8 +1101,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
+    <x:numFmt numFmtId="200" formatCode="dd mmm yyyy"/>
   </x:numFmts>
   <x:fonts count="13">
     <x:font>
@@ -1211,7 +1179,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1273,6 +1241,26 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -1280,7 +1268,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1348,11 +1336,123 @@
     <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="5">
+  <x:dxfs count="9">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF990000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF38761D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF595959"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1413,9 +1513,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:S42" totalsRowShown="0">
-  <x:autoFilter ref="A1:S42"/>
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:T42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:T42"/>
+  <x:tableColumns count="20">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Deadline"/>
     <x:tableColumn id="3" name="Funder"/>
@@ -1428,13 +1528,14 @@
     <x:tableColumn id="10" name="Internal action / note"/>
     <x:tableColumn id="11" name="Source"/>
     <x:tableColumn id="12" name="Source list"/>
-    <x:tableColumn id="13" name="Manual Status"/>
-    <x:tableColumn id="14" name="Notify?"/>
-    <x:tableColumn id="15" name="Email subject"/>
-    <x:tableColumn id="16" name="Email body"/>
-    <x:tableColumn id="17" name="Official opportunity link"/>
-    <x:tableColumn id="18" name="Funding Finder link"/>
-    <x:tableColumn id="19" name="Notification date"/>
+    <x:tableColumn id="13" name="Research / Scholarship"/>
+    <x:tableColumn id="14" name="Status setting"/>
+    <x:tableColumn id="15" name="Notify?"/>
+    <x:tableColumn id="16" name="Email subject"/>
+    <x:tableColumn id="17" name="Email body"/>
+    <x:tableColumn id="18" name="Official opportunity link"/>
+    <x:tableColumn id="19" name="Funding Finder link"/>
+    <x:tableColumn id="20" name="Notification date"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1647,13 +1748,14 @@
     <x:col min="10" max="10" width="42" customWidth="1"/>
     <x:col min="11" max="11" width="50" customWidth="1"/>
     <x:col min="12" max="12" width="18" customWidth="1"/>
-    <x:col min="13" max="13" width="27" customWidth="1"/>
-    <x:col min="14" max="14" width="11" customWidth="1"/>
-    <x:col min="15" max="15" width="32" customWidth="1"/>
-    <x:col min="16" max="16" width="48" customWidth="1"/>
-    <x:col min="17" max="17" width="24" customWidth="1"/>
-    <x:col min="18" max="18" width="20" customWidth="1"/>
-    <x:col min="19" max="19" width="17" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="27" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="11" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="32" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="48" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="60.25" customHeight="1">
@@ -1693,2350 +1795,2561 @@
       <x:c r="L1" s="1" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="15" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="N1" s="12" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="O1" s="12" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="P1" s="12" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="Q1" s="12" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="R1" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="S1" s="12" t="s">
-        <x:v>18</x:v>
+      <x:c r="M1" s="39" t="str">
+        <x:v>Research / Scholarship</x:v>
+      </x:c>
+      <x:c r="N1" s="39" t="str">
+        <x:v>Status setting</x:v>
+      </x:c>
+      <x:c r="O1" s="39" t="str">
+        <x:v>Notify?</x:v>
+      </x:c>
+      <x:c r="P1" s="39" t="str">
+        <x:v>Email subject</x:v>
+      </x:c>
+      <x:c r="Q1" s="39" t="str">
+        <x:v>Email body</x:v>
+      </x:c>
+      <x:c r="R1" s="39" t="str">
+        <x:v>Official opportunity link</x:v>
+      </x:c>
+      <x:c r="S1" s="39" t="str">
+        <x:v>Funding Finder link</x:v>
+      </x:c>
+      <x:c r="T1" s="39" t="str">
+        <x:v>Notification date</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="30">
       <x:c r="A2" s="16" t="str">
-        <x:f t="shared" ref="A2:A42" ca="1" si="0">IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",M2)</x:f>
+        <x:f t="shared" ref="A2:A42" ca="1" si="0">IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",N2)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B2" s="3">
         <x:v>46295</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="s">
+      <x:c r="K2" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F2" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G2" s="2" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="H2" s="2" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="I2" s="2" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="J2" s="2" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="K2" s="2" t="s">
-        <x:v>27</x:v>
-      </x:c>
       <x:c r="L2" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M2" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N2" s="8"/>
-      <x:c r="O2" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M2" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N2" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O2" s="23">
         <x:f t="shared" ref="O2:O42" si="1">IF(N2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
       </x:c>
-      <x:c r="P2" s="9" t="str">
-        <x:f t="shared" ref="P2:P42" si="2">IF(N2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
-      </x:c>
-      <x:c r="Q2" s="10" t="str">
-        <x:f t="shared" ref="Q2:Q42" si="3">IF(N2&lt;&gt;"Yes","",HYPERLINK(K2,"View official opportunity"))</x:f>
-      </x:c>
-      <x:c r="R2" s="10" t="str">
-        <x:f t="shared" ref="R2:R42" si="4">IF(N2&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
-      </x:c>
-      <x:c r="S2" s="11"/>
+      <x:c r="P2" s="31" t="str">
+        <x:f t="shared" ref="P2:P42" si="2">IF(O2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
+      </x:c>
+      <x:c r="Q2" s="32" t="str">
+        <x:f t="shared" ref="Q2:Q42" si="3">IF(O2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R2" s="32" t="str">
+        <x:f t="shared" ref="R2:R42" si="4">IF(O2&lt;&gt;"Yes","",HYPERLINK(K2,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S2" s="32" t="str">
+        <x:f>IF(O2&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T2" s="38"/>
     </x:row>
     <x:row r="3" ht="30">
       <x:c r="A3" s="16" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B3),B3&lt;TODAY()),"DEADLINE PASSED",N3)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>46295</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J3" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F3" s="2" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="G3" s="2" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H3" s="2" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="I3" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="J3" s="2" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="K3" s="2" t="s">
-        <x:v>37</x:v>
-      </x:c>
       <x:c r="L3" s="2" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="M3" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N3" s="8"/>
-      <x:c r="O3" s="9" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M3" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N3" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O3" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P3" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q3" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R3" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S3" s="11"/>
+      <x:c r="P3" s="31" t="str">
+        <x:f t="shared" si="2">IF(O3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
+      </x:c>
+      <x:c r="Q3" s="32" t="str">
+        <x:f t="shared" si="3">IF(O3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R3" s="32" t="str">
+        <x:f t="shared" si="4">IF(O3&lt;&gt;"Yes","",HYPERLINK(K3,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S3" s="32" t="str">
+        <x:f>IF(O3&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T3" s="38"/>
     </x:row>
     <x:row r="4" ht="30">
       <x:c r="A4" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B4),B4&lt;TODAY()),"DEADLINE PASSED",N4)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B4" s="3">
         <x:v>46296</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="J4" s="2" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="K4" s="2" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="E4" s="2" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F4" s="2" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G4" s="2" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="H4" s="2" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="I4" s="2" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="J4" s="2" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="K4" s="2" t="s">
-        <x:v>46</x:v>
-      </x:c>
       <x:c r="L4" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M4" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N4" s="8"/>
-      <x:c r="O4" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M4" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N4" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O4" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P4" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q4" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R4" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S4" s="11"/>
+      <x:c r="P4" s="31" t="str">
+        <x:f t="shared" si="2">IF(O4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
+      </x:c>
+      <x:c r="Q4" s="32" t="str">
+        <x:f t="shared" si="3">IF(O4&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D4&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C4&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B4),TEXT(B4,"d mmmm yyyy"),B4)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F4&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G4&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H4&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I4&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R4" s="32" t="str">
+        <x:f t="shared" si="4">IF(O4&lt;&gt;"Yes","",HYPERLINK(K4,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S4" s="32" t="str">
+        <x:f>IF(O4&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T4" s="38"/>
     </x:row>
     <x:row r="5" ht="45">
       <x:c r="A5" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B5),B5&lt;TODAY()),"DEADLINE PASSED",N5)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B5" s="3">
         <x:v>46304</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>29</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="2" t="s">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F5" s="2" t="s">
-        <x:v>48</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G5" s="2" t="s">
-        <x:v>49</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H5" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="I5" s="2" t="s">
-        <x:v>51</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="J5" s="2" t="s">
-        <x:v>52</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="K5" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="L5" s="2" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="M5" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N5" s="8"/>
-      <x:c r="O5" s="9" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M5" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N5" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O5" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P5" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q5" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R5" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S5" s="11"/>
+      <x:c r="P5" s="31" t="str">
+        <x:f t="shared" si="2">IF(O5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
+      </x:c>
+      <x:c r="Q5" s="32" t="str">
+        <x:f t="shared" si="3">IF(O5&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D5&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C5&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B5),TEXT(B5,"d mmmm yyyy"),B5)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F5&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G5&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H5&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I5&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R5" s="32" t="str">
+        <x:f t="shared" si="4">IF(O5&lt;&gt;"Yes","",HYPERLINK(K5,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S5" s="32" t="str">
+        <x:f>IF(O5&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T5" s="38"/>
     </x:row>
     <x:row r="6" ht="30">
       <x:c r="A6" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B6),B6&lt;TODAY()),"DEADLINE PASSED",N6)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B6" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C6" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D6" s="2" t="s">
-        <x:v>54</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E6" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F6" s="2" t="s">
-        <x:v>56</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="G6" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="H6" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="I6" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="J6" s="2" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="K6" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L6" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M6" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N6" s="8"/>
-      <x:c r="O6" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M6" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N6" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O6" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P6" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q6" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R6" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S6" s="11"/>
+      <x:c r="P6" s="31" t="str">
+        <x:f t="shared" si="2">IF(O6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
+      </x:c>
+      <x:c r="Q6" s="32" t="str">
+        <x:f t="shared" si="3">IF(O6&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D6&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C6&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B6),TEXT(B6,"d mmmm yyyy"),B6)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F6&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G6&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H6&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I6&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R6" s="32" t="str">
+        <x:f t="shared" si="4">IF(O6&lt;&gt;"Yes","",HYPERLINK(K6,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S6" s="32" t="str">
+        <x:f>IF(O6&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T6" s="38"/>
     </x:row>
     <x:row r="7" ht="30">
       <x:c r="A7" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B7),B7&lt;TODAY()),"DEADLINE PASSED",N7)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B7" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D7" s="2" t="s">
-        <x:v>61</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>62</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F7" s="2" t="s">
-        <x:v>63</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="G7" s="2" t="s">
-        <x:v>64</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="H7" s="2" t="s">
-        <x:v>65</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="I7" s="2" t="s">
-        <x:v>66</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="J7" s="2" t="s">
-        <x:v>60</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="K7" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L7" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M7" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N7" s="8"/>
-      <x:c r="O7" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M7" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N7" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O7" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P7" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q7" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R7" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S7" s="11"/>
+      <x:c r="P7" s="31" t="str">
+        <x:f t="shared" si="2">IF(O7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
+      </x:c>
+      <x:c r="Q7" s="32" t="str">
+        <x:f t="shared" si="3">IF(O7&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D7&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C7&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B7),TEXT(B7,"d mmmm yyyy"),B7)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F7&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G7&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H7&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I7&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R7" s="32" t="str">
+        <x:f t="shared" si="4">IF(O7&lt;&gt;"Yes","",HYPERLINK(K7,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S7" s="32" t="str">
+        <x:f>IF(O7&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T7" s="38"/>
     </x:row>
     <x:row r="8" ht="45">
       <x:c r="A8" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B8),B8&lt;TODAY()),"DEADLINE PASSED",N8)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B8" s="3">
         <x:v>46310</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D8" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F8" s="2" t="s">
-        <x:v>69</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="G8" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="H8" s="2" t="s">
-        <x:v>71</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="I8" s="2" t="s">
-        <x:v>72</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="J8" s="2" t="s">
-        <x:v>73</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="K8" s="2" t="s">
-        <x:v>74</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="L8" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M8" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N8" s="8"/>
-      <x:c r="O8" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M8" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N8" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O8" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P8" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q8" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R8" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S8" s="11"/>
+      <x:c r="P8" s="31" t="str">
+        <x:f t="shared" si="2">IF(O8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
+      </x:c>
+      <x:c r="Q8" s="32" t="str">
+        <x:f t="shared" si="3">IF(O8&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D8&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C8&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B8),TEXT(B8,"d mmmm yyyy"),B8)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F8&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G8&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H8&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I8&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R8" s="32" t="str">
+        <x:f t="shared" si="4">IF(O8&lt;&gt;"Yes","",HYPERLINK(K8,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S8" s="32" t="str">
+        <x:f>IF(O8&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T8" s="38"/>
     </x:row>
     <x:row r="9" ht="30">
       <x:c r="A9" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B9),B9&lt;TODAY()),"DEADLINE PASSED",N9)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B9" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="J9" s="2" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="K9" s="2" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="D9" s="2" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="E9" s="2" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="F9" s="2" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="G9" s="2" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="H9" s="2" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="I9" s="2" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="J9" s="2" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="K9" s="2" t="s">
-        <x:v>83</x:v>
-      </x:c>
       <x:c r="L9" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M9" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N9" s="8"/>
-      <x:c r="O9" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M9" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N9" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O9" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P9" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q9" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R9" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S9" s="11"/>
+      <x:c r="P9" s="31" t="str">
+        <x:f t="shared" si="2">IF(O9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
+      </x:c>
+      <x:c r="Q9" s="32" t="str">
+        <x:f t="shared" si="3">IF(O9&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D9&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C9&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B9),TEXT(B9,"d mmmm yyyy"),B9)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F9&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G9&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H9&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I9&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R9" s="32" t="str">
+        <x:f t="shared" si="4">IF(O9&lt;&gt;"Yes","",HYPERLINK(K9,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S9" s="32" t="str">
+        <x:f>IF(O9&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T9" s="38"/>
     </x:row>
     <x:row r="10" ht="30">
       <x:c r="A10" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B10),B10&lt;TODAY()),"DEADLINE PASSED",N10)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B10" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D10" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E10" s="2" t="s">
-        <x:v>85</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F10" s="2" t="s">
-        <x:v>86</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="G10" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H10" s="2" t="s">
-        <x:v>88</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="I10" s="2" t="s">
-        <x:v>89</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="J10" s="2" t="s">
-        <x:v>90</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="K10" s="2" t="s">
-        <x:v>91</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="L10" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M10" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N10" s="8"/>
-      <x:c r="O10" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M10" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N10" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O10" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P10" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q10" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R10" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S10" s="11"/>
+      <x:c r="P10" s="31" t="str">
+        <x:f t="shared" si="2">IF(O10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
+      </x:c>
+      <x:c r="Q10" s="32" t="str">
+        <x:f t="shared" si="3">IF(O10&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D10&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C10&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B10),TEXT(B10,"d mmmm yyyy"),B10)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F10&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G10&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H10&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I10&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R10" s="32" t="str">
+        <x:f t="shared" si="4">IF(O10&lt;&gt;"Yes","",HYPERLINK(K10,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S10" s="32" t="str">
+        <x:f>IF(O10&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T10" s="38"/>
     </x:row>
     <x:row r="11" ht="30">
       <x:c r="A11" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B11),B11&lt;TODAY()),"DEADLINE PASSED",N11)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B11" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D11" s="2" t="s">
-        <x:v>92</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E11" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F11" s="2" t="s">
-        <x:v>94</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="G11" s="2" t="s">
-        <x:v>95</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="H11" s="2" t="s">
-        <x:v>96</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="I11" s="2" t="s">
-        <x:v>97</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="J11" s="2" t="s">
-        <x:v>98</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="K11" s="2" t="s">
-        <x:v>99</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="L11" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M11" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N11" s="8"/>
-      <x:c r="O11" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M11" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N11" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O11" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P11" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q11" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R11" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S11" s="11"/>
+      <x:c r="P11" s="31" t="str">
+        <x:f t="shared" si="2">IF(O11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
+      </x:c>
+      <x:c r="Q11" s="32" t="str">
+        <x:f t="shared" si="3">IF(O11&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D11&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C11&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B11),TEXT(B11,"d mmmm yyyy"),B11)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F11&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G11&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H11&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I11&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R11" s="32" t="str">
+        <x:f t="shared" si="4">IF(O11&lt;&gt;"Yes","",HYPERLINK(K11,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S11" s="32" t="str">
+        <x:f>IF(O11&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T11" s="38"/>
     </x:row>
     <x:row r="12" ht="30">
       <x:c r="A12" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B12),B12&lt;TODAY()),"DEADLINE PASSED",N12)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B12" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C12" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D12" s="2" t="s">
-        <x:v>100</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E12" s="2" t="s">
-        <x:v>101</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F12" s="2" t="s">
-        <x:v>102</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="G12" s="2" t="s">
-        <x:v>103</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="H12" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="I12" s="2" t="s">
-        <x:v>105</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="J12" s="2" t="s">
-        <x:v>106</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="K12" s="2" t="s">
-        <x:v>107</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="L12" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M12" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N12" s="8"/>
-      <x:c r="O12" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M12" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N12" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O12" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P12" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q12" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R12" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S12" s="11"/>
+      <x:c r="P12" s="31" t="str">
+        <x:f t="shared" si="2">IF(O12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
+      </x:c>
+      <x:c r="Q12" s="32" t="str">
+        <x:f t="shared" si="3">IF(O12&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D12&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C12&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B12),TEXT(B12,"d mmmm yyyy"),B12)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F12&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G12&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H12&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I12&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R12" s="32" t="str">
+        <x:f t="shared" si="4">IF(O12&lt;&gt;"Yes","",HYPERLINK(K12,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S12" s="32" t="str">
+        <x:f>IF(O12&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T12" s="38"/>
     </x:row>
     <x:row r="13" ht="30">
       <x:c r="A13" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B13),B13&lt;TODAY()),"DEADLINE PASSED",N13)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B13" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C13" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D13" s="2" t="s">
-        <x:v>108</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E13" s="2" t="s">
-        <x:v>109</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="F13" s="2" t="s">
-        <x:v>110</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="G13" s="2" t="s">
-        <x:v>111</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="H13" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="I13" s="2" t="s">
-        <x:v>113</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="J13" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="K13" s="2" t="s">
-        <x:v>115</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="L13" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M13" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N13" s="8"/>
-      <x:c r="O13" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M13" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N13" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O13" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P13" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q13" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R13" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S13" s="11"/>
+      <x:c r="P13" s="31" t="str">
+        <x:f t="shared" si="2">IF(O13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
+      </x:c>
+      <x:c r="Q13" s="32" t="str">
+        <x:f t="shared" si="3">IF(O13&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D13&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C13&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B13),TEXT(B13,"d mmmm yyyy"),B13)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F13&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G13&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H13&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I13&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R13" s="32" t="str">
+        <x:f t="shared" si="4">IF(O13&lt;&gt;"Yes","",HYPERLINK(K13,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S13" s="32" t="str">
+        <x:f>IF(O13&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T13" s="38"/>
     </x:row>
     <x:row r="14" ht="45">
       <x:c r="A14" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B14),B14&lt;TODAY()),"DEADLINE PASSED",N14)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B14" s="3">
         <x:v>46316</x:v>
       </x:c>
       <x:c r="C14" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D14" s="2" t="s">
-        <x:v>116</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="E14" s="2" t="s">
-        <x:v>101</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F14" s="2" t="s">
-        <x:v>117</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="G14" s="2" t="s">
-        <x:v>118</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="H14" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="I14" s="2" t="s">
-        <x:v>120</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="J14" s="2" t="s">
-        <x:v>121</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="K14" s="2" t="s">
-        <x:v>122</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="L14" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M14" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N14" s="8"/>
-      <x:c r="O14" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M14" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N14" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O14" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P14" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q14" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R14" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S14" s="11"/>
+      <x:c r="P14" s="31" t="str">
+        <x:f t="shared" si="2">IF(O14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
+      </x:c>
+      <x:c r="Q14" s="32" t="str">
+        <x:f t="shared" si="3">IF(O14&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D14&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C14&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B14),TEXT(B14,"d mmmm yyyy"),B14)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F14&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G14&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H14&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I14&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R14" s="32" t="str">
+        <x:f t="shared" si="4">IF(O14&lt;&gt;"Yes","",HYPERLINK(K14,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S14" s="32" t="str">
+        <x:f>IF(O14&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T14" s="38"/>
     </x:row>
     <x:row r="15" ht="45">
       <x:c r="A15" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B15),B15&lt;TODAY()),"DEADLINE PASSED",N15)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B15" s="3">
         <x:v>46323</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="G15" s="2" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="H15" s="2" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="I15" s="2" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="J15" s="2" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="K15" s="2" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="D15" s="2" t="s">
+      <x:c r="L15" s="2" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="E15" s="2" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F15" s="2" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G15" s="2" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="H15" s="2" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="I15" s="2" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="J15" s="2" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="K15" s="2" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="L15" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M15" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N15" s="8"/>
-      <x:c r="O15" s="9" t="str">
+      <x:c r="M15" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N15" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O15" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P15" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q15" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R15" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S15" s="11"/>
+      <x:c r="P15" s="31" t="str">
+        <x:f t="shared" si="2">IF(O15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
+      </x:c>
+      <x:c r="Q15" s="32" t="str">
+        <x:f t="shared" si="3">IF(O15&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D15&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C15&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B15),TEXT(B15,"d mmmm yyyy"),B15)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F15&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G15&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I15&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R15" s="32" t="str">
+        <x:f t="shared" si="4">IF(O15&lt;&gt;"Yes","",HYPERLINK(K15,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S15" s="32" t="str">
+        <x:f>IF(O15&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T15" s="38"/>
     </x:row>
     <x:row r="16" ht="30">
       <x:c r="A16" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B16),B16&lt;TODAY()),"DEADLINE PASSED",N16)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B16" s="3">
         <x:v>46328</x:v>
       </x:c>
       <x:c r="C16" s="2" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="G16" s="2" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="H16" s="2" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="I16" s="2" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="J16" s="2" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="K16" s="2" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="D16" s="2" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="E16" s="2" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="F16" s="2" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="G16" s="2" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="H16" s="2" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="I16" s="2" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="J16" s="2" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="K16" s="2" t="s">
-        <x:v>141</x:v>
-      </x:c>
       <x:c r="L16" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M16" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N16" s="8"/>
-      <x:c r="O16" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M16" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N16" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O16" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P16" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q16" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R16" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S16" s="11"/>
+      <x:c r="P16" s="31" t="str">
+        <x:f t="shared" si="2">IF(O16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
+      </x:c>
+      <x:c r="Q16" s="32" t="str">
+        <x:f t="shared" si="3">IF(O16&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D16&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C16&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B16),TEXT(B16,"d mmmm yyyy"),B16)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F16&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G16&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I16&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R16" s="32" t="str">
+        <x:f t="shared" si="4">IF(O16&lt;&gt;"Yes","",HYPERLINK(K16,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S16" s="32" t="str">
+        <x:f>IF(O16&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T16" s="38"/>
     </x:row>
     <x:row r="17" ht="30">
       <x:c r="A17" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B17),B17&lt;TODAY()),"DEADLINE PASSED",N17)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B17" s="3">
         <x:v>46336</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
-        <x:v>142</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D17" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="E17" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F17" s="2" t="s">
-        <x:v>144</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="G17" s="2" t="s">
-        <x:v>145</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H17" s="2" t="s">
-        <x:v>146</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="I17" s="2" t="s">
-        <x:v>147</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="J17" s="2" t="s">
-        <x:v>148</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="K17" s="2" t="s">
-        <x:v>149</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="L17" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M17" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N17" s="8"/>
-      <x:c r="O17" s="9" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M17" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N17" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O17" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P17" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q17" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R17" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S17" s="11"/>
+      <x:c r="P17" s="31" t="str">
+        <x:f t="shared" si="2">IF(O17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
+      </x:c>
+      <x:c r="Q17" s="32" t="str">
+        <x:f t="shared" si="3">IF(O17&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D17&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C17&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B17),TEXT(B17,"d mmmm yyyy"),B17)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F17&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G17&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I17&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R17" s="32" t="str">
+        <x:f t="shared" si="4">IF(O17&lt;&gt;"Yes","",HYPERLINK(K17,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S17" s="32" t="str">
+        <x:f>IF(O17&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T17" s="38"/>
     </x:row>
     <x:row r="18" ht="45">
       <x:c r="A18" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B18),B18&lt;TODAY()),"DEADLINE PASSED",N18)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B18" s="3">
         <x:v>46338</x:v>
       </x:c>
       <x:c r="C18" s="2" t="s">
-        <x:v>150</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D18" s="2" t="s">
-        <x:v>151</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E18" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F18" s="2" t="s">
-        <x:v>152</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="G18" s="2" t="s">
-        <x:v>153</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="H18" s="2" t="s">
-        <x:v>154</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="I18" s="2" t="s">
-        <x:v>155</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="J18" s="2" t="s">
-        <x:v>156</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="K18" s="2" t="s">
-        <x:v>157</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="L18" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M18" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N18" s="8"/>
-      <x:c r="O18" s="9" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M18" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N18" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O18" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P18" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q18" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R18" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S18" s="11"/>
+      <x:c r="P18" s="31" t="str">
+        <x:f t="shared" si="2">IF(O18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
+      </x:c>
+      <x:c r="Q18" s="32" t="str">
+        <x:f t="shared" si="3">IF(O18&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D18&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C18&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B18),TEXT(B18,"d mmmm yyyy"),B18)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F18&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G18&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I18&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R18" s="32" t="str">
+        <x:f t="shared" si="4">IF(O18&lt;&gt;"Yes","",HYPERLINK(K18,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S18" s="32" t="str">
+        <x:f>IF(O18&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T18" s="38"/>
     </x:row>
     <x:row r="19" ht="30">
       <x:c r="A19" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B19),B19&lt;TODAY()),"DEADLINE PASSED",N19)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B19" s="3">
         <x:v>46356</x:v>
       </x:c>
       <x:c r="C19" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D19" s="2" t="s">
-        <x:v>158</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E19" s="2" t="s">
-        <x:v>159</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="F19" s="2" t="s">
-        <x:v>160</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="G19" s="2" t="s">
-        <x:v>161</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="H19" s="2" t="s">
-        <x:v>162</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="I19" s="2" t="s">
-        <x:v>163</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="J19" s="2" t="s">
-        <x:v>164</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="K19" s="2" t="s">
-        <x:v>165</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="L19" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M19" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N19" s="8"/>
-      <x:c r="O19" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M19" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N19" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O19" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P19" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q19" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R19" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S19" s="11"/>
+      <x:c r="P19" s="31" t="str">
+        <x:f t="shared" si="2">IF(O19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
+      </x:c>
+      <x:c r="Q19" s="32" t="str">
+        <x:f t="shared" si="3">IF(O19&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D19&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C19&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B19),TEXT(B19,"d mmmm yyyy"),B19)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F19&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G19&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H19&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I19&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R19" s="32" t="str">
+        <x:f t="shared" si="4">IF(O19&lt;&gt;"Yes","",HYPERLINK(K19,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S19" s="32" t="str">
+        <x:f>IF(O19&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T19" s="38"/>
     </x:row>
     <x:row r="20" ht="45">
       <x:c r="A20" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B20),B20&lt;TODAY()),"DEADLINE PASSED",N20)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B20" s="3">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C20" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D20" s="2" t="s">
-        <x:v>166</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E20" s="2" t="s">
-        <x:v>167</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="F20" s="2" t="s">
-        <x:v>168</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="G20" s="2" t="s">
-        <x:v>169</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="H20" s="2" t="s">
-        <x:v>170</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="I20" s="2" t="s">
-        <x:v>171</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="J20" s="2" t="s">
-        <x:v>172</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="K20" s="2" t="s">
-        <x:v>173</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="L20" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M20" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N20" s="8"/>
-      <x:c r="O20" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M20" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N20" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O20" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P20" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q20" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R20" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S20" s="11"/>
+      <x:c r="P20" s="31" t="str">
+        <x:f t="shared" si="2">IF(O20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
+      </x:c>
+      <x:c r="Q20" s="32" t="str">
+        <x:f t="shared" si="3">IF(O20&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D20&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C20&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B20),TEXT(B20,"d mmmm yyyy"),B20)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F20&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G20&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H20&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I20&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R20" s="32" t="str">
+        <x:f t="shared" si="4">IF(O20&lt;&gt;"Yes","",HYPERLINK(K20,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S20" s="32" t="str">
+        <x:f>IF(O20&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T20" s="38"/>
     </x:row>
     <x:row r="21" ht="30">
       <x:c r="A21" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B21),B21&lt;TODAY()),"DEADLINE PASSED",N21)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B21" s="3">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C21" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D21" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="E21" s="2" t="s">
-        <x:v>175</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="F21" s="2" t="s">
-        <x:v>176</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="G21" s="2" t="s">
-        <x:v>177</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="H21" s="2" t="s">
-        <x:v>178</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="I21" s="2" t="s">
-        <x:v>179</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="J21" s="2" t="s">
-        <x:v>180</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="K21" s="2" t="s">
-        <x:v>173</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="L21" s="2" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="M21" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N21" s="8"/>
-      <x:c r="O21" s="9" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="M21" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N21" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O21" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P21" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q21" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R21" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S21" s="11"/>
+      <x:c r="P21" s="31" t="str">
+        <x:f t="shared" si="2">IF(O21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
+      </x:c>
+      <x:c r="Q21" s="32" t="str">
+        <x:f t="shared" si="3">IF(O21&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D21&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C21&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B21),TEXT(B21,"d mmmm yyyy"),B21)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F21&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G21&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H21&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I21&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R21" s="32" t="str">
+        <x:f t="shared" si="4">IF(O21&lt;&gt;"Yes","",HYPERLINK(K21,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S21" s="32" t="str">
+        <x:f>IF(O21&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T21" s="38"/>
     </x:row>
     <x:row r="22" ht="30">
       <x:c r="A22" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B22),B22&lt;TODAY()),"DEADLINE PASSED",N22)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B22" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C22" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D22" s="2" t="s">
-        <x:v>181</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E22" s="2" t="s">
-        <x:v>182</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F22" s="2" t="s">
-        <x:v>183</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G22" s="2" t="s">
-        <x:v>184</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="H22" s="2" t="s">
-        <x:v>185</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="I22" s="2" t="s">
-        <x:v>186</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="J22" s="2" t="s">
-        <x:v>187</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="K22" s="2" t="s">
-        <x:v>188</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="L22" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M22" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N22" s="8"/>
-      <x:c r="O22" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M22" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N22" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O22" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P22" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q22" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R22" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S22" s="11"/>
+      <x:c r="P22" s="31" t="str">
+        <x:f t="shared" si="2">IF(O22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
+      </x:c>
+      <x:c r="Q22" s="32" t="str">
+        <x:f t="shared" si="3">IF(O22&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D22&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C22&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B22),TEXT(B22,"d mmmm yyyy"),B22)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F22&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G22&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H22&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I22&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R22" s="32" t="str">
+        <x:f t="shared" si="4">IF(O22&lt;&gt;"Yes","",HYPERLINK(K22,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S22" s="32" t="str">
+        <x:f>IF(O22&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T22" s="38"/>
     </x:row>
     <x:row r="23" ht="30">
       <x:c r="A23" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B23),B23&lt;TODAY()),"DEADLINE PASSED",N23)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B23" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C23" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D23" s="2" t="s">
-        <x:v>189</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="E23" s="2" t="s">
-        <x:v>190</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="F23" s="2" t="s">
-        <x:v>191</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="G23" s="2" t="s">
-        <x:v>192</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="H23" s="2" t="s">
-        <x:v>193</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="I23" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="J23" s="2" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="K23" s="2" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="K23" s="2" t="s">
-        <x:v>195</x:v>
-      </x:c>
       <x:c r="L23" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M23" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N23" s="8"/>
-      <x:c r="O23" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M23" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N23" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O23" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P23" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q23" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R23" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S23" s="11"/>
+      <x:c r="P23" s="31" t="str">
+        <x:f t="shared" si="2">IF(O23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
+      </x:c>
+      <x:c r="Q23" s="32" t="str">
+        <x:f t="shared" si="3">IF(O23&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D23&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C23&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B23),TEXT(B23,"d mmmm yyyy"),B23)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F23&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G23&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I23&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R23" s="32" t="str">
+        <x:f t="shared" si="4">IF(O23&lt;&gt;"Yes","",HYPERLINK(K23,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S23" s="32" t="str">
+        <x:f>IF(O23&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T23" s="38"/>
     </x:row>
     <x:row r="24" ht="30">
       <x:c r="A24" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B24),B24&lt;TODAY()),"DEADLINE PASSED",N24)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B24" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C24" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D24" s="2" t="s">
-        <x:v>196</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="E24" s="2" t="s">
-        <x:v>197</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F24" s="2" t="s">
-        <x:v>198</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="G24" s="2" t="s">
-        <x:v>199</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="H24" s="2" t="s">
-        <x:v>200</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="I24" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J24" s="2" t="s">
-        <x:v>187</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="K24" s="2" t="s">
-        <x:v>201</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="L24" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M24" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N24" s="8"/>
-      <x:c r="O24" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M24" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N24" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O24" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P24" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q24" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R24" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S24" s="11"/>
+      <x:c r="P24" s="31" t="str">
+        <x:f t="shared" si="2">IF(O24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
+      </x:c>
+      <x:c r="Q24" s="32" t="str">
+        <x:f t="shared" si="3">IF(O24&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D24&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C24&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B24),TEXT(B24,"d mmmm yyyy"),B24)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F24&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G24&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I24&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R24" s="32" t="str">
+        <x:f t="shared" si="4">IF(O24&lt;&gt;"Yes","",HYPERLINK(K24,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S24" s="32" t="str">
+        <x:f>IF(O24&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T24" s="38"/>
     </x:row>
     <x:row r="25" ht="30">
       <x:c r="A25" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B25),B25&lt;TODAY()),"DEADLINE PASSED",N25)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B25" s="3">
         <x:v>46409</x:v>
       </x:c>
       <x:c r="C25" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D25" s="2" t="s">
-        <x:v>202</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E25" s="2" t="s">
-        <x:v>101</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F25" s="2" t="s">
-        <x:v>203</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G25" s="2" t="s">
-        <x:v>204</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="H25" s="2" t="s">
-        <x:v>205</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="I25" s="2" t="s">
-        <x:v>206</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="J25" s="2" t="s">
-        <x:v>187</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="K25" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L25" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M25" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N25" s="8"/>
-      <x:c r="O25" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M25" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N25" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O25" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P25" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q25" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R25" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S25" s="11"/>
+      <x:c r="P25" s="31" t="str">
+        <x:f t="shared" si="2">IF(O25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
+      </x:c>
+      <x:c r="Q25" s="32" t="str">
+        <x:f t="shared" si="3">IF(O25&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D25&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C25&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B25),TEXT(B25,"d mmmm yyyy"),B25)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F25&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G25&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H25&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I25&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R25" s="32" t="str">
+        <x:f t="shared" si="4">IF(O25&lt;&gt;"Yes","",HYPERLINK(K25,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S25" s="32" t="str">
+        <x:f>IF(O25&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T25" s="38"/>
     </x:row>
     <x:row r="26" ht="30">
       <x:c r="A26" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B26),B26&lt;TODAY()),"DEADLINE PASSED",N26)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B26" s="3">
         <x:v>46418</x:v>
       </x:c>
       <x:c r="C26" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D26" s="2" t="s">
-        <x:v>207</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="E26" s="2" t="s">
-        <x:v>208</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="F26" s="2" t="s">
-        <x:v>209</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G26" s="2" t="s">
-        <x:v>210</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H26" s="2" t="s">
-        <x:v>211</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="I26" s="2" t="s">
-        <x:v>206</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="J26" s="2" t="s">
-        <x:v>212</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="K26" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L26" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M26" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N26" s="8"/>
-      <x:c r="O26" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M26" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N26" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O26" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P26" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q26" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R26" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S26" s="11"/>
+      <x:c r="P26" s="31" t="str">
+        <x:f t="shared" si="2">IF(O26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
+      </x:c>
+      <x:c r="Q26" s="32" t="str">
+        <x:f t="shared" si="3">IF(O26&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D26&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C26&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B26),TEXT(B26,"d mmmm yyyy"),B26)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F26&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G26&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I26&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R26" s="32" t="str">
+        <x:f t="shared" si="4">IF(O26&lt;&gt;"Yes","",HYPERLINK(K26,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S26" s="32" t="str">
+        <x:f>IF(O26&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T26" s="38"/>
     </x:row>
     <x:row r="27" ht="30">
       <x:c r="A27" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B27),B27&lt;TODAY()),"DEADLINE PASSED",N27)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B27" s="3">
         <x:v>46419</x:v>
       </x:c>
       <x:c r="C27" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D27" s="2" t="s">
-        <x:v>213</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="E27" s="2" t="s">
-        <x:v>214</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="F27" s="2" t="s">
-        <x:v>215</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="G27" s="2" t="s">
-        <x:v>216</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="H27" s="2" t="s">
-        <x:v>217</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="I27" s="2" t="s">
-        <x:v>218</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="J27" s="2" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="K27" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L27" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M27" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N27" s="8"/>
-      <x:c r="O27" s="9" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M27" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N27" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O27" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P27" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q27" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R27" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S27" s="11"/>
+      <x:c r="P27" s="31" t="str">
+        <x:f t="shared" si="2">IF(O27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
+      </x:c>
+      <x:c r="Q27" s="32" t="str">
+        <x:f t="shared" si="3">IF(O27&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D27&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C27&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B27),TEXT(B27,"d mmmm yyyy"),B27)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F27&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G27&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I27&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R27" s="32" t="str">
+        <x:f t="shared" si="4">IF(O27&lt;&gt;"Yes","",HYPERLINK(K27,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S27" s="32" t="str">
+        <x:f>IF(O27&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T27" s="38"/>
     </x:row>
     <x:row r="28" ht="45">
       <x:c r="A28" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B28),B28&lt;TODAY()),"DEADLINE PASSED",N28)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="G28" s="2" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="H28" s="2" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="I28" s="2" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="J28" s="2" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="C28" s="2" t="s">
+      <x:c r="K28" s="2" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="D28" s="2" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="E28" s="2" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="F28" s="2" t="s">
-        <x:v>224</x:v>
-      </x:c>
-      <x:c r="G28" s="2" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="H28" s="2" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="I28" s="2" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="J28" s="2" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="K28" s="2" t="s">
-        <x:v>229</x:v>
-      </x:c>
       <x:c r="L28" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M28" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N28" s="8"/>
-      <x:c r="O28" s="9" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M28" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N28" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O28" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P28" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q28" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R28" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S28" s="11"/>
+      <x:c r="P28" s="31" t="str">
+        <x:f t="shared" si="2">IF(O28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
+      </x:c>
+      <x:c r="Q28" s="32" t="str">
+        <x:f t="shared" si="3">IF(O28&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D28&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C28&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B28),TEXT(B28,"d mmmm yyyy"),B28)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F28&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G28&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I28&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R28" s="32" t="str">
+        <x:f t="shared" si="4">IF(O28&lt;&gt;"Yes","",HYPERLINK(K28,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S28" s="32" t="str">
+        <x:f>IF(O28&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T28" s="38"/>
     </x:row>
     <x:row r="29" ht="45">
       <x:c r="A29" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B29),B29&lt;TODAY()),"DEADLINE PASSED",N29)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C29" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G29" s="2" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="H29" s="2" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="I29" s="2" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="J29" s="2" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="K29" s="2" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="L29" s="2" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="D29" s="2" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="E29" s="2" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="F29" s="2" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="G29" s="2" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="H29" s="2" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="I29" s="2" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="J29" s="2" t="s">
-        <x:v>236</x:v>
-      </x:c>
-      <x:c r="K29" s="2" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="L29" s="2" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="M29" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N29" s="8"/>
-      <x:c r="O29" s="9" t="str">
+      <x:c r="M29" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N29" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O29" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P29" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q29" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R29" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S29" s="11"/>
+      <x:c r="P29" s="31" t="str">
+        <x:f t="shared" si="2">IF(O29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
+      </x:c>
+      <x:c r="Q29" s="32" t="str">
+        <x:f t="shared" si="3">IF(O29&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D29&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C29&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B29),TEXT(B29,"d mmmm yyyy"),B29)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F29&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G29&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I29&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R29" s="32" t="str">
+        <x:f t="shared" si="4">IF(O29&lt;&gt;"Yes","",HYPERLINK(K29,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S29" s="32" t="str">
+        <x:f>IF(O29&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T29" s="38"/>
     </x:row>
     <x:row r="30" ht="30">
       <x:c r="A30" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B30),B30&lt;TODAY()),"DEADLINE PASSED",N30)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C30" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="G30" s="2" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="H30" s="2" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="I30" s="2" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="J30" s="2" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="K30" s="2" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="L30" s="2" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="D30" s="2" t="s">
-        <x:v>239</x:v>
-      </x:c>
-      <x:c r="E30" s="2" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="F30" s="2" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="G30" s="2" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="H30" s="2" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="I30" s="2" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="J30" s="2" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="K30" s="2" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="L30" s="2" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="M30" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N30" s="8"/>
-      <x:c r="O30" s="9" t="str">
+      <x:c r="M30" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N30" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O30" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P30" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q30" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R30" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S30" s="11"/>
+      <x:c r="P30" s="31" t="str">
+        <x:f t="shared" si="2">IF(O30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
+      </x:c>
+      <x:c r="Q30" s="32" t="str">
+        <x:f t="shared" si="3">IF(O30&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D30&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C30&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B30),TEXT(B30,"d mmmm yyyy"),B30)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F30&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G30&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I30&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R30" s="32" t="str">
+        <x:f t="shared" si="4">IF(O30&lt;&gt;"Yes","",HYPERLINK(K30,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S30" s="32" t="str">
+        <x:f>IF(O30&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T30" s="38"/>
     </x:row>
     <x:row r="31" ht="30">
       <x:c r="A31" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B31),B31&lt;TODAY()),"DEADLINE PASSED",N31)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C31" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="G31" s="2" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="H31" s="2" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="I31" s="2" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="J31" s="2" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="K31" s="2" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="L31" s="2" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="D31" s="2" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="E31" s="2" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="F31" s="2" t="s">
-        <x:v>248</x:v>
-      </x:c>
-      <x:c r="G31" s="2" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="H31" s="2" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="I31" s="2" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="J31" s="2" t="s">
-        <x:v>236</x:v>
-      </x:c>
-      <x:c r="K31" s="2" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="L31" s="2" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="M31" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N31" s="8"/>
-      <x:c r="O31" s="9" t="str">
+      <x:c r="M31" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N31" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O31" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P31" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q31" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R31" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S31" s="11"/>
+      <x:c r="P31" s="31" t="str">
+        <x:f t="shared" si="2">IF(O31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
+      </x:c>
+      <x:c r="Q31" s="32" t="str">
+        <x:f t="shared" si="3">IF(O31&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D31&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C31&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B31),TEXT(B31,"d mmmm yyyy"),B31)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F31&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G31&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H31&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I31&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R31" s="32" t="str">
+        <x:f t="shared" si="4">IF(O31&lt;&gt;"Yes","",HYPERLINK(K31,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S31" s="32" t="str">
+        <x:f>IF(O31&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T31" s="38"/>
     </x:row>
     <x:row r="32" ht="45">
       <x:c r="A32" s="19" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B32),B32&lt;TODAY()),"DEADLINE PASSED",N32)</x:f>
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C32" s="2" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="G32" s="2" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="H32" s="2" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="I32" s="2" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="J32" s="2" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="K32" s="2" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="L32" s="2" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="D32" s="2" t="s">
-        <x:v>252</x:v>
-      </x:c>
-      <x:c r="E32" s="2" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F32" s="2" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="G32" s="2" t="s">
-        <x:v>254</x:v>
-      </x:c>
-      <x:c r="H32" s="2" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="I32" s="2" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="J32" s="2" t="s">
-        <x:v>256</x:v>
-      </x:c>
-      <x:c r="K32" s="2" t="s">
-        <x:v>257</x:v>
-      </x:c>
-      <x:c r="L32" s="2" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="M32" s="8" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="N32" s="8"/>
-      <x:c r="O32" s="9" t="str">
+      <x:c r="M32" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N32" s="23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="O32" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P32" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q32" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R32" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S32" s="11"/>
+      <x:c r="P32" s="31" t="str">
+        <x:f t="shared" si="2">IF(O32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
+      </x:c>
+      <x:c r="Q32" s="32" t="str">
+        <x:f t="shared" si="3">IF(O32&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D32&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C32&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B32),TEXT(B32,"d mmmm yyyy"),B32)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F32&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G32&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H32&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I32&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R32" s="32" t="str">
+        <x:f t="shared" si="4">IF(O32&lt;&gt;"Yes","",HYPERLINK(K32,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S32" s="32" t="str">
+        <x:f>IF(O32&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T32" s="38"/>
     </x:row>
     <x:row r="33" ht="60">
       <x:c r="A33" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B33),B33&lt;TODAY()),"DEADLINE PASSED",N33)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="G33" s="2" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="H33" s="2" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="I33" s="2" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="J33" s="2" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="K33" s="2" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="L33" s="2" t="s">
         <x:v>258</x:v>
       </x:c>
-      <x:c r="C33" s="2" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="D33" s="2" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="E33" s="2" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="F33" s="2" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="G33" s="2" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="H33" s="2" t="s">
-        <x:v>262</x:v>
-      </x:c>
-      <x:c r="I33" s="2" t="s">
-        <x:v>263</x:v>
-      </x:c>
-      <x:c r="J33" s="2" t="s">
-        <x:v>264</x:v>
-      </x:c>
-      <x:c r="K33" s="2" t="s">
-        <x:v>265</x:v>
-      </x:c>
-      <x:c r="L33" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M33" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N33" s="8"/>
-      <x:c r="O33" s="9" t="str">
+      <x:c r="M33" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N33" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O33" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P33" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q33" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R33" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S33" s="11"/>
+      <x:c r="P33" s="31" t="str">
+        <x:f t="shared" si="2">IF(O33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
+      </x:c>
+      <x:c r="Q33" s="32" t="str">
+        <x:f t="shared" si="3">IF(O33&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D33&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C33&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B33),TEXT(B33,"d mmmm yyyy"),B33)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F33&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G33&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H33&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I33&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R33" s="32" t="str">
+        <x:f t="shared" si="4">IF(O33&lt;&gt;"Yes","",HYPERLINK(K33,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S33" s="32" t="str">
+        <x:f>IF(O33&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T33" s="38"/>
     </x:row>
     <x:row r="34" ht="45">
       <x:c r="A34" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B34),B34&lt;TODAY()),"DEADLINE PASSED",N34)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
-        <x:v>268</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="C34" s="2" t="s">
-        <x:v>269</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D34" s="2" t="s">
-        <x:v>270</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="E34" s="2" t="s">
-        <x:v>271</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="F34" s="2" t="s">
-        <x:v>272</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="G34" s="2" t="s">
-        <x:v>273</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="H34" s="2" t="s">
-        <x:v>274</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="I34" s="2" t="s">
-        <x:v>275</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="J34" s="2" t="s">
-        <x:v>276</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="K34" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L34" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M34" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N34" s="8"/>
-      <x:c r="O34" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M34" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N34" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O34" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P34" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q34" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R34" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S34" s="11"/>
+      <x:c r="P34" s="31" t="str">
+        <x:f t="shared" si="2">IF(O34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
+      </x:c>
+      <x:c r="Q34" s="32" t="str">
+        <x:f t="shared" si="3">IF(O34&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D34&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C34&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B34),TEXT(B34,"d mmmm yyyy"),B34)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F34&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G34&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H34&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I34&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R34" s="32" t="str">
+        <x:f t="shared" si="4">IF(O34&lt;&gt;"Yes","",HYPERLINK(K34,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S34" s="32" t="str">
+        <x:f>IF(O34&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T34" s="38"/>
     </x:row>
     <x:row r="35" ht="30">
       <x:c r="A35" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B35),B35&lt;TODAY()),"DEADLINE PASSED",N35)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="C35" s="2" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="D35" s="2" t="s">
-        <x:v>277</x:v>
-      </x:c>
       <x:c r="E35" s="2" t="s">
-        <x:v>278</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="F35" s="2" t="s">
-        <x:v>279</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="G35" s="2" t="s">
-        <x:v>280</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="H35" s="2" t="s">
-        <x:v>281</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="I35" s="2" t="s">
-        <x:v>282</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="J35" s="2" t="s">
-        <x:v>283</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="K35" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L35" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M35" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N35" s="8"/>
-      <x:c r="O35" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M35" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N35" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O35" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P35" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q35" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R35" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S35" s="11"/>
+      <x:c r="P35" s="31" t="str">
+        <x:f t="shared" si="2">IF(O35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
+      </x:c>
+      <x:c r="Q35" s="32" t="str">
+        <x:f t="shared" si="3">IF(O35&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D35&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C35&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B35),TEXT(B35,"d mmmm yyyy"),B35)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F35&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G35&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H35&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I35&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R35" s="32" t="str">
+        <x:f t="shared" si="4">IF(O35&lt;&gt;"Yes","",HYPERLINK(K35,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S35" s="32" t="str">
+        <x:f>IF(O35&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T35" s="38"/>
     </x:row>
     <x:row r="36" ht="30">
       <x:c r="A36" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B36),B36&lt;TODAY()),"DEADLINE PASSED",N36)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
-        <x:v>284</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="C36" s="2" t="s">
-        <x:v>142</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D36" s="2" t="s">
-        <x:v>285</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="E36" s="2" t="s">
-        <x:v>286</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="F36" s="2" t="s">
-        <x:v>287</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="G36" s="2" t="s">
-        <x:v>288</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="H36" s="2" t="s">
-        <x:v>289</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="I36" s="2" t="s">
-        <x:v>290</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="J36" s="2" t="s">
-        <x:v>291</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="K36" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L36" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M36" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N36" s="8"/>
-      <x:c r="O36" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M36" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N36" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O36" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P36" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q36" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R36" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S36" s="11"/>
+      <x:c r="P36" s="31" t="str">
+        <x:f t="shared" si="2">IF(O36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
+      </x:c>
+      <x:c r="Q36" s="32" t="str">
+        <x:f t="shared" si="3">IF(O36&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D36&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C36&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B36),TEXT(B36,"d mmmm yyyy"),B36)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F36&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G36&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H36&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I36&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R36" s="32" t="str">
+        <x:f t="shared" si="4">IF(O36&lt;&gt;"Yes","",HYPERLINK(K36,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S36" s="32" t="str">
+        <x:f>IF(O36&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T36" s="38"/>
     </x:row>
     <x:row r="37" ht="30">
       <x:c r="A37" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B37),B37&lt;TODAY()),"DEADLINE PASSED",N37)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="C37" s="2" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="D37" s="2" t="s">
-        <x:v>293</x:v>
-      </x:c>
       <x:c r="E37" s="2" t="s">
-        <x:v>294</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="F37" s="2" t="s">
-        <x:v>295</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="G37" s="2" t="s">
-        <x:v>296</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="H37" s="2" t="s">
-        <x:v>297</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="I37" s="2" t="s">
-        <x:v>298</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="J37" s="2" t="s">
-        <x:v>299</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="K37" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L37" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M37" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N37" s="8"/>
-      <x:c r="O37" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M37" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N37" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O37" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P37" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q37" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R37" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S37" s="11"/>
+      <x:c r="P37" s="31" t="str">
+        <x:f t="shared" si="2">IF(O37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
+      </x:c>
+      <x:c r="Q37" s="32" t="str">
+        <x:f t="shared" si="3">IF(O37&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D37&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C37&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B37),TEXT(B37,"d mmmm yyyy"),B37)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F37&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G37&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H37&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I37&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R37" s="32" t="str">
+        <x:f t="shared" si="4">IF(O37&lt;&gt;"Yes","",HYPERLINK(K37,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S37" s="32" t="str">
+        <x:f>IF(O37&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T37" s="38"/>
     </x:row>
     <x:row r="38" ht="30">
       <x:c r="A38" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B38),B38&lt;TODAY()),"DEADLINE PASSED",N38)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
-        <x:v>300</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C38" s="2" t="s">
-        <x:v>142</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D38" s="2" t="s">
-        <x:v>301</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="E38" s="2" t="s">
-        <x:v>302</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="F38" s="2" t="s">
-        <x:v>303</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="G38" s="2" t="s">
-        <x:v>304</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="H38" s="2" t="s">
-        <x:v>305</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="I38" s="2" t="s">
-        <x:v>306</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="J38" s="2" t="s">
-        <x:v>307</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="K38" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L38" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M38" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N38" s="8"/>
-      <x:c r="O38" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M38" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N38" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O38" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P38" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q38" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R38" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S38" s="11"/>
+      <x:c r="P38" s="31" t="str">
+        <x:f t="shared" si="2">IF(O38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
+      </x:c>
+      <x:c r="Q38" s="32" t="str">
+        <x:f t="shared" si="3">IF(O38&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D38&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C38&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B38),TEXT(B38,"d mmmm yyyy"),B38)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F38&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G38&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H38&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I38&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R38" s="32" t="str">
+        <x:f t="shared" si="4">IF(O38&lt;&gt;"Yes","",HYPERLINK(K38,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S38" s="32" t="str">
+        <x:f>IF(O38&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T38" s="38"/>
     </x:row>
     <x:row r="39" ht="30">
       <x:c r="A39" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B39),B39&lt;TODAY()),"DEADLINE PASSED",N39)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D39" s="2" t="s">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="E39" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F39" s="2" t="s">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="C39" s="2" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="D39" s="2" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="E39" s="2" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F39" s="2" t="s">
-        <x:v>309</x:v>
-      </x:c>
       <x:c r="G39" s="2" t="s">
-        <x:v>310</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="H39" s="2" t="s">
-        <x:v>311</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="I39" s="2" t="s">
-        <x:v>312</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="J39" s="2" t="s">
-        <x:v>313</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="K39" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L39" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M39" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N39" s="8"/>
-      <x:c r="O39" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M39" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N39" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O39" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P39" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q39" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R39" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S39" s="11"/>
+      <x:c r="P39" s="31" t="str">
+        <x:f t="shared" si="2">IF(O39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
+      </x:c>
+      <x:c r="Q39" s="32" t="str">
+        <x:f t="shared" si="3">IF(O39&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D39&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C39&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B39),TEXT(B39,"d mmmm yyyy"),B39)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F39&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G39&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H39&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I39&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R39" s="32" t="str">
+        <x:f t="shared" si="4">IF(O39&lt;&gt;"Yes","",HYPERLINK(K39,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S39" s="32" t="str">
+        <x:f>IF(O39&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T39" s="38"/>
     </x:row>
     <x:row r="40" ht="30">
       <x:c r="A40" s="22" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B40),B40&lt;TODAY()),"DEADLINE PASSED",N40)</x:f>
         <x:v>FORTHCOMING</x:v>
       </x:c>
       <x:c r="B40" s="3" t="s">
-        <x:v>314</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="C40" s="2" t="s">
-        <x:v>142</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D40" s="2" t="s">
-        <x:v>315</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="E40" s="2" t="s">
-        <x:v>40</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F40" s="2" t="s">
-        <x:v>316</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="G40" s="2" t="s">
-        <x:v>317</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="H40" s="2" t="s">
-        <x:v>318</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="I40" s="2" t="s">
-        <x:v>319</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="J40" s="2" t="s">
-        <x:v>320</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="K40" s="2" t="s">
-        <x:v>265</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="L40" s="2" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="M40" s="8" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="N40" s="8"/>
-      <x:c r="O40" s="9" t="str">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="M40" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N40" s="23" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O40" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P40" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q40" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R40" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S40" s="11"/>
+      <x:c r="P40" s="31" t="str">
+        <x:f t="shared" si="2">IF(O40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
+      </x:c>
+      <x:c r="Q40" s="32" t="str">
+        <x:f t="shared" si="3">IF(O40&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D40&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C40&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B40),TEXT(B40,"d mmmm yyyy"),B40)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F40&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G40&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H40&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I40&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R40" s="32" t="str">
+        <x:f t="shared" si="4">IF(O40&lt;&gt;"Yes","",HYPERLINK(K40,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S40" s="32" t="str">
+        <x:f>IF(O40&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T40" s="38"/>
     </x:row>
     <x:row r="41" ht="45">
       <x:c r="A41" s="16" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B41),B41&lt;TODAY()),"DEADLINE PASSED",N41)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B41" s="3">
         <x:v>46283</x:v>
       </x:c>
       <x:c r="C41" s="2" t="s">
-        <x:v>321</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D41" s="2" t="s">
-        <x:v>322</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="E41" s="2" t="s">
-        <x:v>323</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="F41" s="2" t="s">
-        <x:v>324</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="G41" s="2" t="s">
-        <x:v>325</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="H41" s="2" t="s">
-        <x:v>326</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="I41" s="2" t="s">
-        <x:v>327</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="J41" s="2" t="s">
-        <x:v>328</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="K41" s="2" t="s">
-        <x:v>329</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="L41" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M41" s="8" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="N41" s="8"/>
-      <x:c r="O41" s="9" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M41" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N41" s="23" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="O41" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P41" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q41" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R41" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S41" s="11"/>
+      <x:c r="P41" s="31" t="str">
+        <x:f t="shared" si="2">IF(O41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
+      </x:c>
+      <x:c r="Q41" s="32" t="str">
+        <x:f t="shared" si="3">IF(O41&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D41&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C41&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B41),TEXT(B41,"d mmmm yyyy"),B41)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F41&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G41&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H41&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I41&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R41" s="32" t="str">
+        <x:f t="shared" si="4">IF(O41&lt;&gt;"Yes","",HYPERLINK(K41,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S41" s="32" t="str">
+        <x:f>IF(O41&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T41" s="38"/>
     </x:row>
     <x:row r="42" ht="45">
       <x:c r="A42" s="16" t="str">
-        <x:f t="shared" ca="1" si="0"/>
+        <x:f t="shared" ca="1" si="0">IF(AND(ISNUMBER(B42),B42&lt;TODAY()),"DEADLINE PASSED",N42)</x:f>
         <x:v>DEADLINE PASSED</x:v>
       </x:c>
       <x:c r="B42" s="3">
         <x:v>46286</x:v>
       </x:c>
       <x:c r="C42" s="2" t="s">
-        <x:v>331</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D42" s="2" t="s">
-        <x:v>332</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E42" s="2" t="s">
-        <x:v>333</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F42" s="2" t="s">
-        <x:v>334</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="G42" s="2" t="s">
-        <x:v>335</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="H42" s="2" t="s">
-        <x:v>336</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="I42" s="2" t="s">
-        <x:v>337</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="J42" s="2" t="s">
-        <x:v>338</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="K42" s="2" t="s">
-        <x:v>339</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="L42" s="2" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="M42" s="8" t="s">
-        <x:v>340</x:v>
-      </x:c>
-      <x:c r="N42" s="8"/>
-      <x:c r="O42" s="9" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="M42" s="23" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="N42" s="23" t="str">
+        <x:v>CLOSED – invited stage continues</x:v>
+      </x:c>
+      <x:c r="O42" s="23">
         <x:f t="shared" si="1"/>
       </x:c>
-      <x:c r="P42" s="9" t="str">
-        <x:f t="shared" si="2"/>
-      </x:c>
-      <x:c r="Q42" s="10" t="str">
-        <x:f t="shared" si="3"/>
-      </x:c>
-      <x:c r="R42" s="10" t="str">
-        <x:f t="shared" si="4"/>
-      </x:c>
-      <x:c r="S42" s="11"/>
+      <x:c r="P42" s="31" t="str">
+        <x:f t="shared" si="2">IF(O42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
+      </x:c>
+      <x:c r="Q42" s="32" t="str">
+        <x:f t="shared" si="3">IF(O42&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D42&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C42&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B42),TEXT(B42,"d mmmm yyyy"),B42)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F42&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G42&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H42&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I42&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R42" s="32" t="str">
+        <x:f t="shared" si="4">IF(O42&lt;&gt;"Yes","",HYPERLINK(K42,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S42" s="32" t="str">
+        <x:f>IF(O42&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T42" s="38"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
-    <x:cfRule type="expression" dxfId="1" priority="1">
+    <x:cfRule type="expression" dxfId="5" priority="1">
       <x:formula>$A2="OPEN"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="2" priority="2">
+    <x:cfRule type="expression" dxfId="6" priority="2">
       <x:formula>$A2="FORTHCOMING"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="3" priority="3">
+    <x:cfRule type="expression" dxfId="7" priority="3">
       <x:formula>LEFT($A2,6)="CLOSED"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="4" priority="4">
+    <x:cfRule type="expression" dxfId="8" priority="4">
       <x:formula>$A2="DEADLINE PASSED"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="M2:M500">
+      <x:formula1>"Research,Scholarship,Research and Scholarship"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N2:N500">
       <x:formula1>"OPEN,FORTHCOMING,CLOSED – monitor recurrence,CLOSED – invited stage continues"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="N2:N500">
+    <x:dataValidation type="list" sqref="O2:O500">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c41408dbb064834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d4c24f27d7e4920"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4051,192 +4364,200 @@
   <x:sheetData>
     <x:row r="1" ht="21">
       <x:c r="A1" s="14" t="s">
-        <x:v>341</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
     </x:row>
     <x:row r="2" ht="30">
       <x:c r="A2" s="4" t="s">
-        <x:v>342</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>343</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="16">
       <x:c r="A3" s="4" t="s">
-        <x:v>344</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>345</x:v>
+        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45">
       <x:c r="A4" s="4" t="s">
-        <x:v>346</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>347</x:v>
+        <x:v>336</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45">
       <x:c r="A5" s="4" t="s">
-        <x:v>348</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>349</x:v>
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32">
       <x:c r="A6" s="4" t="s">
-        <x:v>350</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>351</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30">
       <x:c r="A7" s="4" t="s">
-        <x:v>352</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>353</x:v>
+        <x:v>342</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>355</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>356</x:v>
+        <x:v>345</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>222</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>357</x:v>
+        <x:v>346</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>358</x:v>
+        <x:v>347</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B13" s="2" t="s">
-        <x:v>359</x:v>
+        <x:v>348</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B14" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B15" s="2" t="s">
-        <x:v>360</x:v>
+        <x:v>349</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="16">
       <x:c r="A16" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B16" s="2" t="s">
-        <x:v>332</x:v>
+        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="16">
       <x:c r="A17" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B17" s="2" t="s">
-        <x:v>124</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="16">
       <x:c r="A18" s="4" t="s">
-        <x:v>354</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B18" s="2" t="s">
-        <x:v>151</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="45">
       <x:c r="A19" s="4" t="s">
-        <x:v>361</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="B19" s="2" t="s">
-        <x:v>362</x:v>
+        <x:v>351</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47" t="str">
+        <x:v>Research / Scholarship</x:v>
+      </x:c>
+      <x:c r="B20" s="50" t="str">
+        <x:v>Use Research for research funding, research career development, research events, visits and impact activity. Use Scholarship for teaching, learning or educational-development opportunities. Use Research and Scholarship when both apply.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42.75" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>363</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
-        <x:v>364</x:v>
+        <x:v>353</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15">
       <x:c r="A22" s="7" t="s">
-        <x:v>365</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>366</x:v>
+        <x:v>355</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15">
       <x:c r="A23" s="7" t="s">
-        <x:v>367</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>368</x:v>
+        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30">
       <x:c r="A24" s="7" t="s">
-        <x:v>369</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>370</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15">
       <x:c r="A25" s="7" t="s">
-        <x:v>371</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>372</x:v>
+        <x:v>361</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add scholarship funding opportunities
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R19e92bb378c240d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R792b31c736944b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R30c2fb5e73db4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R1a13069f9ac04b15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1011,9 +1011,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Last reviewed</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">29 September 2026</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Curation rule</x:t>
@@ -1105,7 +1102,7 @@
     <x:numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
     <x:numFmt numFmtId="200" formatCode="dd mmm yyyy"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1178,8 +1175,14 @@
       <x:color rgb="FF7F6000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF595959"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1261,6 +1264,21 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -1268,7 +1286,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1404,11 +1422,87 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="9">
+  <x:dxfs count="13">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF990000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF38761D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF595959"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1513,8 +1607,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:T42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:T42"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:T49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:T49"/>
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Deadline"/>
@@ -1864,7 +1958,7 @@
       <x:c r="N2" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O2" s="23">
+      <x:c r="O2" s="23" t="str">
         <x:f t="shared" ref="O2:O42" si="1">IF(N2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
       </x:c>
       <x:c r="P2" s="31" t="str">
@@ -4320,6 +4414,419 @@
         <x:f>IF(O42&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
       </x:c>
       <x:c r="T42" s="38"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="64" t="str">
+        <x:f>IF(AND(ISNUMBER(B43),B43&lt;TODAY()),"DEADLINE PASSED",N43)</x:f>
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>Next call TBC</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>University of Glasgow</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>Scholarship of Teaching &amp; Learning (SoTL) Fund</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>Teaching and learning scholarship</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>Amount and terms available on the UofG staff sign-in page</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>University of Glasgow staff; check the internal call for full eligibility</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>Strong fit for evaluating statistics teaching, assessment, student learning and evidence-based educational change.</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>Scholarship; teaching; learning; assessment; evaluation</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>The 2026 call opened on 5 January 2026. Check the internal funding page or L&amp;T newsletter for the next round.</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>https://www.gla.ac.uk/myglasgow/learningandteaching/staff-support/funding/</x:v>
+      </x:c>
+      <x:c r="L43" t="str">
+        <x:v>UofG Learning &amp; Teaching</x:v>
+      </x:c>
+      <x:c r="M43" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N43" s="54" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="O43" s="54"/>
+      <x:c r="P43" s="58" t="str">
+        <x:f>IF(O43&lt;&gt;"Yes","","New funding opportunity added: "&amp;D43)</x:f>
+      </x:c>
+      <x:c r="Q43" s="58" t="str">
+        <x:f>IF(O43&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D43&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C43&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B43),TEXT(B43,"d mmmm yyyy"),B43)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F43&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G43&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H43&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I43&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R43" s="58" t="str">
+        <x:f>IF(O43&lt;&gt;"Yes","",HYPERLINK(K43,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S43" s="58" t="str">
+        <x:f>IF(O43&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T43" s="61"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="64" t="str">
+        <x:f>IF(AND(ISNUMBER(B44),B44&lt;TODAY()),"DEADLINE PASSED",N44)</x:f>
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>Next call TBC</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>University of Glasgow</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>Learning &amp; Teaching Development Fund (LTDF)</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>Teaching development</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>Amount and terms available on the UofG staff sign-in page</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>All University of Glasgow staff may bid; check the internal call for full terms</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>Relevant for developing and evaluating innovative Statistics teaching, curricula, assessment and inclusive learning practice.</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>Scholarship; teaching; curriculum; assessment; innovation</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>The 2026 call opened on 5 January 2026. Check the internal funding page or L&amp;T newsletter for the next round.</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>https://www.gla.ac.uk/myglasgow/learningandteaching/staff-support/funding/</x:v>
+      </x:c>
+      <x:c r="L44" t="str">
+        <x:v>UofG Learning &amp; Teaching</x:v>
+      </x:c>
+      <x:c r="M44" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N44" s="54" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="O44" s="54"/>
+      <x:c r="P44" s="58" t="str">
+        <x:f>IF(O44&lt;&gt;"Yes","","New funding opportunity added: "&amp;D44)</x:f>
+      </x:c>
+      <x:c r="Q44" s="58" t="str">
+        <x:f>IF(O44&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D44&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C44&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B44),TEXT(B44,"d mmmm yyyy"),B44)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F44&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G44&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H44&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I44&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R44" s="58" t="str">
+        <x:f>IF(O44&lt;&gt;"Yes","",HYPERLINK(K44,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S44" s="58" t="str">
+        <x:f>IF(O44&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T44" s="61"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="64" t="str">
+        <x:f>IF(AND(ISNUMBER(B45),B45&lt;TODAY()),"DEADLINE PASSED",N45)</x:f>
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>Check internal call</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>University of Glasgow</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>Student–Staff Partnership Schemes (SSPS)</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Student–staff partnership</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>Funding and terms available on the UofG staff sign-in page</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>University of Glasgow staff and students working in partnership; check the internal scheme details</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>Suitable for co-created Statistics projects on curriculum, assessment, belonging, student experience or quantitative learning support.</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>Scholarship; students as partners; co-creation; student experience</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>Monitor the internal Learning &amp; Teaching funding page for the next available scheme and deadlines.</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>https://www.gla.ac.uk/myglasgow/learningandteaching/staff-support/funding/</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>UofG Learning &amp; Teaching</x:v>
+      </x:c>
+      <x:c r="M45" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N45" s="54" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="O45" s="54"/>
+      <x:c r="P45" s="58" t="str">
+        <x:f>IF(O45&lt;&gt;"Yes","","New funding opportunity added: "&amp;D45)</x:f>
+      </x:c>
+      <x:c r="Q45" s="58" t="str">
+        <x:f>IF(O45&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D45&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C45&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B45),TEXT(B45,"d mmmm yyyy"),B45)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F45&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G45&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H45&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I45&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R45" s="58" t="str">
+        <x:f>IF(O45&lt;&gt;"Yes","",HYPERLINK(K45,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S45" s="58" t="str">
+        <x:f>IF(O45&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T45" s="61"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="66" t="str">
+        <x:f>IF(AND(ISNUMBER(B46),B46&lt;TODAY()),"DEADLINE PASSED",N46)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>TBC – next academic year</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>London Mathematical Society</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>Single-Institution Teaching &amp; Scholarship Project Grants</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>Teaching and scholarship project</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>Up to £2,000; project delivered in the academic year following the award</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>UK mathematical scientists building a teaching and scholarship profile; single-university team; lead below Associate Professor/Reader/Professor level; PhD students ineligible</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>Excellent fit for a Statistics education project on teaching quality, curriculum, assessment, student experience or outcomes at Glasgow.</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>Scholarship; mathematics education; curriculum; student success; evaluation</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>Latest round closed; LMS states that a new call will take place in the next academic year. Monitor the scheme page.</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>https://www.lms.ac.uk/grants/single-teaching-scholarship</x:v>
+      </x:c>
+      <x:c r="L46" t="str">
+        <x:v>LMS</x:v>
+      </x:c>
+      <x:c r="M46" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N46" s="54" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O46" s="54"/>
+      <x:c r="P46" s="58" t="str">
+        <x:f>IF(O46&lt;&gt;"Yes","","New funding opportunity added: "&amp;D46)</x:f>
+      </x:c>
+      <x:c r="Q46" s="58" t="str">
+        <x:f>IF(O46&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D46&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C46&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B46),TEXT(B46,"d mmmm yyyy"),B46)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F46&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G46&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H46&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I46&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R46" s="58" t="str">
+        <x:f>IF(O46&lt;&gt;"Yes","",HYPERLINK(K46,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S46" s="58" t="str">
+        <x:f>IF(O46&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T46" s="61"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="66" t="str">
+        <x:f>IF(AND(ISNUMBER(B47),B47&lt;TODAY()),"DEADLINE PASSED",N47)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>TBC – next academic year</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>London Mathematical Society</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>Collaborative Teaching &amp; Scholarship Project Grants</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>Collaborative teaching scholarship</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>Up to £3,000; project delivered in the academic year following the award</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>UK mathematical scientists across at least two universities; lead below Associate Professor/Reader/Professor level; PhD students ineligible</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>Strong route for multi-university Statistics education work on curricula, assessment, teaching methods, student experience or outcomes.</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>Scholarship; collaboration; mathematics education; curriculum; evaluation</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>Latest round closed; LMS states that a new call will take place in the next academic year. Identify potential partner universities early.</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>https://www.lms.ac.uk/grants/collaborative-teaching-scholarship</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>LMS</x:v>
+      </x:c>
+      <x:c r="M47" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N47" s="54" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O47" s="54"/>
+      <x:c r="P47" s="58" t="str">
+        <x:f>IF(O47&lt;&gt;"Yes","","New funding opportunity added: "&amp;D47)</x:f>
+      </x:c>
+      <x:c r="Q47" s="58" t="str">
+        <x:f>IF(O47&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D47&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C47&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B47),TEXT(B47,"d mmmm yyyy"),B47)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F47&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G47&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H47&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I47&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R47" s="58" t="str">
+        <x:f>IF(O47&lt;&gt;"Yes","",HYPERLINK(K47,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S47" s="58" t="str">
+        <x:f>IF(O47&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T47" s="61"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="66" t="str">
+        <x:f>IF(AND(ISNUMBER(B48),B48&lt;TODAY()),"DEADLINE PASSED",N48)</x:f>
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>TBC – next academic year</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>London Mathematical Society</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>Scholarship Network Grants</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Teaching scholarship network</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Up to £1,000 per funding round for remote or in-person networking activity</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>UK mathematical scientists from at least three HE institutions; applicant below Associate Professor/Reader/Professor level; PhD students ineligible</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>Useful for building a Statistics education network around assessment, data literacy, inclusive quantitative education or curriculum innovation.</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>Scholarship; network; mathematics education; events; collaboration</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>Latest round closed; LMS states that a new call will take place in the next academic year. At least one event is expected to be in person.</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>https://www.lms.ac.uk/grants/scholarship-networks</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>LMS</x:v>
+      </x:c>
+      <x:c r="M48" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N48" s="54" t="str">
+        <x:v>FORTHCOMING</x:v>
+      </x:c>
+      <x:c r="O48" s="54"/>
+      <x:c r="P48" s="58" t="str">
+        <x:f>IF(O48&lt;&gt;"Yes","","New funding opportunity added: "&amp;D48)</x:f>
+      </x:c>
+      <x:c r="Q48" s="58" t="str">
+        <x:f>IF(O48&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D48&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C48&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B48),TEXT(B48,"d mmmm yyyy"),B48)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F48&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G48&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H48&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I48&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R48" s="58" t="str">
+        <x:f>IF(O48&lt;&gt;"Yes","",HYPERLINK(K48,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S48" s="58" t="str">
+        <x:f>IF(O48&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T48" s="61"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="64" t="str">
+        <x:f>IF(AND(ISNUMBER(B49),B49&lt;TODAY()),"DEADLINE PASSED",N49)</x:f>
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Next call TBC</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>QAA Scotland / CDN / SFC</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Scotland’s Tertiary Enhancement Programme (STEP) funded projects</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Collaborative educational enhancement</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Previous targeted call offered up to £10,000; future call value and terms TBC</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>Previous call was open to staff and students at Scottish colleges and universities; multi-institution or agency collaboration and student partnership required</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>Statistics could contribute evaluation design, quantitative evidence and projects supporting diverse learner journeys, assessment and student success.</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>Scholarship; educational enhancement; student experience; collaboration; evaluation</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>The verified £10,000 call closed on 3 December 2025. Monitor QAA Scotland and STEP for future funded project calls.</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>https://www.qaa.ac.uk/scotland/news-events/news/step-calls-for-proposals-for-funded-project</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>QAA Scotland</x:v>
+      </x:c>
+      <x:c r="M49" s="54" t="str">
+        <x:v>Scholarship</x:v>
+      </x:c>
+      <x:c r="N49" s="54" t="str">
+        <x:v>CLOSED – monitor recurrence</x:v>
+      </x:c>
+      <x:c r="O49" s="54"/>
+      <x:c r="P49" s="58" t="str">
+        <x:f>IF(O49&lt;&gt;"Yes","","New funding opportunity added: "&amp;D49)</x:f>
+      </x:c>
+      <x:c r="Q49" s="58" t="str">
+        <x:f>IF(O49&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;D49&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C49&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B49),TEXT(B49,"d mmmm yyyy"),B49)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F49&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply:"&amp;CHAR(10)&amp;G49&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics:"&amp;CHAR(10)&amp;H49&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I49&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder:"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela"&amp;CHAR(10)&amp;CHAR(10)&amp;"Statistics Research &amp; Scholarship"&amp;CHAR(10)&amp;"School of Mathematics &amp; Statistics"&amp;CHAR(10)&amp;"University of Glasgow")</x:f>
+      </x:c>
+      <x:c r="R49" s="58" t="str">
+        <x:f>IF(O49&lt;&gt;"Yes","",HYPERLINK(K49,"View official opportunity"))</x:f>
+      </x:c>
+      <x:c r="S49" s="58" t="str">
+        <x:f>IF(O49&lt;&gt;"Yes","",HYPERLINK("https://uofgstats.github.io/research-and-scholarship/","Open Funding Finder"))</x:f>
+      </x:c>
+      <x:c r="T49" s="61"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A2:A42">
@@ -4333,6 +4840,20 @@
       <x:formula>LEFT($A2,6)="CLOSED"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="8" priority="4">
+      <x:formula>$A2="DEADLINE PASSED"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="A2:A49">
+    <x:cfRule type="expression" dxfId="9" priority="5">
+      <x:formula>$A2="OPEN"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="10" priority="6">
+      <x:formula>$A2="FORTHCOMING"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="11" priority="7">
+      <x:formula>LEFT($A2,6)="CLOSED"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="12" priority="8">
       <x:formula>$A2="DEADLINE PASSED"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -4349,7 +4870,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d4c24f27d7e4920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19e8221b81d44eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4380,61 +4901,61 @@
       <x:c r="A3" s="4" t="s">
         <x:v>333</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>334</x:v>
+      <x:c r="B3" s="2" t="str">
+        <x:v>1 October 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45">
       <x:c r="A4" s="4" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>335</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>336</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45">
       <x:c r="A5" s="4" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="s">
         <x:v>337</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32">
       <x:c r="A6" s="4" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
         <x:v>339</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="s">
-        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30">
       <x:c r="A7" s="4" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
         <x:v>341</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>342</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="4" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
         <x:v>343</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>345</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
         <x:v>214</x:v>
@@ -4442,31 +4963,31 @@
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>346</x:v>
+        <x:v>345</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>347</x:v>
+        <x:v>346</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B13" s="2" t="s">
-        <x:v>348</x:v>
+        <x:v>347</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B14" s="2" t="s">
         <x:v>135</x:v>
@@ -4474,15 +4995,15 @@
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B15" s="2" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="16">
       <x:c r="A16" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B16" s="2" t="s">
         <x:v>322</x:v>
@@ -4490,7 +5011,7 @@
     </x:row>
     <x:row r="17" ht="16">
       <x:c r="A17" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B17" s="2" t="s">
         <x:v>116</x:v>
@@ -4498,7 +5019,7 @@
     </x:row>
     <x:row r="18" ht="16">
       <x:c r="A18" s="4" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B18" s="2" t="s">
         <x:v>143</x:v>
@@ -4506,10 +5027,10 @@
     </x:row>
     <x:row r="19" ht="45">
       <x:c r="A19" s="4" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="s">
         <x:v>350</x:v>
-      </x:c>
-      <x:c r="B19" s="2" t="s">
-        <x:v>351</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -4522,42 +5043,42 @@
     </x:row>
     <x:row r="21" ht="42.75" customHeight="1">
       <x:c r="A21" s="6" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="s">
         <x:v>352</x:v>
-      </x:c>
-      <x:c r="B21" s="6" t="s">
-        <x:v>353</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15">
       <x:c r="A22" s="7" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B22" s="5" t="s">
         <x:v>354</x:v>
-      </x:c>
-      <x:c r="B22" s="5" t="s">
-        <x:v>355</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15">
       <x:c r="A23" s="7" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="B23" s="5" t="s">
-        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30">
       <x:c r="A24" s="7" t="s">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="s">
         <x:v>358</x:v>
-      </x:c>
-      <x:c r="B24" s="5" t="s">
-        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15">
       <x:c r="A25" s="7" t="s">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
         <x:v>360</x:v>
-      </x:c>
-      <x:c r="B25" s="5" t="s">
-        <x:v>361</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Mark launch opportunities as not notified
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R30c2fb5e73db4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R1a13069f9ac04b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding opportunities" sheetId="1" r:id="R873e560c95b14efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; sources" sheetId="2" r:id="R07ffef5285a14554"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1071,9 +1071,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Step 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Set Notify? to Yes on the opportunity you want to announce.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Step 2</x:t>
@@ -1564,7 +1561,7 @@
         <x:color rgb="FF38761D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1575,7 +1572,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1586,7 +1583,7 @@
         <x:color rgb="FF595959"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7E6E6"/>
         </x:patternFill>
       </x:fill>
@@ -1597,7 +1594,7 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -1844,7 +1841,7 @@
     <x:col min="12" max="12" width="18" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="27" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="11" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="32" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="48" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
@@ -1960,6 +1957,7 @@
       </x:c>
       <x:c r="O2" s="23" t="str">
         <x:f t="shared" ref="O2:O42" si="1">IF(N2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P2" s="31" t="str">
         <x:f t="shared" ref="P2:P42" si="2">IF(O2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</x:f>
@@ -2019,8 +2017,9 @@
       <x:c r="N3" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O3" s="23">
+      <x:c r="O3" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P3" s="31" t="str">
         <x:f t="shared" si="2">IF(O3&lt;&gt;"Yes","","New funding opportunity added: "&amp;D3)</x:f>
@@ -2080,8 +2079,9 @@
       <x:c r="N4" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O4" s="23">
+      <x:c r="O4" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P4" s="31" t="str">
         <x:f t="shared" si="2">IF(O4&lt;&gt;"Yes","","New funding opportunity added: "&amp;D4)</x:f>
@@ -2141,8 +2141,9 @@
       <x:c r="N5" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O5" s="23">
+      <x:c r="O5" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P5" s="31" t="str">
         <x:f t="shared" si="2">IF(O5&lt;&gt;"Yes","","New funding opportunity added: "&amp;D5)</x:f>
@@ -2202,8 +2203,9 @@
       <x:c r="N6" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O6" s="23">
+      <x:c r="O6" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P6" s="31" t="str">
         <x:f t="shared" si="2">IF(O6&lt;&gt;"Yes","","New funding opportunity added: "&amp;D6)</x:f>
@@ -2263,8 +2265,9 @@
       <x:c r="N7" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O7" s="23">
+      <x:c r="O7" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P7" s="31" t="str">
         <x:f t="shared" si="2">IF(O7&lt;&gt;"Yes","","New funding opportunity added: "&amp;D7)</x:f>
@@ -2324,8 +2327,9 @@
       <x:c r="N8" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O8" s="23">
+      <x:c r="O8" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P8" s="31" t="str">
         <x:f t="shared" si="2">IF(O8&lt;&gt;"Yes","","New funding opportunity added: "&amp;D8)</x:f>
@@ -2385,8 +2389,9 @@
       <x:c r="N9" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O9" s="23">
+      <x:c r="O9" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P9" s="31" t="str">
         <x:f t="shared" si="2">IF(O9&lt;&gt;"Yes","","New funding opportunity added: "&amp;D9)</x:f>
@@ -2446,8 +2451,9 @@
       <x:c r="N10" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O10" s="23">
+      <x:c r="O10" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P10" s="31" t="str">
         <x:f t="shared" si="2">IF(O10&lt;&gt;"Yes","","New funding opportunity added: "&amp;D10)</x:f>
@@ -2507,8 +2513,9 @@
       <x:c r="N11" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O11" s="23">
+      <x:c r="O11" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P11" s="31" t="str">
         <x:f t="shared" si="2">IF(O11&lt;&gt;"Yes","","New funding opportunity added: "&amp;D11)</x:f>
@@ -2568,8 +2575,9 @@
       <x:c r="N12" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O12" s="23">
+      <x:c r="O12" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P12" s="31" t="str">
         <x:f t="shared" si="2">IF(O12&lt;&gt;"Yes","","New funding opportunity added: "&amp;D12)</x:f>
@@ -2629,8 +2637,9 @@
       <x:c r="N13" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O13" s="23">
+      <x:c r="O13" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P13" s="31" t="str">
         <x:f t="shared" si="2">IF(O13&lt;&gt;"Yes","","New funding opportunity added: "&amp;D13)</x:f>
@@ -2690,8 +2699,9 @@
       <x:c r="N14" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O14" s="23">
+      <x:c r="O14" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P14" s="31" t="str">
         <x:f t="shared" si="2">IF(O14&lt;&gt;"Yes","","New funding opportunity added: "&amp;D14)</x:f>
@@ -2751,8 +2761,9 @@
       <x:c r="N15" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O15" s="23">
+      <x:c r="O15" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P15" s="31" t="str">
         <x:f t="shared" si="2">IF(O15&lt;&gt;"Yes","","New funding opportunity added: "&amp;D15)</x:f>
@@ -2812,8 +2823,9 @@
       <x:c r="N16" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O16" s="23">
+      <x:c r="O16" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P16" s="31" t="str">
         <x:f t="shared" si="2">IF(O16&lt;&gt;"Yes","","New funding opportunity added: "&amp;D16)</x:f>
@@ -2873,8 +2885,9 @@
       <x:c r="N17" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O17" s="23">
+      <x:c r="O17" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P17" s="31" t="str">
         <x:f t="shared" si="2">IF(O17&lt;&gt;"Yes","","New funding opportunity added: "&amp;D17)</x:f>
@@ -2934,8 +2947,9 @@
       <x:c r="N18" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O18" s="23">
+      <x:c r="O18" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P18" s="31" t="str">
         <x:f t="shared" si="2">IF(O18&lt;&gt;"Yes","","New funding opportunity added: "&amp;D18)</x:f>
@@ -2995,8 +3009,9 @@
       <x:c r="N19" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O19" s="23">
+      <x:c r="O19" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P19" s="31" t="str">
         <x:f t="shared" si="2">IF(O19&lt;&gt;"Yes","","New funding opportunity added: "&amp;D19)</x:f>
@@ -3056,8 +3071,9 @@
       <x:c r="N20" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O20" s="23">
+      <x:c r="O20" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P20" s="31" t="str">
         <x:f t="shared" si="2">IF(O20&lt;&gt;"Yes","","New funding opportunity added: "&amp;D20)</x:f>
@@ -3117,8 +3133,9 @@
       <x:c r="N21" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O21" s="23">
+      <x:c r="O21" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P21" s="31" t="str">
         <x:f t="shared" si="2">IF(O21&lt;&gt;"Yes","","New funding opportunity added: "&amp;D21)</x:f>
@@ -3178,8 +3195,9 @@
       <x:c r="N22" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O22" s="23">
+      <x:c r="O22" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P22" s="31" t="str">
         <x:f t="shared" si="2">IF(O22&lt;&gt;"Yes","","New funding opportunity added: "&amp;D22)</x:f>
@@ -3239,8 +3257,9 @@
       <x:c r="N23" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O23" s="23">
+      <x:c r="O23" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P23" s="31" t="str">
         <x:f t="shared" si="2">IF(O23&lt;&gt;"Yes","","New funding opportunity added: "&amp;D23)</x:f>
@@ -3300,8 +3319,9 @@
       <x:c r="N24" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O24" s="23">
+      <x:c r="O24" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P24" s="31" t="str">
         <x:f t="shared" si="2">IF(O24&lt;&gt;"Yes","","New funding opportunity added: "&amp;D24)</x:f>
@@ -3361,8 +3381,9 @@
       <x:c r="N25" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O25" s="23">
+      <x:c r="O25" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P25" s="31" t="str">
         <x:f t="shared" si="2">IF(O25&lt;&gt;"Yes","","New funding opportunity added: "&amp;D25)</x:f>
@@ -3422,8 +3443,9 @@
       <x:c r="N26" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O26" s="23">
+      <x:c r="O26" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P26" s="31" t="str">
         <x:f t="shared" si="2">IF(O26&lt;&gt;"Yes","","New funding opportunity added: "&amp;D26)</x:f>
@@ -3483,8 +3505,9 @@
       <x:c r="N27" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O27" s="23">
+      <x:c r="O27" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P27" s="31" t="str">
         <x:f t="shared" si="2">IF(O27&lt;&gt;"Yes","","New funding opportunity added: "&amp;D27)</x:f>
@@ -3544,8 +3567,9 @@
       <x:c r="N28" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O28" s="23">
+      <x:c r="O28" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P28" s="31" t="str">
         <x:f t="shared" si="2">IF(O28&lt;&gt;"Yes","","New funding opportunity added: "&amp;D28)</x:f>
@@ -3605,8 +3629,9 @@
       <x:c r="N29" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O29" s="23">
+      <x:c r="O29" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P29" s="31" t="str">
         <x:f t="shared" si="2">IF(O29&lt;&gt;"Yes","","New funding opportunity added: "&amp;D29)</x:f>
@@ -3666,8 +3691,9 @@
       <x:c r="N30" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O30" s="23">
+      <x:c r="O30" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P30" s="31" t="str">
         <x:f t="shared" si="2">IF(O30&lt;&gt;"Yes","","New funding opportunity added: "&amp;D30)</x:f>
@@ -3727,8 +3753,9 @@
       <x:c r="N31" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O31" s="23">
+      <x:c r="O31" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P31" s="31" t="str">
         <x:f t="shared" si="2">IF(O31&lt;&gt;"Yes","","New funding opportunity added: "&amp;D31)</x:f>
@@ -3788,8 +3815,9 @@
       <x:c r="N32" s="23" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="O32" s="23">
+      <x:c r="O32" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P32" s="31" t="str">
         <x:f t="shared" si="2">IF(O32&lt;&gt;"Yes","","New funding opportunity added: "&amp;D32)</x:f>
@@ -3849,8 +3877,9 @@
       <x:c r="N33" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O33" s="23">
+      <x:c r="O33" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P33" s="31" t="str">
         <x:f t="shared" si="2">IF(O33&lt;&gt;"Yes","","New funding opportunity added: "&amp;D33)</x:f>
@@ -3910,8 +3939,9 @@
       <x:c r="N34" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O34" s="23">
+      <x:c r="O34" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P34" s="31" t="str">
         <x:f t="shared" si="2">IF(O34&lt;&gt;"Yes","","New funding opportunity added: "&amp;D34)</x:f>
@@ -3971,8 +4001,9 @@
       <x:c r="N35" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O35" s="23">
+      <x:c r="O35" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P35" s="31" t="str">
         <x:f t="shared" si="2">IF(O35&lt;&gt;"Yes","","New funding opportunity added: "&amp;D35)</x:f>
@@ -4032,8 +4063,9 @@
       <x:c r="N36" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O36" s="23">
+      <x:c r="O36" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P36" s="31" t="str">
         <x:f t="shared" si="2">IF(O36&lt;&gt;"Yes","","New funding opportunity added: "&amp;D36)</x:f>
@@ -4093,8 +4125,9 @@
       <x:c r="N37" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O37" s="23">
+      <x:c r="O37" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P37" s="31" t="str">
         <x:f t="shared" si="2">IF(O37&lt;&gt;"Yes","","New funding opportunity added: "&amp;D37)</x:f>
@@ -4154,8 +4187,9 @@
       <x:c r="N38" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O38" s="23">
+      <x:c r="O38" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P38" s="31" t="str">
         <x:f t="shared" si="2">IF(O38&lt;&gt;"Yes","","New funding opportunity added: "&amp;D38)</x:f>
@@ -4215,8 +4249,9 @@
       <x:c r="N39" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O39" s="23">
+      <x:c r="O39" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P39" s="31" t="str">
         <x:f t="shared" si="2">IF(O39&lt;&gt;"Yes","","New funding opportunity added: "&amp;D39)</x:f>
@@ -4276,8 +4311,9 @@
       <x:c r="N40" s="23" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O40" s="23">
+      <x:c r="O40" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P40" s="31" t="str">
         <x:f t="shared" si="2">IF(O40&lt;&gt;"Yes","","New funding opportunity added: "&amp;D40)</x:f>
@@ -4337,8 +4373,9 @@
       <x:c r="N41" s="23" t="str">
         <x:v>CLOSED – monitor recurrence</x:v>
       </x:c>
-      <x:c r="O41" s="23">
+      <x:c r="O41" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P41" s="31" t="str">
         <x:f t="shared" si="2">IF(O41&lt;&gt;"Yes","","New funding opportunity added: "&amp;D41)</x:f>
@@ -4398,8 +4435,9 @@
       <x:c r="N42" s="23" t="str">
         <x:v>CLOSED – invited stage continues</x:v>
       </x:c>
-      <x:c r="O42" s="23">
+      <x:c r="O42" s="23" t="str">
         <x:f t="shared" si="1"/>
+        <x:v>Added at launch – no notification</x:v>
       </x:c>
       <x:c r="P42" s="31" t="str">
         <x:f t="shared" si="2">IF(O42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</x:f>
@@ -4459,7 +4497,9 @@
       <x:c r="N43" s="54" t="str">
         <x:v>CLOSED – monitor recurrence</x:v>
       </x:c>
-      <x:c r="O43" s="54"/>
+      <x:c r="O43" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P43" s="58" t="str">
         <x:f>IF(O43&lt;&gt;"Yes","","New funding opportunity added: "&amp;D43)</x:f>
       </x:c>
@@ -4518,7 +4558,9 @@
       <x:c r="N44" s="54" t="str">
         <x:v>CLOSED – monitor recurrence</x:v>
       </x:c>
-      <x:c r="O44" s="54"/>
+      <x:c r="O44" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P44" s="58" t="str">
         <x:f>IF(O44&lt;&gt;"Yes","","New funding opportunity added: "&amp;D44)</x:f>
       </x:c>
@@ -4577,7 +4619,9 @@
       <x:c r="N45" s="54" t="str">
         <x:v>CLOSED – monitor recurrence</x:v>
       </x:c>
-      <x:c r="O45" s="54"/>
+      <x:c r="O45" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P45" s="58" t="str">
         <x:f>IF(O45&lt;&gt;"Yes","","New funding opportunity added: "&amp;D45)</x:f>
       </x:c>
@@ -4636,7 +4680,9 @@
       <x:c r="N46" s="54" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O46" s="54"/>
+      <x:c r="O46" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P46" s="58" t="str">
         <x:f>IF(O46&lt;&gt;"Yes","","New funding opportunity added: "&amp;D46)</x:f>
       </x:c>
@@ -4695,7 +4741,9 @@
       <x:c r="N47" s="54" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O47" s="54"/>
+      <x:c r="O47" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P47" s="58" t="str">
         <x:f>IF(O47&lt;&gt;"Yes","","New funding opportunity added: "&amp;D47)</x:f>
       </x:c>
@@ -4754,7 +4802,9 @@
       <x:c r="N48" s="54" t="str">
         <x:v>FORTHCOMING</x:v>
       </x:c>
-      <x:c r="O48" s="54"/>
+      <x:c r="O48" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P48" s="58" t="str">
         <x:f>IF(O48&lt;&gt;"Yes","","New funding opportunity added: "&amp;D48)</x:f>
       </x:c>
@@ -4813,7 +4863,9 @@
       <x:c r="N49" s="54" t="str">
         <x:v>CLOSED – monitor recurrence</x:v>
       </x:c>
-      <x:c r="O49" s="54"/>
+      <x:c r="O49" s="54" t="str">
+        <x:v>Added at launch – no notification</x:v>
+      </x:c>
       <x:c r="P49" s="58" t="str">
         <x:f>IF(O49&lt;&gt;"Yes","","New funding opportunity added: "&amp;D49)</x:f>
       </x:c>
@@ -4865,12 +4917,12 @@
       <x:formula1>"OPEN,FORTHCOMING,CLOSED – monitor recurrence,CLOSED – invited stage continues"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O2:O500">
-      <x:formula1>"Yes,No"</x:formula1>
+      <x:formula1>"Yes,No,Added at launch – no notification"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19e8221b81d44eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R706c2a24e94f46bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5053,32 +5105,32 @@
       <x:c r="A22" s="7" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="s">
-        <x:v>354</x:v>
+      <x:c r="B22" s="5" t="str">
+        <x:v>Set Notify? to Yes for a genuinely new opportunity. Existing launch entries are marked Added at launch – no notification.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15">
       <x:c r="A23" s="7" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>355</x:v>
-      </x:c>
-      <x:c r="B23" s="5" t="s">
-        <x:v>356</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30">
       <x:c r="A24" s="7" t="s">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="s">
         <x:v>357</x:v>
-      </x:c>
-      <x:c r="B24" s="5" t="s">
-        <x:v>358</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15">
       <x:c r="A25" s="7" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
         <x:v>359</x:v>
-      </x:c>
-      <x:c r="B25" s="5" t="s">
-        <x:v>360</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
two new opportunities added
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielacastrocamilo/Dropbox/Glasgow/Admin/ResearchLead4Statistics/research-and-scholarship/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063A9612-AC22-1E4D-ADD7-0732ED13EA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C557CAB3-B793-AB49-A11F-54FCBF7095A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34400" yWindow="600" windowWidth="34400" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="34400" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Funding opportunities" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="475">
   <si>
     <t>Status</t>
   </si>
@@ -1119,9 +1119,6 @@
     <t>Research / Scholarship</t>
   </si>
   <si>
-    <t>Status setting</t>
-  </si>
-  <si>
     <t>Notify?</t>
   </si>
   <si>
@@ -1401,10 +1398,67 @@
     <t>Institutional demand management applies for 2027: Glasgow can submit max. 8 applications. Check UofG internal selection/deadline when announced. UK Sponsor may support only one application per round. Funding figures currently based on 2026 guidance; update once full 2027 scheme guidance is published.</t>
   </si>
   <si>
-    <t>https://www.thebritishacademy.ac.uk/documents/6283/International_Fellowships_2027_-_FAQs.pdf?utm_source=chatgpt.com</t>
-  </si>
-  <si>
     <t>British Academy / Royal Society</t>
+  </si>
+  <si>
+    <t>15 December 2026, 16:00</t>
+  </si>
+  <si>
+    <t>ESRC / UKRI, co-funded by Defra</t>
+  </si>
+  <si>
+    <t>Up to £21.1m funder contribution; 44 months; single award; 80% FEC (with some exceptions at 100%). Must start by 1 August 2027.</t>
+  </si>
+  <si>
+    <t>Researchers based at UK research organisations eligible for UKRI/ESRC funding. At least one project co-lead from a UK business, third-sector or government organisation is required.</t>
+  </si>
+  <si>
+    <t>Major interdisciplinary opportunity with a strong methodological component, explicitly including robust evaluation, experimental and quasi-experimental methods, and causal reasoning, with applications including wildfire, drought, flooding and extreme heat.</t>
+  </si>
+  <si>
+    <t>Climate resilience; environmental statistics; causal inference; evaluation; extremes; interdisciplinary research</t>
+  </si>
+  <si>
+    <t>Demand management applies. Check UofG internal selection process/deadline before preparing an application. Large centre-scale opportunity requiring a broad interdisciplinary consortium and at least one UK non-academic co-lead.</t>
+  </si>
+  <si>
+    <t>Research programme / Centre</t>
+  </si>
+  <si>
+    <t>Manual status</t>
+  </si>
+  <si>
+    <t>https://www.ukri.org/opportunity/what-works-centre-for-a-climate-resilient-uk/</t>
+  </si>
+  <si>
+    <t>Open – no fixed deadline</t>
+  </si>
+  <si>
+    <t>NERC / UKRI</t>
+  </si>
+  <si>
+    <t>NERC urgency funding</t>
+  </si>
+  <si>
+    <t>Up to £100,000 FEC (NERC funds 80%); up to 1 year</t>
+  </si>
+  <si>
+    <t>Researchers at UK organisations eligible for NERC funding. Must respond to an unexpected, transient environmental event; outline required within 4 weeks of the event starting. Applicants cannot have been PL/PcL on another full application to this scheme in the previous 2 years.</t>
+  </si>
+  <si>
+    <t>Strong fit for environmental statistics and extremes, supporting rapid research following unexpected events such as droughts, floods and earthquakes, including collection and initial analysis of critical early data.</t>
+  </si>
+  <si>
+    <t>Environmental statistics; Extremes; Climate &amp; environment; Urgency funding</t>
+  </si>
+  <si>
+    <t>Outline (1 page) must be emailed to NERC within 4 weeks of the event starting. If approved, full application is due within 10 working days of invitation. Intended for genuinely unexpected events where waiting for normal funding would mean losing the research opportunity.</t>
+  </si>
+  <si>
+    <t>https://www.ukri.org/opportunity/nerc-urgency-funding-open/</t>
+  </si>
+  <si>
+    <t>https://www.thebritishacademy.ac.uk/documents/6283/International_Fellowships_2027_-_FAQs.pdf</t>
   </si>
 </sst>
 </file>
@@ -1667,7 +1721,51 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF38761D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1822,8 +1920,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R51" totalsRowShown="0">
-  <autoFilter ref="A1:R51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R53" totalsRowShown="0">
+  <autoFilter ref="A1:R53" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Status">
       <calculatedColumnFormula>IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",N2)</calculatedColumnFormula>
@@ -1840,10 +1938,10 @@
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Source"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Source list"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Research / Scholarship"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Status setting"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Manual status"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notify?"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Email subject"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Email body" dataDxfId="8">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Email body" dataDxfId="12">
       <calculatedColumnFormula>IF(O2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D2&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Notification date"/>
@@ -2047,7 +2145,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2111,19 +2209,19 @@
         <v>360</v>
       </c>
       <c r="N1" s="14" t="s">
+        <v>463</v>
+      </c>
+      <c r="O1" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="P1" s="14" t="s">
         <v>362</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="Q1" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="Q1" s="14" t="s">
+      <c r="R1" s="14" t="s">
         <v>364</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="30">
@@ -2165,13 +2263,13 @@
         <v>12</v>
       </c>
       <c r="M2" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N2" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N2" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O2" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P2" s="12" t="str">
         <f t="shared" ref="P2:P42" si="1">IF(O2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</f>
@@ -2182,7 +2280,7 @@
         <v/>
       </c>
       <c r="R2" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="30">
@@ -2224,13 +2322,13 @@
         <v>21</v>
       </c>
       <c r="M3" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N3" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N3" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O3" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P3" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2241,13 +2339,13 @@
         <v/>
       </c>
       <c r="R3" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="30">
       <c r="A4" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>DEADLINE PASSED</v>
       </c>
       <c r="B4" s="3">
         <v>46296</v>
@@ -2283,13 +2381,13 @@
         <v>12</v>
       </c>
       <c r="M4" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N4" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N4" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O4" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P4" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2300,7 +2398,7 @@
         <v/>
       </c>
       <c r="R4" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="45">
@@ -2342,13 +2440,13 @@
         <v>21</v>
       </c>
       <c r="M5" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N5" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N5" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O5" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P5" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2359,7 +2457,7 @@
         <v/>
       </c>
       <c r="R5" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="30">
@@ -2401,13 +2499,13 @@
         <v>12</v>
       </c>
       <c r="M6" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N6" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N6" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O6" s="11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="P6" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2432,7 +2530,7 @@
 Research Lead for Statistics</v>
       </c>
       <c r="R6" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="30">
@@ -2474,13 +2572,13 @@
         <v>12</v>
       </c>
       <c r="M7" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N7" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N7" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O7" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P7" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2491,7 +2589,7 @@
         <v/>
       </c>
       <c r="R7" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="45">
@@ -2533,13 +2631,13 @@
         <v>12</v>
       </c>
       <c r="M8" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N8" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N8" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O8" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P8" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2550,7 +2648,7 @@
         <v/>
       </c>
       <c r="R8" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="30">
@@ -2592,13 +2690,13 @@
         <v>67</v>
       </c>
       <c r="M9" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N9" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N9" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O9" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P9" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2609,7 +2707,7 @@
         <v/>
       </c>
       <c r="R9" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="30">
@@ -2651,13 +2749,13 @@
         <v>67</v>
       </c>
       <c r="M10" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N10" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N10" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O10" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P10" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2668,7 +2766,7 @@
         <v/>
       </c>
       <c r="R10" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="30">
@@ -2710,13 +2808,13 @@
         <v>67</v>
       </c>
       <c r="M11" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N11" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N11" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O11" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P11" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2727,7 +2825,7 @@
         <v/>
       </c>
       <c r="R11" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="30">
@@ -2769,13 +2867,13 @@
         <v>67</v>
       </c>
       <c r="M12" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N12" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N12" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O12" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P12" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2786,7 +2884,7 @@
         <v/>
       </c>
       <c r="R12" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="30">
@@ -2828,13 +2926,13 @@
         <v>67</v>
       </c>
       <c r="M13" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N13" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N13" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O13" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P13" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2845,7 +2943,7 @@
         <v/>
       </c>
       <c r="R13" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="45">
@@ -2887,13 +2985,13 @@
         <v>67</v>
       </c>
       <c r="M14" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N14" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N14" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O14" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P14" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2904,7 +3002,7 @@
         <v/>
       </c>
       <c r="R14" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="45">
@@ -2946,13 +3044,13 @@
         <v>124</v>
       </c>
       <c r="M15" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N15" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N15" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O15" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P15" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2963,7 +3061,7 @@
         <v/>
       </c>
       <c r="R15" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="30">
@@ -3005,13 +3103,13 @@
         <v>67</v>
       </c>
       <c r="M16" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N16" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N16" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O16" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P16" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3022,7 +3120,7 @@
         <v/>
       </c>
       <c r="R16" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="30">
@@ -3064,13 +3162,13 @@
         <v>124</v>
       </c>
       <c r="M17" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N17" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N17" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O17" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P17" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3081,7 +3179,7 @@
         <v/>
       </c>
       <c r="R17" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="45">
@@ -3123,13 +3221,13 @@
         <v>124</v>
       </c>
       <c r="M18" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N18" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N18" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O18" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P18" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3140,7 +3238,7 @@
         <v/>
       </c>
       <c r="R18" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="19" spans="1:18" ht="30">
@@ -3182,13 +3280,13 @@
         <v>12</v>
       </c>
       <c r="M19" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N19" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N19" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O19" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P19" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3199,7 +3297,7 @@
         <v/>
       </c>
       <c r="R19" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="45">
@@ -3241,13 +3339,13 @@
         <v>67</v>
       </c>
       <c r="M20" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N20" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N20" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O20" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P20" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3258,7 +3356,7 @@
         <v/>
       </c>
       <c r="R20" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="21" spans="1:18" ht="30">
@@ -3300,13 +3398,13 @@
         <v>67</v>
       </c>
       <c r="M21" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N21" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N21" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O21" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P21" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3317,7 +3415,7 @@
         <v/>
       </c>
       <c r="R21" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="22" spans="1:18" ht="30">
@@ -3359,13 +3457,13 @@
         <v>12</v>
       </c>
       <c r="M22" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N22" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N22" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O22" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P22" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3376,7 +3474,7 @@
         <v/>
       </c>
       <c r="R22" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="23" spans="1:18" ht="30">
@@ -3418,13 +3516,13 @@
         <v>12</v>
       </c>
       <c r="M23" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N23" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N23" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O23" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P23" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3435,7 +3533,7 @@
         <v/>
       </c>
       <c r="R23" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="30">
@@ -3477,13 +3575,13 @@
         <v>12</v>
       </c>
       <c r="M24" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N24" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N24" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O24" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P24" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3494,7 +3592,7 @@
         <v/>
       </c>
       <c r="R24" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="25" spans="1:18" ht="30">
@@ -3536,13 +3634,13 @@
         <v>12</v>
       </c>
       <c r="M25" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N25" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N25" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O25" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P25" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3553,7 +3651,7 @@
         <v/>
       </c>
       <c r="R25" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="30">
@@ -3595,13 +3693,13 @@
         <v>12</v>
       </c>
       <c r="M26" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N26" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N26" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O26" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P26" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3612,7 +3710,7 @@
         <v/>
       </c>
       <c r="R26" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="27" spans="1:18" ht="30">
@@ -3654,13 +3752,13 @@
         <v>12</v>
       </c>
       <c r="M27" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N27" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N27" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O27" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P27" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3671,7 +3769,7 @@
         <v/>
       </c>
       <c r="R27" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="45">
@@ -3713,13 +3811,13 @@
         <v>124</v>
       </c>
       <c r="M28" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N28" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N28" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O28" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P28" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3730,7 +3828,7 @@
         <v/>
       </c>
       <c r="R28" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="29" spans="1:18" ht="45">
@@ -3772,13 +3870,13 @@
         <v>230</v>
       </c>
       <c r="M29" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N29" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N29" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O29" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P29" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3789,7 +3887,7 @@
         <v/>
       </c>
       <c r="R29" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="30" spans="1:18" ht="30">
@@ -3831,13 +3929,13 @@
         <v>230</v>
       </c>
       <c r="M30" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N30" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N30" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O30" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P30" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3848,7 +3946,7 @@
         <v/>
       </c>
       <c r="R30" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="30">
@@ -3890,13 +3988,13 @@
         <v>230</v>
       </c>
       <c r="M31" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N31" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N31" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O31" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P31" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3907,7 +4005,7 @@
         <v/>
       </c>
       <c r="R31" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="32" spans="1:18" ht="45">
@@ -3949,13 +4047,13 @@
         <v>230</v>
       </c>
       <c r="M32" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N32" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N32" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O32" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P32" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3966,7 +4064,7 @@
         <v/>
       </c>
       <c r="R32" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="33" spans="1:18" ht="60">
@@ -4008,13 +4106,13 @@
         <v>258</v>
       </c>
       <c r="M33" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P33" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4025,7 +4123,7 @@
         <v/>
       </c>
       <c r="R33" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="34" spans="1:18" ht="45">
@@ -4067,13 +4165,13 @@
         <v>258</v>
       </c>
       <c r="M34" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P34" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4084,7 +4182,7 @@
         <v/>
       </c>
       <c r="R34" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="35" spans="1:18" ht="30">
@@ -4126,13 +4224,13 @@
         <v>258</v>
       </c>
       <c r="M35" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P35" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4143,7 +4241,7 @@
         <v/>
       </c>
       <c r="R35" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="30">
@@ -4185,13 +4283,13 @@
         <v>258</v>
       </c>
       <c r="M36" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P36" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4202,7 +4300,7 @@
         <v/>
       </c>
       <c r="R36" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="37" spans="1:18" ht="30">
@@ -4244,13 +4342,13 @@
         <v>258</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P37" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4261,7 +4359,7 @@
         <v/>
       </c>
       <c r="R37" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="38" spans="1:18" ht="30">
@@ -4303,13 +4401,13 @@
         <v>258</v>
       </c>
       <c r="M38" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P38" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4320,7 +4418,7 @@
         <v/>
       </c>
       <c r="R38" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="39" spans="1:18" ht="30">
@@ -4362,13 +4460,13 @@
         <v>258</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O39" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P39" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4379,7 +4477,7 @@
         <v/>
       </c>
       <c r="R39" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="40" spans="1:18" ht="30">
@@ -4421,13 +4519,13 @@
         <v>258</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P40" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4438,7 +4536,7 @@
         <v/>
       </c>
       <c r="R40" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="41" spans="1:18" ht="45">
@@ -4480,13 +4578,13 @@
         <v>124</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P41" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4497,7 +4595,7 @@
         <v/>
       </c>
       <c r="R41" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="42" spans="1:18" ht="45">
@@ -4539,13 +4637,13 @@
         <v>124</v>
       </c>
       <c r="M42" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N42" s="11" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="O42" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P42" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4556,7 +4654,7 @@
         <v/>
       </c>
       <c r="R42" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="43" spans="1:18" ht="45">
@@ -4565,46 +4663,46 @@
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B43" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C43" t="s">
         <v>312</v>
       </c>
       <c r="D43" t="s">
+        <v>371</v>
+      </c>
+      <c r="E43" t="s">
         <v>372</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="G43" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="I43" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="K43" s="2" t="s">
+      <c r="L43" t="s">
         <v>379</v>
       </c>
-      <c r="L43" t="s">
+      <c r="M43" s="16" t="s">
         <v>380</v>
       </c>
-      <c r="M43" s="16" t="s">
+      <c r="N43" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O43" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N43" s="16" t="s">
-        <v>369</v>
-      </c>
-      <c r="O43" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P43" s="17" t="str">
         <f t="shared" ref="P43:P49" si="4">IF(O43&lt;&gt;"Yes","","New funding opportunity added: "&amp;D43)</f>
@@ -4615,7 +4713,7 @@
         <v/>
       </c>
       <c r="R43" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="44" spans="1:18" ht="45">
@@ -4624,46 +4722,46 @@
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B44" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C44" t="s">
         <v>312</v>
       </c>
       <c r="D44" t="s">
+        <v>382</v>
+      </c>
+      <c r="E44" t="s">
         <v>383</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="I44" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>387</v>
-      </c>
       <c r="J44" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="K44" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="L44" t="s">
         <v>379</v>
       </c>
-      <c r="L44" t="s">
+      <c r="M44" s="16" t="s">
         <v>380</v>
       </c>
-      <c r="M44" s="16" t="s">
+      <c r="N44" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O44" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N44" s="16" t="s">
-        <v>369</v>
-      </c>
-      <c r="O44" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P44" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4674,7 +4772,7 @@
         <v/>
       </c>
       <c r="R44" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="45" spans="1:18" ht="45">
@@ -4683,46 +4781,46 @@
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B45" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C45" t="s">
         <v>312</v>
       </c>
       <c r="D45" t="s">
+        <v>388</v>
+      </c>
+      <c r="E45" t="s">
         <v>389</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="J45" s="2" t="s">
-        <v>395</v>
-      </c>
       <c r="K45" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="L45" t="s">
         <v>379</v>
       </c>
-      <c r="L45" t="s">
+      <c r="M45" s="16" t="s">
         <v>380</v>
       </c>
-      <c r="M45" s="16" t="s">
+      <c r="N45" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O45" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N45" s="16" t="s">
-        <v>369</v>
-      </c>
-      <c r="O45" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P45" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4733,7 +4831,7 @@
         <v/>
       </c>
       <c r="R45" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="46" spans="1:18" ht="60">
@@ -4742,46 +4840,46 @@
         <v>FORTHCOMING</v>
       </c>
       <c r="B46" t="s">
+        <v>395</v>
+      </c>
+      <c r="C46" t="s">
         <v>396</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>397</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>398</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="I46" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="J46" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="J46" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>404</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>405</v>
       </c>
       <c r="L46" t="s">
         <v>12</v>
       </c>
       <c r="M46" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="N46" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="O46" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N46" s="16" t="s">
-        <v>368</v>
-      </c>
-      <c r="O46" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P46" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4792,7 +4890,7 @@
         <v/>
       </c>
       <c r="R46" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="47" spans="1:18" ht="60">
@@ -4801,46 +4899,46 @@
         <v>FORTHCOMING</v>
       </c>
       <c r="B47" t="s">
+        <v>395</v>
+      </c>
+      <c r="C47" t="s">
         <v>396</v>
       </c>
-      <c r="C47" t="s">
-        <v>397</v>
-      </c>
       <c r="D47" t="s">
+        <v>405</v>
+      </c>
+      <c r="E47" t="s">
         <v>406</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="G47" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="I47" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="J47" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="J47" s="2" t="s">
+      <c r="K47" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>413</v>
       </c>
       <c r="L47" t="s">
         <v>12</v>
       </c>
       <c r="M47" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="N47" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="O47" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N47" s="16" t="s">
-        <v>368</v>
-      </c>
-      <c r="O47" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P47" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4851,7 +4949,7 @@
         <v/>
       </c>
       <c r="R47" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="60">
@@ -4860,46 +4958,46 @@
         <v>FORTHCOMING</v>
       </c>
       <c r="B48" t="s">
+        <v>395</v>
+      </c>
+      <c r="C48" t="s">
         <v>396</v>
       </c>
-      <c r="C48" t="s">
-        <v>397</v>
-      </c>
       <c r="D48" t="s">
+        <v>413</v>
+      </c>
+      <c r="E48" t="s">
         <v>414</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="G48" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="I48" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="J48" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="J48" s="2" t="s">
+      <c r="K48" s="2" t="s">
         <v>420</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>421</v>
       </c>
       <c r="L48" t="s">
         <v>12</v>
       </c>
       <c r="M48" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="N48" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="O48" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N48" s="16" t="s">
-        <v>368</v>
-      </c>
-      <c r="O48" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P48" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4910,7 +5008,7 @@
         <v/>
       </c>
       <c r="R48" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="49" spans="1:18" ht="60">
@@ -4919,46 +5017,46 @@
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B49" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C49" t="s">
+        <v>421</v>
+      </c>
+      <c r="D49" t="s">
         <v>422</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>423</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="G49" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="H49" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="I49" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="J49" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="J49" s="2" t="s">
+      <c r="K49" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="L49" t="s">
         <v>430</v>
       </c>
-      <c r="L49" t="s">
-        <v>431</v>
-      </c>
       <c r="M49" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="N49" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="O49" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="N49" s="16" t="s">
-        <v>369</v>
-      </c>
-      <c r="O49" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="P49" s="17" t="str">
         <f t="shared" si="4"/>
@@ -4969,7 +5067,7 @@
         <v/>
       </c>
       <c r="R49" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="50" spans="1:18" ht="60">
@@ -4981,43 +5079,43 @@
         <v>46362</v>
       </c>
       <c r="C50" t="s">
+        <v>436</v>
+      </c>
+      <c r="D50" t="s">
         <v>437</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>438</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="H50" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="I50" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="J50" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="J50" s="2" t="s">
+      <c r="K50" s="21" t="s">
         <v>444</v>
       </c>
-      <c r="K50" s="21" t="s">
+      <c r="L50" t="s">
         <v>445</v>
       </c>
-      <c r="L50" t="s">
-        <v>446</v>
-      </c>
       <c r="M50" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N50" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="N50" s="11" t="s">
-        <v>367</v>
-      </c>
       <c r="O50" s="11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="P50" s="17" t="str">
         <f t="shared" ref="P50" si="5">IF(O50&lt;&gt;"Yes","","New funding opportunity added: "&amp;D50)</f>
@@ -5051,53 +5149,53 @@
         <v>FORTHCOMING</v>
       </c>
       <c r="B51" t="s">
+        <v>446</v>
+      </c>
+      <c r="C51" t="s">
         <v>447</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>448</v>
-      </c>
-      <c r="D51" t="s">
-        <v>449</v>
       </c>
       <c r="E51" t="s">
         <v>32</v>
       </c>
       <c r="F51" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="G51" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="H51" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="I51" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="J51" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="J51" s="2" t="s">
+      <c r="K51" s="21" t="s">
+        <v>474</v>
+      </c>
+      <c r="L51" t="s">
         <v>454</v>
       </c>
-      <c r="K51" s="21" t="s">
-        <v>455</v>
-      </c>
-      <c r="L51" t="s">
-        <v>456</v>
-      </c>
       <c r="M51" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="N51" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O51" s="11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="P51" s="17" t="str">
-        <f t="shared" ref="P51" si="7">IF(O51&lt;&gt;"Yes","","New funding opportunity added: "&amp;D51)</f>
+        <f t="shared" ref="P51:P52" si="7">IF(O51&lt;&gt;"Yes","","New funding opportunity added: "&amp;D51)</f>
         <v>New funding opportunity added: International Fellowships 2027</v>
       </c>
       <c r="Q51" s="20" t="str">
-        <f t="shared" ref="Q51" si="8">IF(O51&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D51&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C51&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B51),TEXT(B51,"d mmmm yyyy"),B51)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F51&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G51&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H51&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I51&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K51&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+        <f t="shared" ref="Q51:Q52" si="8">IF(O51&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D51&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C51&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B51),TEXT(B51,"d mmmm yyyy"),B51)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F51&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G51&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H51&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I51&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K51&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **International Fellowships 2027**
@@ -5107,7 +5205,7 @@
 Who can apply: International ECRs based outside the UK; normally ≤5 years active full-time postdoctoral experience. Applicant must have/complete PhD by final awards stage, must not hold UK citizenship, and generally must not have lived/worked/researched in UK during previous 12 months. UK Sponsor required. For 2027, max. 8 applications per UK institution.
 Why it may be relevant to Statistics: Opportunity to recruit an international ECR to Glasgow for two years. Mathematics is explicitly within Royal Society remit; potentially relevant across Statistics research areas. Glasgow Statistics academics can act as UK Sponsors.
 Themes: All research areas; ECR; International; Fellowship
-Official opportunity: https://www.thebritishacademy.ac.uk/documents/6283/International_Fellowships_2027_-_FAQs.pdf?utm_source=chatgpt.com
+Official opportunity: https://www.thebritishacademy.ac.uk/documents/6283/International_Fellowships_2027_-_FAQs.pdf
 Funding Finder: https://uofgstats.github.io/research-and-scholarship/
 Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
 Best wishes,
@@ -5118,32 +5216,175 @@
         <v>46296</v>
       </c>
     </row>
+    <row r="52" spans="1:18" ht="75">
+      <c r="A52" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B52),B52&lt;TODAY()),"DEADLINE PASSED",N52)</f>
+        <v>OPEN</v>
+      </c>
+      <c r="B52" t="s">
+        <v>455</v>
+      </c>
+      <c r="C52" t="s">
+        <v>456</v>
+      </c>
+      <c r="D52" t="s">
+        <v>261</v>
+      </c>
+      <c r="E52" t="s">
+        <v>462</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="K52" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="M52" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N52" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="O52" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="P52" s="17" t="str">
+        <f t="shared" si="7"/>
+        <v>New funding opportunity added: What Works Centre for a climate resilient UK</v>
+      </c>
+      <c r="Q52" s="20" t="str">
+        <f t="shared" si="8"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**What Works Centre for a climate resilient UK**
+Funder: ESRC / UKRI, co-funded by Defra
+Deadline: 15 December 2026, 16:00
+Funding and duration: Up to £21.1m funder contribution; 44 months; single award; 80% FEC (with some exceptions at 100%). Must start by 1 August 2027.
+Who can apply: Researchers based at UK research organisations eligible for UKRI/ESRC funding. At least one project co-lead from a UK business, third-sector or government organisation is required.
+Why it may be relevant to Statistics: Major interdisciplinary opportunity with a strong methodological component, explicitly including robust evaluation, experimental and quasi-experimental methods, and causal reasoning, with applications including wildfire, drought, flooding and extreme heat.
+Themes: Climate resilience; environmental statistics; causal inference; evaluation; extremes; interdisciplinary research
+Official opportunity: https://www.ukri.org/opportunity/what-works-centre-for-a-climate-resilient-uk/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R52" s="13">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="105">
+      <c r="A53" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B53),B53&lt;TODAY()),"DEADLINE PASSED",N53)</f>
+        <v>OPEN</v>
+      </c>
+      <c r="B53" t="s">
+        <v>465</v>
+      </c>
+      <c r="C53" t="s">
+        <v>466</v>
+      </c>
+      <c r="D53" t="s">
+        <v>467</v>
+      </c>
+      <c r="E53" t="s">
+        <v>85</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="K53" s="21" t="s">
+        <v>473</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M53" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="N53" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="O53" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="P53" s="17" t="str">
+        <f t="shared" ref="P53" si="9">IF(O53&lt;&gt;"Yes","","New funding opportunity added: "&amp;D53)</f>
+        <v>New funding opportunity added: NERC urgency funding</v>
+      </c>
+      <c r="Q53" s="20" t="str">
+        <f t="shared" ref="Q53" si="10">IF(O53&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D53&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C53&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B53),TEXT(B53,"d mmmm yyyy"),B53)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F53&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G53&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H53&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I53&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K53&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**NERC urgency funding**
+Funder: NERC / UKRI
+Deadline: Open – no fixed deadline
+Funding and duration: Up to £100,000 FEC (NERC funds 80%); up to 1 year
+Who can apply: Researchers at UK organisations eligible for NERC funding. Must respond to an unexpected, transient environmental event; outline required within 4 weeks of the event starting. Applicants cannot have been PL/PcL on another full application to this scheme in the previous 2 years.
+Why it may be relevant to Statistics: Strong fit for environmental statistics and extremes, supporting rapid research following unexpected events such as droughts, floods and earthquakes, including collection and initial analysis of critical early data.
+Themes: Environmental statistics; Extremes; Climate &amp; environment; Urgency funding
+Official opportunity: https://www.ukri.org/opportunity/nerc-urgency-funding-open/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R53" s="13">
+        <v>46297</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A42 A50:A51">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>$A2="OPEN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="2">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>$A2="FORTHCOMING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="3">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>LEFT($A2,6)="CLOSED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="4">
+    <cfRule type="expression" dxfId="13" priority="4">
       <formula>$A2="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A51">
-    <cfRule type="expression" dxfId="7" priority="5">
+  <conditionalFormatting sqref="A2:A53">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>$A2="OPEN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>$A2="FORTHCOMING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>LEFT($A2,6)="CLOSED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="8">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>$A2="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5160,11 +5401,12 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="K50" r:id="rId1" xr:uid="{983CD2BB-548A-CA46-B886-1D5A7F03FD6A}"/>
-    <hyperlink ref="K51" r:id="rId2" xr:uid="{0A543A7C-0D01-4D47-8579-515FA800D65F}"/>
+    <hyperlink ref="K52" r:id="rId2" xr:uid="{CEDBB7D3-D861-6348-9912-50FD352C627E}"/>
+    <hyperlink ref="K53" r:id="rId3" xr:uid="{5E871FF8-6856-3F46-A97A-BF5C75823330}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5197,7 +5439,7 @@
         <v>333</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45">
@@ -5333,7 +5575,7 @@
         <v>360</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="57" customHeight="1">
@@ -5349,7 +5591,7 @@
         <v>353</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15">

</xml_diff>

<commit_message>
opportunity update, data fixed
</commit_message>
<xml_diff>
--- a/Funding_Finder_for_Statistics_FFS.xlsx
+++ b/Funding_Finder_for_Statistics_FFS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielacastrocamilo/Dropbox/Glasgow/Admin/ResearchLead4Statistics/research-and-scholarship/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F9CFF1-066D-694B-A27A-E29F5ADD2043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0521FA-E7E7-454A-B185-C5DBF0BFFBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="592">
   <si>
     <t>Status</t>
   </si>
@@ -816,15 +816,9 @@
     <t>Oct 2026</t>
   </si>
   <si>
-    <t>UKRI / NERC</t>
-  </si>
-  <si>
     <t>What Works Centre for a climate resilient UK</t>
   </si>
   <si>
-    <t>Centre / evidence synthesis</t>
-  </si>
-  <si>
     <t>NERC Climate Adaptation ICURe Discover</t>
   </si>
   <si>
@@ -1515,24 +1509,6 @@
     <t>https://www.lms.ac.uk/grants/lms-inclusion-and-diversity-fund</t>
   </si>
   <si>
-    <t>15 Dec 2026 4pm</t>
-  </si>
-  <si>
-    <t>Up to £21.1m funder contribution; 44 months; one award</t>
-  </si>
-  <si>
-    <t>UK research organisations eligible for ESRC funding; interdisciplinary centre-scale application. At least one project co-lead must be from UK business, third sector or government.</t>
-  </si>
-  <si>
-    <t>Strong scope for environmental statistics, climate/extremes modelling, causal inference and evaluation, evidence synthesis and uncertainty quantification within climate adaptation research.</t>
-  </si>
-  <si>
-    <t>Climate resilience; Environmental statistics; Extremes; Causal inference; Evaluation; Interdisciplinary</t>
-  </si>
-  <si>
-    <t>Demand management applies. Check UofG internal selection/deadline. Large interdisciplinary consortium required, including a non-academic co-lead.</t>
-  </si>
-  <si>
     <t>Glasgow Mathematical Journal Trust</t>
   </si>
   <si>
@@ -1666,6 +1642,174 @@
   </si>
   <si>
     <t>Research and Scholarship</t>
+  </si>
+  <si>
+    <t>Heilbronn Institute for Mathematical Research (HIMR)</t>
+  </si>
+  <si>
+    <t>HIMR</t>
+  </si>
+  <si>
+    <t>08/11/2026 23:59 GMT</t>
+  </si>
+  <si>
+    <t>Heilbronn Research Fellowships 2027</t>
+  </si>
+  <si>
+    <t>Postdoctoral research fellowship</t>
+  </si>
+  <si>
+    <t>3 years; salary approximately £46,874–£52,517 per year (London weighting where applicable)</t>
+  </si>
+  <si>
+    <t>Researchers in relevant mathematical sciences, including Statistics, probability and data science. Restricted to UK residents who are UK or dual UK nationals and eligible for national security clearance. Appointments at Bristol, Imperial, King's College London, UCL or Manchester.</t>
+  </si>
+  <si>
+    <t>Excellent postdoctoral career opportunity for eligible Statistics PhD graduates and ECRs, particularly those working in probability, statistical methodology, data science and mathematical research.</t>
+  </si>
+  <si>
+    <t>Statistics; Probability; Data science; ECR; Postdoctoral fellowship; Mathematical sciences</t>
+  </si>
+  <si>
+    <t>Requires national security clearance and includes classified research alongside independent research. Applicants submit CV, cover letter, one-page research statement and three references via MathJobs. Interviews expected 11–13 January 2027.</t>
+  </si>
+  <si>
+    <t>https://heilbronn.ac.uk/fellowships/</t>
+  </si>
+  <si>
+    <t>Rolling – verify</t>
+  </si>
+  <si>
+    <t>HIMR Small Grant Call</t>
+  </si>
+  <si>
+    <t>Research activity / event grant</t>
+  </si>
+  <si>
+    <t>Typically up to £5,000; applications up to £10,000 or exceptionally more considered</t>
+  </si>
+  <si>
+    <t>Researchers proposing activities supporting UK mathematical research and the mathematical sciences community; confirm current applicant eligibility</t>
+  </si>
+  <si>
+    <t>Supports Statistics workshops, conferences, research networks, collaborative activities, visiting researchers and PhD student development</t>
+  </si>
+  <si>
+    <t>Statistics; Mathematical sciences; Workshops; Research collaboration; ECR; Training</t>
+  </si>
+  <si>
+    <t>Flexible small-scale support for activities that may not be eligible for other funding. Historical guidance indicates rolling applications; confirm current arrangements</t>
+  </si>
+  <si>
+    <t>https://heilbronn.ac.uk/small-grants-call/</t>
+  </si>
+  <si>
+    <t>HIMR Focused Research Grants</t>
+  </si>
+  <si>
+    <t>Focused research event grant</t>
+  </si>
+  <si>
+    <t>Project-dependent; current award limit not verified</t>
+  </si>
+  <si>
+    <t>Groups of researchers proposing focused mathematical research activities; confirm current eligibility</t>
+  </si>
+  <si>
+    <t>Could fund focused research meetings addressing open problems in statistical methodology, probability, extremes, spatial statistics or computational statistics</t>
+  </si>
+  <si>
+    <t>Statistics; Mathematical sciences; Focused research; Workshops; Collaboration</t>
+  </si>
+  <si>
+    <t>Separate from the Small Grant Call. Designed for focused research meetings. Monitor the next application round and confirm award limits</t>
+  </si>
+  <si>
+    <t>https://heilbronn.ac.uk/frg/</t>
+  </si>
+  <si>
+    <t>Not confirmed</t>
+  </si>
+  <si>
+    <t>HIMR International Visitors Scheme</t>
+  </si>
+  <si>
+    <t>International research visit / collaboration</t>
+  </si>
+  <si>
+    <t>Financial support for eligible international research visits; amount and duration not verified</t>
+  </si>
+  <si>
+    <t>Scheme centred on leading international mathematicians with research interests shared by Heilbronn Fellows; confirm whether applications must be initiated by a Fellow</t>
+  </si>
+  <si>
+    <t>Potentially supports international collaboration in Statistics, probability and related mathematical sciences, particularly through partnerships with Heilbronn Fellows</t>
+  </si>
+  <si>
+    <t>Statistics; Mathematical sciences; International collaboration; Research visits; Networking</t>
+  </si>
+  <si>
+    <t>Restricted relevance: establish a connection with a Heilbronn Fellow before considering an application. Not a general-purpose Glasgow visitor grant</t>
+  </si>
+  <si>
+    <t>ELIGIBILITY TO VERIFY</t>
+  </si>
+  <si>
+    <t>EPSRC SUM4Products Network+</t>
+  </si>
+  <si>
+    <t>SUM4Products Research Project Scheme</t>
+  </si>
+  <si>
+    <t>ndustry–academia research grant</t>
+  </si>
+  <si>
+    <t>Up to 3 months full-time or 6 months part-time; researcher costs funded at 80% FEC, normally with industry co-funding</t>
+  </si>
+  <si>
+    <t>UK university academic mathematical scientist as project lead, working with at least one named industry partner. Researcher may be an RA or eligible PhD student</t>
+  </si>
+  <si>
+    <t>SUM4Products Mini-grants</t>
+  </si>
+  <si>
+    <t>Travel / networking / activity grant</t>
+  </si>
+  <si>
+    <t>Normally up to £500; larger requests may be discussed</t>
+  </si>
+  <si>
+    <t>UK-based SUM4Products network members, generally with previous participation. PhD students eligible with supervisor support. UK travel only</t>
+  </si>
+  <si>
+    <t>Supports applied statistical modelling, uncertainty quantification, experimental design and data-driven research addressing industrial challenges</t>
+  </si>
+  <si>
+    <t>Supports Statistics researchers and PhD students engaging with industry through workshops, conferences, site visits and collaborative activities</t>
+  </si>
+  <si>
+    <t>Industrial collaboration; Applied statistics; Mathematical modelling; Research; Knowledge exchange</t>
+  </si>
+  <si>
+    <t>2026 EOI deadline passed. Monitor next round. Requires an industry partner; no funding for academic lead time when employing a researcher. Projects must relate to formulated products</t>
+  </si>
+  <si>
+    <t>https://www.sum4products.co.uk/research-project-scheme</t>
+  </si>
+  <si>
+    <t>SUM4Products / EPSRC</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Industrial collaboration; Networking; Travel; Workshops; PhD; Knowledge exchange</t>
+  </si>
+  <si>
+    <t>Rolling applications; decisions within 4 weeks. Must demonstrate a direct connection to the mathematics of formulated products. Industry co-funding normally expected for co-hosted activities</t>
+  </si>
+  <si>
+    <t>https://www.sum4products.co.uk/flexible-funding</t>
   </si>
 </sst>
 </file>
@@ -1775,7 +1919,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1870,8 +2014,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0E7F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1916,12 +2066,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2006,62 +2165,24 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <font>
         <b/>
@@ -2245,6 +2366,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC0E7F6"/>
       <color rgb="FF1F4E78"/>
       <color rgb="FFFFF2CC"/>
     </mruColors>
@@ -2261,8 +2383,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R56" totalsRowShown="0">
-  <autoFilter ref="A1:R56" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingFinderStats" displayName="FundingFinderStats" ref="A1:R55" totalsRowShown="0">
+  <autoFilter ref="A1:R55" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Status">
       <calculatedColumnFormula>IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",N2)</calculatedColumnFormula>
@@ -2282,7 +2404,7 @@
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Manual status"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notify?"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Email subject"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Email body" dataDxfId="20">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Email body" dataDxfId="16">
       <calculatedColumnFormula>IF(O2&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D2&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C2&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B2),TEXT(B2,"d mmmm yyyy"),B2)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F2&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G2&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H2&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I2&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K2&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Notification date"/>
@@ -2486,8 +2608,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:R66"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -2547,27 +2669,27 @@
         <v>11</v>
       </c>
       <c r="M1" s="14" t="s">
+        <v>353</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>456</v>
+      </c>
+      <c r="O1" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="P1" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="N1" s="14" t="s">
-        <v>458</v>
-      </c>
-      <c r="O1" s="14" t="s">
+      <c r="Q1" s="14" t="s">
         <v>356</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="R1" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="Q1" s="14" t="s">
-        <v>358</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="30">
+    </row>
+    <row r="2" spans="1:18" ht="32">
       <c r="A2" s="8" t="str">
-        <f t="shared" ref="A2:A42" ca="1" si="0">IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",N2)</f>
+        <f t="shared" ref="A2:A41" ca="1" si="0">IF(AND(ISNUMBER(B2),B2&lt;TODAY()),"DEADLINE PASSED",N2)</f>
         <v>DEADLINE PASSED</v>
       </c>
       <c r="B2" s="3">
@@ -2604,16 +2726,16 @@
         <v>12</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P2" s="12" t="str">
-        <f t="shared" ref="P2:P42" si="1">IF(O2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</f>
+        <f t="shared" ref="P2:P41" si="1">IF(O2&lt;&gt;"Yes","","New funding opportunity added: "&amp;D2)</f>
         <v/>
       </c>
       <c r="Q2" s="20" t="str">
@@ -2621,10 +2743,10 @@
         <v/>
       </c>
       <c r="R2" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="32">
       <c r="A3" s="8" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>DEADLINE PASSED</v>
@@ -2663,27 +2785,27 @@
         <v>21</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O3" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P3" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q3" s="20" t="str">
-        <f t="shared" ref="Q3:Q49" si="2">IF(O3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D3&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+        <f t="shared" ref="Q3:Q48" si="2">IF(O3&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D3&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C3&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B3),TEXT(B3,"d mmmm yyyy"),B3)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F3&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G3&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H3&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I3&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K3&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v/>
       </c>
       <c r="R3" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="32">
       <c r="A4" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>DEADLINE PASSED</v>
@@ -2722,13 +2844,13 @@
         <v>12</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O4" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P4" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2739,13 +2861,13 @@
         <v/>
       </c>
       <c r="R4" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="48">
       <c r="A5" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>DEADLINE PASSED</v>
       </c>
       <c r="B5" s="3">
         <v>46304</v>
@@ -2781,13 +2903,13 @@
         <v>21</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P5" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2798,13 +2920,13 @@
         <v/>
       </c>
       <c r="R5" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="32">
       <c r="A6" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>DEADLINE PASSED</v>
       </c>
       <c r="B6" s="3">
         <v>46310</v>
@@ -2840,13 +2962,13 @@
         <v>12</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="P6" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2871,13 +2993,13 @@
 Research Lead for Statistics</v>
       </c>
       <c r="R6" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="32">
       <c r="A7" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>DEADLINE PASSED</v>
       </c>
       <c r="B7" s="3">
         <v>46310</v>
@@ -2913,13 +3035,13 @@
         <v>12</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P7" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2930,13 +3052,13 @@
         <v/>
       </c>
       <c r="R7" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="48">
       <c r="A8" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>DEADLINE PASSED</v>
       </c>
       <c r="B8" s="3">
         <v>46310</v>
@@ -2972,13 +3094,13 @@
         <v>12</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P8" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2989,10 +3111,10 @@
         <v/>
       </c>
       <c r="R8" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="32">
       <c r="A9" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3031,13 +3153,13 @@
         <v>67</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P9" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3048,10 +3170,10 @@
         <v/>
       </c>
       <c r="R9" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="32">
       <c r="A10" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3090,13 +3212,13 @@
         <v>67</v>
       </c>
       <c r="M10" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N10" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O10" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P10" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3107,10 +3229,10 @@
         <v/>
       </c>
       <c r="R10" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="32">
       <c r="A11" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3149,13 +3271,13 @@
         <v>67</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P11" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3166,10 +3288,10 @@
         <v/>
       </c>
       <c r="R11" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="48">
       <c r="A12" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3208,13 +3330,13 @@
         <v>67</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P12" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3225,10 +3347,10 @@
         <v/>
       </c>
       <c r="R12" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="32">
       <c r="A13" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3267,13 +3389,13 @@
         <v>67</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P13" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3284,10 +3406,10 @@
         <v/>
       </c>
       <c r="R13" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="48">
       <c r="A14" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3326,13 +3448,13 @@
         <v>67</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P14" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3343,10 +3465,10 @@
         <v/>
       </c>
       <c r="R14" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="48">
       <c r="A15" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3385,13 +3507,13 @@
         <v>124</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P15" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3402,10 +3524,10 @@
         <v/>
       </c>
       <c r="R15" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="32">
       <c r="A16" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3444,13 +3566,13 @@
         <v>67</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P16" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3461,10 +3583,10 @@
         <v/>
       </c>
       <c r="R16" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="32">
       <c r="A17" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3503,13 +3625,13 @@
         <v>124</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P17" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3520,10 +3642,10 @@
         <v/>
       </c>
       <c r="R17" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="48">
       <c r="A18" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3562,13 +3684,13 @@
         <v>124</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P18" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3579,10 +3701,10 @@
         <v/>
       </c>
       <c r="R18" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="48">
       <c r="A19" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3621,13 +3743,13 @@
         <v>12</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P19" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3638,10 +3760,10 @@
         <v/>
       </c>
       <c r="R19" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="48">
       <c r="A20" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3680,13 +3802,13 @@
         <v>67</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P20" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3697,10 +3819,10 @@
         <v/>
       </c>
       <c r="R20" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="32">
       <c r="A21" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3739,13 +3861,13 @@
         <v>67</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P21" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3756,10 +3878,10 @@
         <v/>
       </c>
       <c r="R21" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="32">
       <c r="A22" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3798,13 +3920,13 @@
         <v>12</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P22" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3815,10 +3937,10 @@
         <v/>
       </c>
       <c r="R22" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="32">
       <c r="A23" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3857,13 +3979,13 @@
         <v>12</v>
       </c>
       <c r="M23" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N23" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O23" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P23" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3874,10 +3996,10 @@
         <v/>
       </c>
       <c r="R23" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="32">
       <c r="A24" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3916,13 +4038,13 @@
         <v>12</v>
       </c>
       <c r="M24" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P24" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3933,10 +4055,10 @@
         <v/>
       </c>
       <c r="R24" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="32">
       <c r="A25" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -3975,13 +4097,13 @@
         <v>12</v>
       </c>
       <c r="M25" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P25" s="12" t="str">
         <f t="shared" si="1"/>
@@ -3992,10 +4114,10 @@
         <v/>
       </c>
       <c r="R25" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="32">
       <c r="A26" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4034,13 +4156,13 @@
         <v>12</v>
       </c>
       <c r="M26" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P26" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4051,10 +4173,10 @@
         <v/>
       </c>
       <c r="R26" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="32">
       <c r="A27" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4093,13 +4215,13 @@
         <v>12</v>
       </c>
       <c r="M27" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P27" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4110,10 +4232,10 @@
         <v/>
       </c>
       <c r="R27" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="48">
       <c r="A28" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4152,13 +4274,13 @@
         <v>124</v>
       </c>
       <c r="M28" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P28" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4169,10 +4291,10 @@
         <v/>
       </c>
       <c r="R28" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="48">
       <c r="A29" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4211,13 +4333,13 @@
         <v>230</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P29" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4228,10 +4350,10 @@
         <v/>
       </c>
       <c r="R29" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="32">
       <c r="A30" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4270,13 +4392,13 @@
         <v>230</v>
       </c>
       <c r="M30" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P30" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4287,10 +4409,10 @@
         <v/>
       </c>
       <c r="R30" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="31" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="32">
       <c r="A31" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4329,13 +4451,13 @@
         <v>230</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P31" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4346,10 +4468,10 @@
         <v/>
       </c>
       <c r="R31" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="64">
       <c r="A32" s="9" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>OPEN</v>
@@ -4388,13 +4510,13 @@
         <v>230</v>
       </c>
       <c r="M32" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P32" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4405,10 +4527,10 @@
         <v/>
       </c>
       <c r="R32" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="60">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="64">
       <c r="A33" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
@@ -4447,13 +4569,13 @@
         <v>258</v>
       </c>
       <c r="M33" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N33" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N33" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O33" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P33" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4464,19 +4586,19 @@
         <v/>
       </c>
       <c r="R33" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="60">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="32">
       <c r="A34" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>OPEN</v>
+        <v>FORTHCOMING</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>493</v>
+        <v>259</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>260</v>
+        <v>142</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>261</v>
@@ -4485,92 +4607,78 @@
         <v>262</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>494</v>
+        <v>263</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>495</v>
+        <v>264</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>496</v>
+        <v>265</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>497</v>
+        <v>266</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>498</v>
+        <v>267</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>257</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>134</v>
+        <v>258</v>
       </c>
       <c r="M34" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N34" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N34" s="11" t="s">
-        <v>361</v>
-      </c>
       <c r="O34" s="11" t="s">
-        <v>429</v>
+        <v>374</v>
       </c>
       <c r="P34" s="12" t="str">
         <f t="shared" si="1"/>
-        <v>New funding opportunity added: What Works Centre for a climate resilient UK</v>
+        <v/>
       </c>
       <c r="Q34" s="20" t="str">
         <f t="shared" si="2"/>
-        <v>Hello,
-A new funding opportunity has been added to the Funding Finder for Statistics.
-**What Works Centre for a climate resilient UK**
-Funder: UKRI / NERC
-Deadline: 15 Dec 2026 4pm
-Funding and duration: Up to £21.1m funder contribution; 44 months; one award
-Who can apply: UK research organisations eligible for ESRC funding; interdisciplinary centre-scale application. At least one project co-lead must be from UK business, third sector or government.
-Why it may be relevant to Statistics: Strong scope for environmental statistics, climate/extremes modelling, causal inference and evaluation, evidence synthesis and uncertainty quantification within climate adaptation research.
-Themes: Climate resilience; Environmental statistics; Extremes; Causal inference; Evaluation; Interdisciplinary
-Official opportunity: https://www.ukri.org/apply-for-funding/future-research-and-innovation-funding-opportunities/
-Funding Finder: https://uofgstats.github.io/research-and-scholarship/
-Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
-Best wishes,
-Daniela &amp; Vinny
-Research Lead for Statistics</v>
+        <v/>
       </c>
       <c r="R34" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="48">
       <c r="A35" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>257</v>
@@ -4579,13 +4687,13 @@
         <v>258</v>
       </c>
       <c r="M35" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N35" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N35" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O35" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P35" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4596,40 +4704,40 @@
         <v/>
       </c>
       <c r="R35" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="32">
       <c r="A36" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>134</v>
+        <v>276</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>257</v>
@@ -4638,13 +4746,13 @@
         <v>258</v>
       </c>
       <c r="M36" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N36" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N36" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O36" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P36" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4655,40 +4763,40 @@
         <v/>
       </c>
       <c r="R36" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="32">
       <c r="A37" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>278</v>
+        <v>134</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>257</v>
@@ -4697,13 +4805,13 @@
         <v>258</v>
       </c>
       <c r="M37" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N37" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N37" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O37" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P37" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4714,40 +4822,40 @@
         <v/>
       </c>
       <c r="R37" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="32">
       <c r="A38" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>134</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>288</v>
+        <v>23</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>257</v>
@@ -4756,13 +4864,13 @@
         <v>258</v>
       </c>
       <c r="M38" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N38" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N38" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O38" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P38" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4773,40 +4881,40 @@
         <v/>
       </c>
       <c r="R38" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="39" spans="1:18" ht="30">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="32">
       <c r="A39" s="10" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>134</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>257</v>
@@ -4815,13 +4923,13 @@
         <v>258</v>
       </c>
       <c r="M39" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N39" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N39" s="11" t="s">
-        <v>362</v>
-      </c>
       <c r="O39" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P39" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4832,55 +4940,55 @@
         <v/>
       </c>
       <c r="R39" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="40" spans="1:18" ht="30">
-      <c r="A40" s="10" t="str">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="48">
+      <c r="A40" s="8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>FORTHCOMING</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>300</v>
+        <v>DEADLINE PASSED</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46283</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>134</v>
+        <v>305</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>32</v>
+        <v>307</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>257</v>
+        <v>313</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>258</v>
+        <v>124</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P40" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4891,55 +4999,55 @@
         <v/>
       </c>
       <c r="R40" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="41" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="64">
       <c r="A41" s="8" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>DEADLINE PASSED</v>
       </c>
       <c r="B41" s="3">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>124</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P41" s="12" t="str">
         <f t="shared" si="1"/>
@@ -4950,58 +5058,58 @@
         <v/>
       </c>
       <c r="R41" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" ht="45">
-      <c r="A42" s="8" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>DEADLINE PASSED</v>
-      </c>
-      <c r="B42" s="3">
-        <v>46286</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>318</v>
+        <v>428</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="48">
+      <c r="A42" s="18" t="str">
+        <f t="shared" ref="A42:A50" ca="1" si="3">IF(AND(ISNUMBER(B42),B42&lt;TODAY()),"DEADLINE PASSED",N42)</f>
+        <v>CLOSED – monitor recurrence</v>
+      </c>
+      <c r="B42" t="s">
+        <v>363</v>
+      </c>
+      <c r="C42" t="s">
+        <v>305</v>
+      </c>
+      <c r="D42" t="s">
+        <v>364</v>
+      </c>
+      <c r="E42" t="s">
+        <v>365</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>319</v>
+        <v>366</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>320</v>
+        <v>367</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>321</v>
+        <v>368</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>322</v>
+        <v>369</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>323</v>
+        <v>370</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="M42" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N42" s="11" t="s">
-        <v>364</v>
+        <v>371</v>
+      </c>
+      <c r="L42" t="s">
+        <v>372</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>373</v>
+      </c>
+      <c r="N42" s="16" t="s">
+        <v>361</v>
       </c>
       <c r="O42" s="11" t="s">
-        <v>376</v>
-      </c>
-      <c r="P42" s="12" t="str">
-        <f t="shared" si="1"/>
+        <v>374</v>
+      </c>
+      <c r="P42" s="17" t="str">
+        <f t="shared" ref="P42:P48" si="4">IF(O42&lt;&gt;"Yes","","New funding opportunity added: "&amp;D42)</f>
         <v/>
       </c>
       <c r="Q42" s="20" t="str">
@@ -5009,58 +5117,58 @@
         <v/>
       </c>
       <c r="R42" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="43" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="48">
       <c r="A43" s="18" t="str">
-        <f t="shared" ref="A43:A51" ca="1" si="3">IF(AND(ISNUMBER(B43),B43&lt;TODAY()),"DEADLINE PASSED",N43)</f>
+        <f t="shared" ca="1" si="3"/>
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B43" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C43" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D43" t="s">
+        <v>375</v>
+      </c>
+      <c r="E43" t="s">
+        <v>376</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E43" t="s">
-        <v>367</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="G43" s="2" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="H43" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="J43" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="L43" t="s">
         <v>372</v>
       </c>
-      <c r="K43" s="2" t="s">
+      <c r="M43" s="16" t="s">
         <v>373</v>
       </c>
-      <c r="L43" t="s">
+      <c r="N43" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="O43" s="11" t="s">
         <v>374</v>
       </c>
-      <c r="M43" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="N43" s="16" t="s">
-        <v>363</v>
-      </c>
-      <c r="O43" s="11" t="s">
-        <v>376</v>
-      </c>
       <c r="P43" s="17" t="str">
-        <f t="shared" ref="P43:P49" si="4">IF(O43&lt;&gt;"Yes","","New funding opportunity added: "&amp;D43)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="Q43" s="20" t="str">
@@ -5068,55 +5176,55 @@
         <v/>
       </c>
       <c r="R43" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="44" spans="1:18" ht="45">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="48">
       <c r="A44" s="18" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B44" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="C44" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D44" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E44" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="J44" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="L44" t="s">
         <v>372</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="M44" s="16" t="s">
         <v>373</v>
       </c>
-      <c r="L44" t="s">
+      <c r="N44" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="O44" s="11" t="s">
         <v>374</v>
-      </c>
-      <c r="M44" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="N44" s="16" t="s">
-        <v>363</v>
-      </c>
-      <c r="O44" s="11" t="s">
-        <v>376</v>
       </c>
       <c r="P44" s="17" t="str">
         <f t="shared" si="4"/>
@@ -5127,55 +5235,55 @@
         <v/>
       </c>
       <c r="R44" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="45" spans="1:18" ht="45">
-      <c r="A45" s="18" t="str">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="80">
+      <c r="A45" s="19" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>CLOSED – monitor recurrence</v>
+        <v>FORTHCOMING</v>
       </c>
       <c r="B45" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C45" t="s">
-        <v>307</v>
+        <v>389</v>
       </c>
       <c r="D45" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="E45" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="K45" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="L45" t="s">
+        <v>12</v>
+      </c>
+      <c r="M45" s="16" t="s">
         <v>373</v>
       </c>
-      <c r="L45" t="s">
+      <c r="N45" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="O45" s="11" t="s">
         <v>374</v>
-      </c>
-      <c r="M45" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="N45" s="16" t="s">
-        <v>363</v>
-      </c>
-      <c r="O45" s="11" t="s">
-        <v>376</v>
       </c>
       <c r="P45" s="17" t="str">
         <f t="shared" si="4"/>
@@ -5186,55 +5294,55 @@
         <v/>
       </c>
       <c r="R45" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" ht="60">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="64">
       <c r="A46" s="19" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B46" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C46" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D46" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="E46" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="L46" t="s">
         <v>12</v>
       </c>
       <c r="M46" s="16" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="N46" s="16" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="O46" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P46" s="17" t="str">
         <f t="shared" si="4"/>
@@ -5245,55 +5353,55 @@
         <v/>
       </c>
       <c r="R46" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" ht="60">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="64">
       <c r="A47" s="19" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>FORTHCOMING</v>
       </c>
       <c r="B47" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C47" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D47" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E47" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="L47" t="s">
         <v>12</v>
       </c>
       <c r="M47" s="16" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="N47" s="16" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="O47" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P47" s="17" t="str">
         <f t="shared" si="4"/>
@@ -5304,55 +5412,55 @@
         <v/>
       </c>
       <c r="R47" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="48" spans="1:18" ht="60">
-      <c r="A48" s="19" t="str">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="64">
+      <c r="A48" s="18" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>FORTHCOMING</v>
+        <v>CLOSED – monitor recurrence</v>
       </c>
       <c r="B48" t="s">
-        <v>390</v>
+        <v>363</v>
       </c>
       <c r="C48" t="s">
-        <v>391</v>
+        <v>414</v>
       </c>
       <c r="D48" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="E48" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="L48" t="s">
-        <v>12</v>
+        <v>423</v>
       </c>
       <c r="M48" s="16" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="N48" s="16" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="O48" s="11" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="P48" s="17" t="str">
         <f t="shared" si="4"/>
@@ -5363,121 +5471,62 @@
         <v/>
       </c>
       <c r="R48" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="49" spans="1:18" ht="60">
-      <c r="A49" s="18" t="str">
-        <f t="shared" ca="1" si="3"/>
-        <v>CLOSED – monitor recurrence</v>
-      </c>
-      <c r="B49" t="s">
-        <v>365</v>
-      </c>
-      <c r="C49" t="s">
-        <v>416</v>
-      </c>
-      <c r="D49" t="s">
-        <v>417</v>
-      </c>
-      <c r="E49" t="s">
-        <v>418</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="L49" t="s">
-        <v>425</v>
-      </c>
-      <c r="M49" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="N49" s="16" t="s">
-        <v>363</v>
-      </c>
-      <c r="O49" s="11" t="s">
-        <v>376</v>
-      </c>
-      <c r="P49" s="17" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="Q49" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="R49" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="50" spans="1:18" ht="60">
-      <c r="A50" s="8" t="str">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="80">
+      <c r="A49" s="8" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>OPEN</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B49" s="3">
         <v>46362</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C49" t="s">
+        <v>429</v>
+      </c>
+      <c r="D49" t="s">
+        <v>430</v>
+      </c>
+      <c r="E49" t="s">
         <v>431</v>
       </c>
-      <c r="D50" t="s">
+      <c r="F49" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="E50" t="s">
+      <c r="G49" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="H49" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="I49" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="J49" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="K49" s="21" t="s">
         <v>437</v>
       </c>
-      <c r="J50" s="2" t="s">
+      <c r="L49" t="s">
         <v>438</v>
       </c>
-      <c r="K50" s="21" t="s">
-        <v>439</v>
-      </c>
-      <c r="L50" t="s">
-        <v>440</v>
-      </c>
-      <c r="M50" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N50" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O50" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P50" s="17" t="str">
-        <f t="shared" ref="P50" si="5">IF(O50&lt;&gt;"Yes","","New funding opportunity added: "&amp;D50)</f>
+      <c r="M49" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N49" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O49" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P49" s="17" t="str">
+        <f t="shared" ref="P49" si="5">IF(O49&lt;&gt;"Yes","","New funding opportunity added: "&amp;D49)</f>
         <v>New funding opportunity added: Venture Scientist 100</v>
       </c>
-      <c r="Q50" s="20" t="str">
-        <f t="shared" ref="Q50" si="6">IF(O50&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D50&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C50&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B50),TEXT(B50,"d mmmm yyyy"),B50)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F50&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G50&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H50&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I50&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K50&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q49" s="20" t="str">
+        <f t="shared" ref="Q49" si="6">IF(O49&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D49&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C49&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B49),TEXT(B49,"d mmmm yyyy"),B49)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F49&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G49&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H49&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I49&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K49&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **Venture Scientist 100**
@@ -5494,63 +5543,63 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R50" s="13">
+      <c r="R49" s="13">
         <v>46296</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="120">
-      <c r="A51" s="8" t="str">
+    <row r="50" spans="1:18" ht="128">
+      <c r="A50" s="8" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>FORTHCOMING</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B50" t="s">
+        <v>439</v>
+      </c>
+      <c r="C50" t="s">
+        <v>440</v>
+      </c>
+      <c r="D50" t="s">
         <v>441</v>
       </c>
-      <c r="C51" t="s">
+      <c r="E50" t="s">
+        <v>32</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="D51" t="s">
+      <c r="G50" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="E51" t="s">
-        <v>32</v>
-      </c>
-      <c r="F51" s="2" t="s">
+      <c r="H50" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="I50" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="J50" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="K50" s="21" t="s">
+        <v>467</v>
+      </c>
+      <c r="L50" t="s">
         <v>447</v>
       </c>
-      <c r="J51" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="K51" s="21" t="s">
-        <v>469</v>
-      </c>
-      <c r="L51" t="s">
-        <v>449</v>
-      </c>
-      <c r="M51" s="11" t="s">
+      <c r="M50" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N50" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="N51" s="11" t="s">
-        <v>362</v>
-      </c>
-      <c r="O51" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P51" s="17" t="str">
-        <f t="shared" ref="P51:P52" si="7">IF(O51&lt;&gt;"Yes","","New funding opportunity added: "&amp;D51)</f>
+      <c r="O50" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P50" s="17" t="str">
+        <f t="shared" ref="P50:P51" si="7">IF(O50&lt;&gt;"Yes","","New funding opportunity added: "&amp;D50)</f>
         <v>New funding opportunity added: International Fellowships 2027</v>
       </c>
-      <c r="Q51" s="20" t="str">
-        <f t="shared" ref="Q51:Q52" si="8">IF(O51&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D51&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C51&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B51),TEXT(B51,"d mmmm yyyy"),B51)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F51&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G51&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H51&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I51&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K51&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q50" s="20" t="str">
+        <f t="shared" ref="Q50:Q51" si="8">IF(O50&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D50&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C50&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B50),TEXT(B50,"d mmmm yyyy"),B50)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F50&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G50&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H50&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I50&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K50&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **International Fellowships 2027**
@@ -5567,59 +5616,59 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R51" s="13">
+      <c r="R50" s="13">
         <v>46296</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="75">
-      <c r="A52" t="str">
-        <f ca="1">IF(AND(ISNUMBER(B52),B52&lt;TODAY()),"DEADLINE PASSED",N52)</f>
+    <row r="51" spans="1:18" ht="96">
+      <c r="A51" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B51),B51&lt;TODAY()),"DEADLINE PASSED",N51)</f>
         <v>OPEN</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B51" t="s">
+        <v>448</v>
+      </c>
+      <c r="C51" t="s">
+        <v>449</v>
+      </c>
+      <c r="D51" t="s">
+        <v>260</v>
+      </c>
+      <c r="E51" t="s">
+        <v>455</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="C52" t="s">
+      <c r="G51" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="D52" t="s">
-        <v>261</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="H51" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="K51" s="21" t="s">
         <v>457</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="K52" s="21" t="s">
-        <v>459</v>
-      </c>
-      <c r="M52" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N52" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O52" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P52" s="17" t="str">
+      <c r="M51" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N51" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O51" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P51" s="17" t="str">
         <f t="shared" si="7"/>
         <v>New funding opportunity added: What Works Centre for a climate resilient UK</v>
       </c>
-      <c r="Q52" s="20" t="str">
+      <c r="Q51" s="20" t="str">
         <f t="shared" si="8"/>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
@@ -5637,63 +5686,63 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R52" s="13">
+      <c r="R51" s="13">
         <v>46297</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="105">
-      <c r="A53" t="str">
-        <f ca="1">IF(AND(ISNUMBER(B53),B53&lt;TODAY()),"DEADLINE PASSED",N53)</f>
+    <row r="52" spans="1:18" ht="112">
+      <c r="A52" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B52),B52&lt;TODAY()),"DEADLINE PASSED",N52)</f>
         <v>OPEN</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B52" t="s">
+        <v>458</v>
+      </c>
+      <c r="C52" t="s">
+        <v>459</v>
+      </c>
+      <c r="D52" t="s">
         <v>460</v>
       </c>
-      <c r="C53" t="s">
+      <c r="E52" t="s">
+        <v>85</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="D53" t="s">
+      <c r="G52" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="E53" t="s">
-        <v>85</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="H52" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="I52" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="H53" s="2" t="s">
+      <c r="J52" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="K52" s="21" t="s">
         <v>466</v>
       </c>
-      <c r="J53" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="K53" s="21" t="s">
-        <v>468</v>
-      </c>
-      <c r="L53" s="2" t="s">
+      <c r="L52" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="M53" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N53" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O53" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P53" s="17" t="str">
-        <f t="shared" ref="P53:P54" si="9">IF(O53&lt;&gt;"Yes","","New funding opportunity added: "&amp;D53)</f>
+      <c r="M52" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N52" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O52" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P52" s="17" t="str">
+        <f t="shared" ref="P52:P53" si="9">IF(O52&lt;&gt;"Yes","","New funding opportunity added: "&amp;D52)</f>
         <v>New funding opportunity added: NERC urgency funding</v>
       </c>
-      <c r="Q53" s="20" t="str">
-        <f t="shared" ref="Q53:Q54" si="10">IF(O53&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D53&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C53&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B53),TEXT(B53,"d mmmm yyyy"),B53)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F53&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G53&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H53&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I53&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K53&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q52" s="20" t="str">
+        <f t="shared" ref="Q52:Q53" si="10">IF(O52&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D52&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C52&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B52),TEXT(B52,"d mmmm yyyy"),B52)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F52&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G52&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H52&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I52&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K52&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **NERC urgency funding**
@@ -5710,62 +5759,62 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R53" s="13">
+      <c r="R52" s="13">
         <v>46298</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="75">
-      <c r="A54" t="str">
-        <f ca="1">IF(AND(ISNUMBER(B54),B54&lt;TODAY()),"DEADLINE PASSED",N54)</f>
+    <row r="53" spans="1:18" ht="80">
+      <c r="A53" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B53),B53&lt;TODAY()),"DEADLINE PASSED",N53)</f>
         <v>OPEN</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B53" s="3">
         <v>46356</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C53" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="I53" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="H54" s="2" t="s">
+      <c r="J53" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="I54" s="2" t="s">
+      <c r="K53" s="21" t="s">
         <v>476</v>
       </c>
-      <c r="J54" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="K54" s="21" t="s">
-        <v>478</v>
-      </c>
-      <c r="L54" t="s">
+      <c r="L53" t="s">
         <v>12</v>
       </c>
-      <c r="M54" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N54" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O54" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P54" s="17" t="str">
+      <c r="M53" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N53" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O53" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P53" s="17" t="str">
         <f t="shared" si="9"/>
         <v>New funding opportunity added: LMS Emmy Noether Fellowships</v>
       </c>
-      <c r="Q54" s="20" t="str">
+      <c r="Q53" s="20" t="str">
         <f t="shared" si="10"/>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
@@ -5783,61 +5832,61 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R54" s="13"/>
-    </row>
-    <row r="55" spans="1:18" ht="30">
-      <c r="A55" t="str">
-        <f ca="1">IF(AND(ISNUMBER(B55),B55&lt;TODAY()),"DEADLINE PASSED",N55)</f>
+      <c r="R53" s="13"/>
+    </row>
+    <row r="54" spans="1:18" ht="32">
+      <c r="A54" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B54),B54&lt;TODAY()),"DEADLINE PASSED",N54)</f>
         <v>OPEN</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B54" s="3">
         <v>46356</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C54" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="F54" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="G54" t="s">
         <v>479</v>
       </c>
-      <c r="E55" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="F55" s="2" t="s">
+      <c r="H54" t="s">
         <v>480</v>
       </c>
-      <c r="G55" t="s">
+      <c r="I54" t="s">
         <v>481</v>
       </c>
-      <c r="H55" t="s">
+      <c r="J54" t="s">
         <v>482</v>
       </c>
-      <c r="I55" t="s">
+      <c r="K54" s="22" t="s">
         <v>483</v>
       </c>
-      <c r="J55" t="s">
-        <v>484</v>
-      </c>
-      <c r="K55" s="22" t="s">
-        <v>485</v>
-      </c>
-      <c r="L55" t="s">
+      <c r="L54" t="s">
         <v>12</v>
       </c>
-      <c r="M55" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N55" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O55" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P55" s="17" t="str">
-        <f t="shared" ref="P55" si="11">IF(O55&lt;&gt;"Yes","","New funding opportunity added: "&amp;D55)</f>
+      <c r="M54" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N54" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O54" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P54" s="17" t="str">
+        <f t="shared" ref="P54" si="11">IF(O54&lt;&gt;"Yes","","New funding opportunity added: "&amp;D54)</f>
         <v>New funding opportunity added: LMS Grace Chisholm Young Fellowship</v>
       </c>
-      <c r="Q55" s="20" t="str">
-        <f t="shared" ref="Q55" si="12">IF(O55&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D55&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C55&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B55),TEXT(B55,"d mmmm yyyy"),B55)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F55&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G55&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H55&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I55&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K55&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q54" s="20" t="str">
+        <f t="shared" ref="Q54" si="12">IF(O54&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D54&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C54&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B54),TEXT(B54,"d mmmm yyyy"),B54)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F54&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G54&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H54&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I54&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K54&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **LMS Grace Chisholm Young Fellowship**
@@ -5854,58 +5903,58 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R55" s="13"/>
-    </row>
-    <row r="56" spans="1:18" ht="30">
-      <c r="A56" t="str">
-        <f ca="1">IF(AND(ISNUMBER(B56),B56&lt;TODAY()),"DEADLINE PASSED",N56)</f>
+      <c r="R54" s="13"/>
+    </row>
+    <row r="55" spans="1:18" ht="32">
+      <c r="A55" t="str">
+        <f ca="1">IF(AND(ISNUMBER(B55),B55&lt;TODAY()),"DEADLINE PASSED",N55)</f>
         <v>OPEN</v>
       </c>
-      <c r="B56" s="3">
+      <c r="B55" s="3">
         <v>46372</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C55" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E55" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="F55" t="s">
+        <v>485</v>
+      </c>
+      <c r="G55" t="s">
         <v>486</v>
       </c>
-      <c r="E56" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="H55" t="s">
         <v>487</v>
       </c>
-      <c r="G56" t="s">
+      <c r="I55" t="s">
         <v>488</v>
       </c>
-      <c r="H56" t="s">
+      <c r="J55" t="s">
         <v>489</v>
       </c>
-      <c r="I56" t="s">
+      <c r="L55" s="22" t="s">
         <v>490</v>
       </c>
-      <c r="J56" t="s">
-        <v>491</v>
-      </c>
-      <c r="L56" s="22" t="s">
-        <v>492</v>
-      </c>
-      <c r="M56" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="N56" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="O56" s="11" t="s">
-        <v>429</v>
-      </c>
-      <c r="P56" s="17" t="str">
-        <f t="shared" ref="P56" si="13">IF(O56&lt;&gt;"Yes","","New funding opportunity added: "&amp;D56)</f>
+      <c r="M55" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="N55" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="O55" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="P55" s="17" t="str">
+        <f t="shared" ref="P55" si="13">IF(O55&lt;&gt;"Yes","","New funding opportunity added: "&amp;D55)</f>
         <v>New funding opportunity added: LMS Inclusion and Diversity Fund</v>
       </c>
-      <c r="Q56" s="20" t="str">
-        <f t="shared" ref="Q56" si="14">IF(O56&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D56&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C56&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B56),TEXT(B56,"d mmmm yyyy"),B56)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F56&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G56&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H56&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I56&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K56&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q55" s="20" t="str">
+        <f t="shared" ref="Q55" si="14">IF(O55&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D55&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C55&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B55),TEXT(B55,"d mmmm yyyy"),B55)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F55&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G55&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H55&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I55&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K55&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **LMS Inclusion and Diversity Fund**
@@ -5922,61 +5971,61 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R56" s="13"/>
-    </row>
-    <row r="57" spans="1:18" ht="60">
-      <c r="A57" s="23" t="str">
-        <f t="shared" ref="A57:A60" ca="1" si="15">IF(AND(ISNUMBER(B57),B57&lt;TODAY()),"DEADLINE PASSED",N57)</f>
-        <v>OPEN</v>
-      </c>
-      <c r="B57" s="24">
+      <c r="R55" s="13"/>
+    </row>
+    <row r="56" spans="1:18" ht="64">
+      <c r="A56" s="23" t="str">
+        <f t="shared" ref="A56:A64" ca="1" si="15">IF(AND(ISNUMBER(B56),B56&lt;TODAY()),"DEADLINE PASSED",N56)</f>
+        <v>DEADLINE PASSED</v>
+      </c>
+      <c r="B56" s="24">
         <v>46310</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C56" t="s">
+        <v>491</v>
+      </c>
+      <c r="D56" t="s">
+        <v>492</v>
+      </c>
+      <c r="E56" t="s">
+        <v>493</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="K56" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="D57" t="s">
-        <v>500</v>
-      </c>
-      <c r="E57" t="s">
-        <v>501</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="I57" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="L57" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="M57" s="25" t="s">
-        <v>543</v>
-      </c>
-      <c r="N57" s="25" t="s">
-        <v>361</v>
-      </c>
-      <c r="O57" s="25" t="s">
-        <v>429</v>
-      </c>
-      <c r="P57" s="26" t="str">
-        <f>IF(O57&lt;&gt;"Yes","","New funding opportunity added: "&amp;D57)</f>
+      <c r="L56" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="M56" s="25" t="s">
+        <v>535</v>
+      </c>
+      <c r="N56" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="O56" s="25" t="s">
+        <v>427</v>
+      </c>
+      <c r="P56" s="26" t="str">
+        <f t="shared" ref="P56:P66" si="16">IF(O56&lt;&gt;"Yes","","New funding opportunity added: "&amp;D56)</f>
         <v>New funding opportunity added: Learning &amp; Research Support Fund</v>
       </c>
-      <c r="Q57" s="26" t="str">
-        <f>IF(O57&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D57&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C57&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B57),TEXT(B57,"d mmmm yyyy"),B57)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F57&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G57&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H57&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I57&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K57&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q56" s="26" t="str">
+        <f t="shared" ref="Q56:Q64" si="17">IF(O56&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D56&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C56&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B56),TEXT(B56,"d mmmm yyyy"),B56)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F56&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G56&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H56&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I56&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K56&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **Learning &amp; Research Support Fund**
@@ -5993,236 +6042,240 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R57" s="27">
+      <c r="R56" s="27">
         <v>46301</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="60">
-      <c r="A58" s="28" t="str">
+    <row r="57" spans="1:18" ht="64">
+      <c r="A57" s="28" t="str">
         <f t="shared" ca="1" si="15"/>
         <v>CLOSED – monitor recurrence</v>
       </c>
-      <c r="B58" s="29" t="s">
+      <c r="B57" s="29" t="s">
+        <v>500</v>
+      </c>
+      <c r="C57" s="30" t="s">
+        <v>305</v>
+      </c>
+      <c r="D57" s="30" t="s">
+        <v>501</v>
+      </c>
+      <c r="E57" s="30" t="s">
+        <v>502</v>
+      </c>
+      <c r="F57" s="31" t="s">
+        <v>503</v>
+      </c>
+      <c r="G57" s="31" t="s">
+        <v>504</v>
+      </c>
+      <c r="H57" s="31" t="s">
+        <v>505</v>
+      </c>
+      <c r="I57" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="J57" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="K57" s="31" t="s">
         <v>508</v>
       </c>
-      <c r="C58" s="30" t="s">
-        <v>307</v>
-      </c>
-      <c r="D58" s="30" t="s">
+      <c r="L57" s="30" t="s">
         <v>509</v>
       </c>
-      <c r="E58" s="30" t="s">
+      <c r="M57" s="25" t="s">
+        <v>373</v>
+      </c>
+      <c r="N57" s="25" t="s">
+        <v>361</v>
+      </c>
+      <c r="O57" s="25" t="s">
+        <v>374</v>
+      </c>
+      <c r="P57" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="Q57" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="R57" s="34" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="80">
+      <c r="A58" s="23" t="str">
+        <f t="shared" ca="1" si="15"/>
+        <v>DEADLINE PASSED</v>
+      </c>
+      <c r="B58" s="24">
+        <v>46273</v>
+      </c>
+      <c r="C58" t="s">
+        <v>305</v>
+      </c>
+      <c r="D58" t="s">
         <v>510</v>
       </c>
-      <c r="F58" s="31" t="s">
+      <c r="E58" t="s">
         <v>511</v>
       </c>
-      <c r="G58" s="31" t="s">
+      <c r="F58" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="H58" s="31" t="s">
+      <c r="G58" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="I58" s="31" t="s">
+      <c r="H58" s="2" t="s">
         <v>514</v>
       </c>
-      <c r="J58" s="31" t="s">
+      <c r="I58" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="K58" s="31" t="s">
+      <c r="J58" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="L58" s="30" t="s">
+      <c r="K58" s="2" t="s">
         <v>517</v>
       </c>
+      <c r="L58" t="s">
+        <v>518</v>
+      </c>
       <c r="M58" s="25" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="N58" s="25" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="O58" s="25" t="s">
-        <v>376</v>
-      </c>
-      <c r="P58" s="34" t="str">
-        <f>IF(O58&lt;&gt;"Yes","","New funding opportunity added: "&amp;D58)</f>
-        <v/>
-      </c>
-      <c r="Q58" s="34" t="str">
-        <f>IF(O58&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D58&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C58&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B58),TEXT(B58,"d mmmm yyyy"),B58)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F58&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G58&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H58&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I58&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K58&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
-        <v/>
-      </c>
-      <c r="R58" s="35" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="59" spans="1:18" ht="60">
+        <v>374</v>
+      </c>
+      <c r="P58" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="Q58" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="R58" s="34" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="80">
       <c r="A59" s="23" t="str">
         <f t="shared" ca="1" si="15"/>
         <v>DEADLINE PASSED</v>
       </c>
-      <c r="B59" s="24">
-        <v>46273</v>
-      </c>
-      <c r="C59" t="s">
-        <v>307</v>
-      </c>
-      <c r="D59" t="s">
-        <v>518</v>
-      </c>
-      <c r="E59" t="s">
+      <c r="B59" s="29">
+        <v>46086</v>
+      </c>
+      <c r="C59" s="30" t="s">
         <v>519</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="D59" s="30" t="s">
         <v>520</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="E59" s="30" t="s">
         <v>521</v>
       </c>
-      <c r="H59" s="2" t="s">
+      <c r="F59" s="31" t="s">
         <v>522</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="G59" s="31" t="s">
         <v>523</v>
       </c>
-      <c r="J59" s="2" t="s">
+      <c r="H59" s="31" t="s">
         <v>524</v>
       </c>
-      <c r="K59" s="2" t="s">
+      <c r="I59" s="31" t="s">
         <v>525</v>
       </c>
-      <c r="L59" t="s">
+      <c r="J59" s="31" t="s">
         <v>526</v>
       </c>
+      <c r="K59" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="L59" s="30" t="s">
+        <v>528</v>
+      </c>
       <c r="M59" s="25" t="s">
-        <v>375</v>
+        <v>535</v>
       </c>
       <c r="N59" s="25" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="O59" s="25" t="s">
-        <v>376</v>
-      </c>
-      <c r="P59" s="34" t="str">
-        <f>IF(O59&lt;&gt;"Yes","","New funding opportunity added: "&amp;D59)</f>
-        <v/>
-      </c>
-      <c r="Q59" s="34" t="str">
-        <f>IF(O59&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D59&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C59&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B59),TEXT(B59,"d mmmm yyyy"),B59)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F59&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G59&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H59&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I59&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K59&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
-        <v/>
-      </c>
-      <c r="R59" s="35" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="60" spans="1:18" ht="75">
+        <v>374</v>
+      </c>
+      <c r="P59" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="Q59" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="R59" s="34" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="16">
       <c r="A60" s="23" t="str">
         <f t="shared" ca="1" si="15"/>
-        <v>DEADLINE PASSED</v>
-      </c>
-      <c r="B60" s="29">
-        <v>46086</v>
-      </c>
-      <c r="C60" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="D60" s="30" t="s">
-        <v>528</v>
-      </c>
-      <c r="E60" s="30" t="s">
+        <v>OPEN</v>
+      </c>
+      <c r="B60" t="s">
         <v>529</v>
       </c>
-      <c r="F60" s="31" t="s">
+      <c r="C60" t="s">
+        <v>134</v>
+      </c>
+      <c r="D60" t="s">
+        <v>135</v>
+      </c>
+      <c r="E60" t="s">
+        <v>85</v>
+      </c>
+      <c r="F60" t="s">
         <v>530</v>
       </c>
-      <c r="G60" s="31" t="s">
+      <c r="G60" t="s">
         <v>531</v>
       </c>
-      <c r="H60" s="31" t="s">
+      <c r="H60" t="s">
         <v>532</v>
       </c>
-      <c r="I60" s="31" t="s">
+      <c r="I60" t="s">
         <v>533</v>
       </c>
-      <c r="J60" s="31" t="s">
+      <c r="J60" t="s">
         <v>534</v>
       </c>
-      <c r="K60" s="31" t="s">
-        <v>535</v>
-      </c>
-      <c r="L60" s="30" t="s">
-        <v>536</v>
+      <c r="K60" t="s">
+        <v>141</v>
+      </c>
+      <c r="L60" s="32" t="s">
+        <v>134</v>
       </c>
       <c r="M60" s="25" t="s">
-        <v>543</v>
+        <v>358</v>
       </c>
       <c r="N60" s="25" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="O60" s="25" t="s">
-        <v>376</v>
-      </c>
-      <c r="P60" s="34" t="str">
-        <f>IF(O60&lt;&gt;"Yes","","New funding opportunity added: "&amp;D60)</f>
-        <v/>
-      </c>
-      <c r="Q60" s="34" t="str">
-        <f>IF(O60&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D60&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C60&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B60),TEXT(B60,"d mmmm yyyy"),B60)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F60&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G60&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H60&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I60&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K60&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
-        <v/>
-      </c>
-      <c r="R60" s="35" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="61" spans="1:18" ht="16">
-      <c r="B61" t="s">
-        <v>537</v>
-      </c>
-      <c r="C61" t="s">
-        <v>134</v>
-      </c>
-      <c r="D61" t="s">
-        <v>135</v>
-      </c>
-      <c r="E61" t="s">
-        <v>85</v>
-      </c>
-      <c r="F61" t="s">
-        <v>538</v>
-      </c>
-      <c r="G61" t="s">
-        <v>539</v>
-      </c>
-      <c r="H61" t="s">
-        <v>540</v>
-      </c>
-      <c r="I61" t="s">
-        <v>541</v>
-      </c>
-      <c r="J61" t="s">
-        <v>542</v>
-      </c>
-      <c r="K61" t="s">
-        <v>141</v>
-      </c>
-      <c r="L61" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="M61" s="25" t="s">
-        <v>360</v>
-      </c>
-      <c r="N61" s="25" t="s">
-        <v>361</v>
-      </c>
-      <c r="O61" s="25" t="s">
-        <v>429</v>
-      </c>
-      <c r="P61" s="26" t="str">
-        <f>IF(O61&lt;&gt;"Yes","","New funding opportunity added: "&amp;D61)</f>
+        <v>427</v>
+      </c>
+      <c r="P60" s="26" t="str">
+        <f t="shared" si="16"/>
         <v>New funding opportunity added: Transformative sustainable AI technologies</v>
       </c>
-      <c r="Q61" s="26" t="str">
-        <f>IF(O61&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D61&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C61&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B61),TEXT(B61,"d mmmm yyyy"),B61)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F61&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G61&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H61&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I61&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K61&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+      <c r="Q60" s="26" t="str">
+        <f t="shared" si="17"/>
         <v>Hello,
 A new funding opportunity has been added to the Funding Finder for Statistics.
 **Transformative sustainable AI technologies**
@@ -6239,103 +6292,508 @@
 Daniela &amp; Vinny
 Research Lead for Statistics</v>
       </c>
-      <c r="R61" s="35" t="s">
-        <v>430</v>
+      <c r="R60" s="27">
+        <v>46301</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18">
+      <c r="A61" s="23" t="str">
+        <f t="shared" ca="1" si="15"/>
+        <v>OPEN</v>
+      </c>
+      <c r="B61" s="37" t="s">
+        <v>538</v>
+      </c>
+      <c r="C61" s="30" t="s">
+        <v>536</v>
+      </c>
+      <c r="D61" s="30" t="s">
+        <v>539</v>
+      </c>
+      <c r="E61" s="30" t="s">
+        <v>540</v>
+      </c>
+      <c r="F61" s="30" t="s">
+        <v>541</v>
+      </c>
+      <c r="G61" s="30" t="s">
+        <v>542</v>
+      </c>
+      <c r="H61" s="30" t="s">
+        <v>543</v>
+      </c>
+      <c r="I61" t="s">
+        <v>544</v>
+      </c>
+      <c r="J61" s="30" t="s">
+        <v>545</v>
+      </c>
+      <c r="K61" s="35" t="s">
+        <v>546</v>
+      </c>
+      <c r="L61" s="30" t="s">
+        <v>537</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N61" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O61" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="P61" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v>New funding opportunity added: Heilbronn Research Fellowships 2027</v>
+      </c>
+      <c r="Q61" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**Heilbronn Research Fellowships 2027**
+Funder: Heilbronn Institute for Mathematical Research (HIMR)
+Deadline: 08/11/2026 23:59 GMT
+Funding and duration: 3 years; salary approximately £46,874–£52,517 per year (London weighting where applicable)
+Who can apply: Researchers in relevant mathematical sciences, including Statistics, probability and data science. Restricted to UK residents who are UK or dual UK nationals and eligible for national security clearance. Appointments at Bristol, Imperial, King's College London, UCL or Manchester.
+Why it may be relevant to Statistics: Excellent postdoctoral career opportunity for eligible Statistics PhD graduates and ECRs, particularly those working in probability, statistical methodology, data science and mathematical research.
+Themes: Statistics; Probability; Data science; ECR; Postdoctoral fellowship; Mathematical sciences
+Official opportunity: https://heilbronn.ac.uk/fellowships/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R61" s="27">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18">
+      <c r="A62" s="23" t="str">
+        <f t="shared" ca="1" si="15"/>
+        <v>OPEN</v>
+      </c>
+      <c r="B62" t="s">
+        <v>547</v>
+      </c>
+      <c r="C62" t="s">
+        <v>536</v>
+      </c>
+      <c r="D62" t="s">
+        <v>548</v>
+      </c>
+      <c r="E62" t="s">
+        <v>549</v>
+      </c>
+      <c r="F62" t="s">
+        <v>550</v>
+      </c>
+      <c r="G62" t="s">
+        <v>551</v>
+      </c>
+      <c r="H62" t="s">
+        <v>552</v>
+      </c>
+      <c r="I62" t="s">
+        <v>553</v>
+      </c>
+      <c r="J62" t="s">
+        <v>554</v>
+      </c>
+      <c r="K62" s="22" t="s">
+        <v>555</v>
+      </c>
+      <c r="L62" t="s">
+        <v>537</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N62" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O62" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="P62" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v>New funding opportunity added: HIMR Small Grant Call</v>
+      </c>
+      <c r="Q62" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**HIMR Small Grant Call**
+Funder: Heilbronn Institute for Mathematical Research (HIMR)
+Deadline: Rolling – verify
+Funding and duration: Typically up to £5,000; applications up to £10,000 or exceptionally more considered
+Who can apply: Researchers proposing activities supporting UK mathematical research and the mathematical sciences community; confirm current applicant eligibility
+Why it may be relevant to Statistics: Supports Statistics workshops, conferences, research networks, collaborative activities, visiting researchers and PhD student development
+Themes: Statistics; Mathematical sciences; Workshops; Research collaboration; ECR; Training
+Official opportunity: https://heilbronn.ac.uk/small-grants-call/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R62" s="27">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18">
+      <c r="A63" s="23" t="str">
+        <f t="shared" ca="1" si="15"/>
+        <v>FORTHCOMING</v>
+      </c>
+      <c r="B63" s="37" t="s">
+        <v>500</v>
+      </c>
+      <c r="C63" s="30" t="s">
+        <v>536</v>
+      </c>
+      <c r="D63" s="30" t="s">
+        <v>556</v>
+      </c>
+      <c r="E63" s="30" t="s">
+        <v>557</v>
+      </c>
+      <c r="F63" s="30" t="s">
+        <v>558</v>
+      </c>
+      <c r="G63" s="30" t="s">
+        <v>559</v>
+      </c>
+      <c r="H63" s="30" t="s">
+        <v>560</v>
+      </c>
+      <c r="I63" s="30" t="s">
+        <v>561</v>
+      </c>
+      <c r="J63" s="30" t="s">
+        <v>562</v>
+      </c>
+      <c r="K63" s="36" t="s">
+        <v>563</v>
+      </c>
+      <c r="L63" s="30" t="s">
+        <v>537</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N63" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="O63" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="P63" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v>New funding opportunity added: HIMR Focused Research Grants</v>
+      </c>
+      <c r="Q63" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**HIMR Focused Research Grants**
+Funder: Heilbronn Institute for Mathematical Research (HIMR)
+Deadline: Next round TBC
+Funding and duration: Project-dependent; current award limit not verified
+Who can apply: Groups of researchers proposing focused mathematical research activities; confirm current eligibility
+Why it may be relevant to Statistics: Could fund focused research meetings addressing open problems in statistical methodology, probability, extremes, spatial statistics or computational statistics
+Themes: Statistics; Mathematical sciences; Focused research; Workshops; Collaboration
+Official opportunity: https://heilbronn.ac.uk/frg/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R63" s="27">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" ht="30">
+      <c r="A64" s="38" t="str">
+        <f t="shared" ca="1" si="15"/>
+        <v>ELIGIBILITY TO VERIFY</v>
+      </c>
+      <c r="B64" t="s">
+        <v>564</v>
+      </c>
+      <c r="C64" t="s">
+        <v>536</v>
+      </c>
+      <c r="D64" t="s">
+        <v>565</v>
+      </c>
+      <c r="E64" t="s">
+        <v>566</v>
+      </c>
+      <c r="F64" t="s">
+        <v>567</v>
+      </c>
+      <c r="G64" t="s">
+        <v>568</v>
+      </c>
+      <c r="H64" t="s">
+        <v>569</v>
+      </c>
+      <c r="I64" t="s">
+        <v>570</v>
+      </c>
+      <c r="J64" t="s">
+        <v>571</v>
+      </c>
+      <c r="K64" s="22" t="s">
+        <v>563</v>
+      </c>
+      <c r="L64" t="s">
+        <v>537</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N64" s="16" t="s">
+        <v>572</v>
+      </c>
+      <c r="O64" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="P64" s="33" t="str">
+        <f t="shared" si="16"/>
+        <v>New funding opportunity added: HIMR International Visitors Scheme</v>
+      </c>
+      <c r="Q64" s="33" t="str">
+        <f t="shared" si="17"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**HIMR International Visitors Scheme**
+Funder: Heilbronn Institute for Mathematical Research (HIMR)
+Deadline: Not confirmed
+Funding and duration: Financial support for eligible international research visits; amount and duration not verified
+Who can apply: Scheme centred on leading international mathematicians with research interests shared by Heilbronn Fellows; confirm whether applications must be initiated by a Fellow
+Why it may be relevant to Statistics: Potentially supports international collaboration in Statistics, probability and related mathematical sciences, particularly through partnerships with Heilbronn Fellows
+Themes: Statistics; Mathematical sciences; International collaboration; Research visits; Networking
+Official opportunity: https://heilbronn.ac.uk/frg/
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
+      </c>
+      <c r="R64" s="27">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="65" spans="2:18">
+      <c r="B65" s="29">
+        <v>46188</v>
+      </c>
+      <c r="C65" s="30" t="s">
+        <v>573</v>
+      </c>
+      <c r="D65" s="30" t="s">
+        <v>574</v>
+      </c>
+      <c r="E65" s="30" t="s">
+        <v>575</v>
+      </c>
+      <c r="F65" s="30" t="s">
+        <v>576</v>
+      </c>
+      <c r="G65" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="H65" s="30" t="s">
+        <v>582</v>
+      </c>
+      <c r="I65" s="30" t="s">
+        <v>584</v>
+      </c>
+      <c r="J65" s="30" t="s">
+        <v>585</v>
+      </c>
+      <c r="K65" s="35" t="s">
+        <v>586</v>
+      </c>
+      <c r="L65" s="30" t="s">
+        <v>587</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N65" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="O65" s="16" t="s">
+        <v>588</v>
+      </c>
+      <c r="P65" s="33" t="str">
+        <f t="shared" ref="P65:P66" si="18">IF(O65&lt;&gt;"Yes","","New funding opportunity added: "&amp;D65)</f>
+        <v/>
+      </c>
+      <c r="Q65" s="33" t="str">
+        <f t="shared" ref="Q65:Q66" si="19">IF(O65&lt;&gt;"Yes","","Hello,"&amp;CHAR(10)&amp;CHAR(10)&amp;"A new funding opportunity has been added to the Funding Finder for Statistics."&amp;CHAR(10)&amp;CHAR(10)&amp;"**"&amp;D65&amp;"**"&amp;CHAR(10)&amp;CHAR(10)&amp;"Funder: "&amp;C65&amp;CHAR(10)&amp;"Deadline: "&amp;IF(ISNUMBER(B65),TEXT(B65,"d mmmm yyyy"),B65)&amp;CHAR(10)&amp;"Funding and duration: "&amp;F65&amp;CHAR(10)&amp;CHAR(10)&amp;"Who can apply: "&amp;G65&amp;CHAR(10)&amp;CHAR(10)&amp;"Why it may be relevant to Statistics: "&amp;H65&amp;CHAR(10)&amp;CHAR(10)&amp;"Themes: "&amp;I65&amp;CHAR(10)&amp;CHAR(10)&amp;"Official opportunity: "&amp;K65&amp;CHAR(10)&amp;CHAR(10)&amp;"Funding Finder: "&amp;"https://uofgstats.github.io/research-and-scholarship/"&amp;CHAR(10)&amp;CHAR(10)&amp;"Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change."&amp;CHAR(10)&amp;CHAR(10)&amp;"Best wishes,"&amp;CHAR(10)&amp;"Daniela &amp; Vinny"&amp;CHAR(10)&amp;"Research Lead for Statistics")</f>
+        <v/>
+      </c>
+      <c r="R65" s="27">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="66" spans="2:18">
+      <c r="B66" s="24" t="s">
+        <v>547</v>
+      </c>
+      <c r="C66" t="s">
+        <v>573</v>
+      </c>
+      <c r="D66" t="s">
+        <v>578</v>
+      </c>
+      <c r="E66" t="s">
+        <v>579</v>
+      </c>
+      <c r="F66" t="s">
+        <v>580</v>
+      </c>
+      <c r="G66" t="s">
+        <v>581</v>
+      </c>
+      <c r="H66" t="s">
+        <v>583</v>
+      </c>
+      <c r="I66" t="s">
+        <v>589</v>
+      </c>
+      <c r="J66" t="s">
+        <v>590</v>
+      </c>
+      <c r="K66" s="22" t="s">
+        <v>591</v>
+      </c>
+      <c r="L66" t="s">
+        <v>587</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="N66" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="O66" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="P66" s="33" t="str">
+        <f t="shared" si="18"/>
+        <v>New funding opportunity added: SUM4Products Mini-grants</v>
+      </c>
+      <c r="Q66" s="33" t="str">
+        <f t="shared" si="19"/>
+        <v>Hello,
+A new funding opportunity has been added to the Funding Finder for Statistics.
+**SUM4Products Mini-grants**
+Funder: EPSRC SUM4Products Network+
+Deadline: Rolling – verify
+Funding and duration: Normally up to £500; larger requests may be discussed
+Who can apply: UK-based SUM4Products network members, generally with previous participation. PhD students eligible with supervisor support. UK travel only
+Why it may be relevant to Statistics: Supports Statistics researchers and PhD students engaging with industry through workshops, conferences, site visits and collaborative activities
+Themes: Industrial collaboration; Networking; Travel; Workshops; PhD; Knowledge exchange
+Official opportunity: https://www.sum4products.co.uk/flexible-funding
+Funding Finder: https://uofgstats.github.io/research-and-scholarship/
+Please check the official funder page before preparing an application, as deadlines and eligibility requirements can change.
+Best wishes,
+Daniela &amp; Vinny
+Research Lead for Statistics</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A42 A50:A51">
-    <cfRule type="expression" dxfId="19" priority="13">
+  <conditionalFormatting sqref="A2:A55">
+    <cfRule type="expression" dxfId="15" priority="13">
       <formula>$A2="OPEN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="14">
+    <cfRule type="expression" dxfId="14" priority="14">
       <formula>$A2="FORTHCOMING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="15">
+    <cfRule type="expression" dxfId="13" priority="15">
       <formula>LEFT($A2,6)="CLOSED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="16">
+    <cfRule type="expression" dxfId="12" priority="16">
       <formula>$A2="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A56">
-    <cfRule type="expression" dxfId="15" priority="17">
-      <formula>$A2="OPEN"</formula>
+  <conditionalFormatting sqref="A56">
+    <cfRule type="expression" dxfId="11" priority="5">
+      <formula>$A56="OPEN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="18">
-      <formula>$A2="FORTHCOMING"</formula>
+    <cfRule type="expression" dxfId="10" priority="6">
+      <formula>$A56="FORTHCOMING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="19">
-      <formula>LEFT($A2,6)="CLOSED"</formula>
+    <cfRule type="expression" dxfId="9" priority="7">
+      <formula>LEFT($A56,6)="CLOSED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="20">
-      <formula>$A2="DEADLINE PASSED"</formula>
+    <cfRule type="expression" dxfId="8" priority="8">
+      <formula>$A56="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A57">
-    <cfRule type="expression" dxfId="11" priority="5">
-      <formula>$A57="OPEN"</formula>
+  <conditionalFormatting sqref="A56:A64">
+    <cfRule type="expression" dxfId="7" priority="9">
+      <formula>$A56="OPEN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="6">
-      <formula>$A57="FORTHCOMING"</formula>
+    <cfRule type="expression" dxfId="6" priority="10">
+      <formula>$A56="FORTHCOMING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="7">
-      <formula>LEFT($A57,6)="CLOSED"</formula>
+    <cfRule type="expression" dxfId="5" priority="11">
+      <formula>LEFT($A56,6)="CLOSED"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="8">
-      <formula>$A57="DEADLINE PASSED"</formula>
+    <cfRule type="expression" dxfId="4" priority="12">
+      <formula>$A56="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A57:A60">
-    <cfRule type="expression" dxfId="7" priority="9">
-      <formula>$A57="OPEN"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="10">
-      <formula>$A57="FORTHCOMING"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="11">
-      <formula>LEFT($A57,6)="CLOSED"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="12">
-      <formula>$A57="DEADLINE PASSED"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A59:A60">
+  <conditionalFormatting sqref="A58:A64">
     <cfRule type="expression" dxfId="3" priority="1">
-      <formula>$A59="OPEN"</formula>
+      <formula>$A58="OPEN"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="2">
-      <formula>$A59="FORTHCOMING"</formula>
+      <formula>$A58="FORTHCOMING"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="3">
-      <formula>LEFT($A59,6)="CLOSED"</formula>
+      <formula>LEFT($A58,6)="CLOSED"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="4">
-      <formula>$A59="DEADLINE PASSED"</formula>
+      <formula>$A58="DEADLINE PASSED"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" sqref="M2:M500" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M499" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Research,Scholarship,Research and Scholarship"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="N2:N500" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="N2:N499" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"OPEN,FORTHCOMING,CLOSED – monitor recurrence,CLOSED – invited stage continues"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="O2:O500" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" sqref="O2:O499" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Yes,No,Added at launch – no notification"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="K50" r:id="rId1" xr:uid="{983CD2BB-548A-CA46-B886-1D5A7F03FD6A}"/>
-    <hyperlink ref="K52" r:id="rId2" xr:uid="{CEDBB7D3-D861-6348-9912-50FD352C627E}"/>
-    <hyperlink ref="K53" r:id="rId3" xr:uid="{5E871FF8-6856-3F46-A97A-BF5C75823330}"/>
-    <hyperlink ref="K54" r:id="rId4" xr:uid="{03C79587-5FB8-6E4D-800F-90A27A753D0A}"/>
-    <hyperlink ref="K55" r:id="rId5" xr:uid="{51B5FE9E-0AEA-6A40-8FC5-EEEC2082F053}"/>
-    <hyperlink ref="L56" r:id="rId6" xr:uid="{716C5825-E552-FD4C-B304-7A428DE7BA28}"/>
+    <hyperlink ref="K49" r:id="rId1" xr:uid="{983CD2BB-548A-CA46-B886-1D5A7F03FD6A}"/>
+    <hyperlink ref="K51" r:id="rId2" xr:uid="{CEDBB7D3-D861-6348-9912-50FD352C627E}"/>
+    <hyperlink ref="K52" r:id="rId3" xr:uid="{5E871FF8-6856-3F46-A97A-BF5C75823330}"/>
+    <hyperlink ref="K53" r:id="rId4" xr:uid="{03C79587-5FB8-6E4D-800F-90A27A753D0A}"/>
+    <hyperlink ref="K54" r:id="rId5" xr:uid="{51B5FE9E-0AEA-6A40-8FC5-EEEC2082F053}"/>
+    <hyperlink ref="L55" r:id="rId6" xr:uid="{716C5825-E552-FD4C-B304-7A428DE7BA28}"/>
+    <hyperlink ref="K61" r:id="rId7" xr:uid="{652B89D9-F013-3647-A57E-C9181DE98F89}"/>
+    <hyperlink ref="K62" r:id="rId8" xr:uid="{828E7974-7FE4-B743-921D-CEA7059FBF02}"/>
+    <hyperlink ref="K63" r:id="rId9" xr:uid="{64FA85FA-F436-B948-84F7-5A169FE28AB7}"/>
+    <hyperlink ref="K64" r:id="rId10" xr:uid="{F3897D68-577A-E445-A0CE-FD72FB6CD5B0}"/>
+    <hyperlink ref="K65" r:id="rId11" xr:uid="{BD58BDFB-0A94-2C43-BEA0-EC774FDC507F}"/>
+    <hyperlink ref="K66" r:id="rId12" xr:uid="{7F0AF101-1D7E-8F4A-8989-A7B5F9F1B410}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6343,85 +6801,85 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="88" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="39" t="s">
+        <v>323</v>
+      </c>
+      <c r="B1" s="39"/>
+    </row>
+    <row r="2" spans="1:2" ht="32">
+      <c r="A2" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>325</v>
-      </c>
-      <c r="B1" s="32"/>
-    </row>
-    <row r="2" spans="1:2" ht="30">
-      <c r="A2" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16">
       <c r="A3" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="48">
+      <c r="A4" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45">
-      <c r="A4" s="4" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="48">
+      <c r="A5" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>330</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="45">
-      <c r="A5" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32">
       <c r="A6" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="32">
+      <c r="A7" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>334</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30">
-      <c r="A7" s="4" t="s">
-        <v>335</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16">
       <c r="A8" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16">
       <c r="A9" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>337</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16">
       <c r="A10" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>214</v>
@@ -6429,31 +6887,31 @@
     </row>
     <row r="11" spans="1:2" ht="16">
       <c r="A11" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="16">
       <c r="A12" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16">
       <c r="A13" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="16">
       <c r="A14" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>135</v>
@@ -6461,23 +6919,23 @@
     </row>
     <row r="15" spans="1:2" ht="16">
       <c r="A15" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16">
       <c r="A16" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16">
       <c r="A17" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>116</v>
@@ -6485,66 +6943,66 @@
     </row>
     <row r="18" spans="1:2" ht="16">
       <c r="A18" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="45">
+    <row r="19" spans="1:2" ht="48">
       <c r="A19" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="45">
       <c r="A20" s="15" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="57" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30">
       <c r="A22" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15">
-      <c r="A23" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30">
       <c r="A24" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B25" s="5" t="s">
         <v>352</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15">
-      <c r="A25" s="7" t="s">
-        <v>353</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>